<commit_message>
2025. 7. 1. (화요일), Weekly Plan 7월 1주차 작성 완료
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\2.project\hkmc_ptc_heater\Doc\1. 일정\1. Weekly Plan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\1. doc\HKMC_AIR_PTC\일정\PTC_HEATER_DOC (250626 Repo 변경, 해당 Repo 사용)\ptc_heater_doc\1. 일정\1. Weekly Plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="17685" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="17685" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="대일정" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="232">
   <si>
     <t>■</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1344,6 +1344,22 @@
     <t>7월</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>[조현진 전임, 임제훈 사원]
+- SWE.1 SRS 작성 완료 : ~ 6/30
+   : 3.1 Hardware - Software Interface
+   : 3.2 CAN Communication - Software Interface
+   : 4.1 Software State Transition Requirements
+   : 4.2.1.1 LV Sensor Fault / LV Over Voltage_Under Voltage Fault
+   : 4.2.1.2 HV Sensor Fault / HV Over Voltage_Under Voltage Fault
+- SWE.2 SADS 작성 계획
+   : Component 다이어그램 작성
+   : LV Sensor Fault / LV Over Voltage_Under Voltage Fault 정적, 동적 작성
+   : HV Sensor Fault / HV Over Voltage_Under Voltage Fault 정적, 동적 작성
+- SWE.3 SDDS 작성 계획
+   : LV Sensor Fault 작성</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -1352,7 +1368,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="mm&quot;월&quot;\ dd&quot;일&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2497,7 +2513,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2914,6 +2930,12 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="57" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3504,7 +3526,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BL24"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.375" customWidth="1"/>
     <col min="2" max="2" width="18.875" customWidth="1"/>
@@ -3515,7 +3537,7 @@
     <col min="36" max="64" width="8.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:64" s="20" customFormat="1" ht="32.25" thickBot="1">
+    <row r="1" spans="1:64" s="20" customFormat="1" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
@@ -3525,7 +3547,7 @@
       <c r="C1" s="21"/>
       <c r="D1" s="21"/>
     </row>
-    <row r="2" spans="1:64" ht="31.5" customHeight="1" thickTop="1">
+    <row r="2" spans="1:64" ht="31.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B2" s="124" t="s">
         <v>2</v>
       </c>
@@ -3606,7 +3628,7 @@
       <c r="BK2" s="128"/>
       <c r="BL2" s="129"/>
     </row>
-    <row r="3" spans="1:64" ht="31.5" customHeight="1" thickBot="1">
+    <row r="3" spans="1:64" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="125"/>
       <c r="C3" s="127"/>
       <c r="D3" s="127"/>
@@ -3791,7 +3813,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:64" ht="183" customHeight="1" thickBot="1">
+    <row r="4" spans="1:64" ht="183" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="63" t="s">
         <v>122</v>
       </c>
@@ -3872,7 +3894,7 @@
       <c r="BK4" s="2"/>
       <c r="BL4" s="5"/>
     </row>
-    <row r="5" spans="1:64" ht="81">
+    <row r="5" spans="1:64" ht="81" x14ac:dyDescent="0.3">
       <c r="B5" s="28" t="s">
         <v>123</v>
       </c>
@@ -3951,7 +3973,7 @@
       <c r="BK5" s="31"/>
       <c r="BL5" s="10"/>
     </row>
-    <row r="6" spans="1:64" ht="67.5">
+    <row r="6" spans="1:64" ht="67.5" x14ac:dyDescent="0.3">
       <c r="B6" s="28" t="s">
         <v>124</v>
       </c>
@@ -4034,7 +4056,7 @@
       <c r="BK6" s="31"/>
       <c r="BL6" s="10"/>
     </row>
-    <row r="7" spans="1:64" ht="61.5" customHeight="1">
+    <row r="7" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="28" t="s">
         <v>125</v>
       </c>
@@ -4115,7 +4137,7 @@
       <c r="BK7" s="31"/>
       <c r="BL7" s="10"/>
     </row>
-    <row r="8" spans="1:64" ht="81">
+    <row r="8" spans="1:64" ht="81" x14ac:dyDescent="0.3">
       <c r="B8" s="28" t="s">
         <v>224</v>
       </c>
@@ -4192,7 +4214,7 @@
       <c r="BK8" s="31"/>
       <c r="BL8" s="10"/>
     </row>
-    <row r="9" spans="1:64" ht="61.5" customHeight="1">
+    <row r="9" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="27" t="s">
         <v>3</v>
       </c>
@@ -4265,7 +4287,7 @@
       <c r="BK9" s="31"/>
       <c r="BL9" s="10"/>
     </row>
-    <row r="10" spans="1:64" ht="61.5" customHeight="1">
+    <row r="10" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="27" t="s">
         <v>46</v>
       </c>
@@ -4342,7 +4364,7 @@
       <c r="BK10" s="31"/>
       <c r="BL10" s="10"/>
     </row>
-    <row r="11" spans="1:64" ht="61.5" customHeight="1">
+    <row r="11" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="28" t="s">
         <v>130</v>
       </c>
@@ -4423,7 +4445,7 @@
       <c r="BK11" s="31"/>
       <c r="BL11" s="10"/>
     </row>
-    <row r="12" spans="1:64" ht="61.5" customHeight="1">
+    <row r="12" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="28" t="s">
         <v>131</v>
       </c>
@@ -4502,7 +4524,7 @@
       <c r="BK12" s="31"/>
       <c r="BL12" s="10"/>
     </row>
-    <row r="13" spans="1:64" ht="183.75" customHeight="1">
+    <row r="13" spans="1:64" ht="183.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="28" t="s">
         <v>63</v>
       </c>
@@ -4591,7 +4613,7 @@
       <c r="BK13" s="31"/>
       <c r="BL13" s="10"/>
     </row>
-    <row r="14" spans="1:64" ht="67.5">
+    <row r="14" spans="1:64" ht="67.5" x14ac:dyDescent="0.3">
       <c r="B14" s="27" t="s">
         <v>74</v>
       </c>
@@ -4680,7 +4702,7 @@
       <c r="BK14" s="31"/>
       <c r="BL14" s="10"/>
     </row>
-    <row r="15" spans="1:64" ht="61.5" customHeight="1">
+    <row r="15" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="27" t="s">
         <v>65</v>
       </c>
@@ -4761,7 +4783,7 @@
       <c r="BK15" s="31"/>
       <c r="BL15" s="10"/>
     </row>
-    <row r="16" spans="1:64" ht="61.5" customHeight="1">
+    <row r="16" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="27" t="s">
         <v>66</v>
       </c>
@@ -4850,7 +4872,7 @@
       <c r="BK16" s="31"/>
       <c r="BL16" s="10"/>
     </row>
-    <row r="17" spans="2:64" ht="61.5" customHeight="1">
+    <row r="17" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="57" t="s">
         <v>76</v>
       </c>
@@ -4937,7 +4959,7 @@
       <c r="BK17" s="71"/>
       <c r="BL17" s="48"/>
     </row>
-    <row r="18" spans="2:64" ht="76.5" customHeight="1">
+    <row r="18" spans="2:64" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="27" t="s">
         <v>86</v>
       </c>
@@ -5028,7 +5050,7 @@
       <c r="BK18" s="73"/>
       <c r="BL18" s="70"/>
     </row>
-    <row r="19" spans="2:64" ht="61.5" customHeight="1">
+    <row r="19" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="77" t="s">
         <v>144</v>
       </c>
@@ -5113,7 +5135,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="2:64" ht="61.5" customHeight="1">
+    <row r="20" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="77" t="s">
         <v>109</v>
       </c>
@@ -5182,7 +5204,7 @@
       <c r="BK20" s="73"/>
       <c r="BL20" s="70"/>
     </row>
-    <row r="21" spans="2:64" ht="61.5" customHeight="1">
+    <row r="21" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="57" t="s">
         <v>112</v>
       </c>
@@ -5251,7 +5273,7 @@
       <c r="BK21" s="73"/>
       <c r="BL21" s="70"/>
     </row>
-    <row r="22" spans="2:64" ht="61.5" customHeight="1">
+    <row r="22" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="57" t="s">
         <v>169</v>
       </c>
@@ -5320,7 +5342,7 @@
       <c r="BK22" s="73"/>
       <c r="BL22" s="70"/>
     </row>
-    <row r="23" spans="2:64" ht="61.5" customHeight="1" thickBot="1">
+    <row r="23" spans="2:64" ht="61.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="79" t="s">
         <v>170</v>
       </c>
@@ -5389,7 +5411,7 @@
       <c r="BK23" s="75"/>
       <c r="BL23" s="55"/>
     </row>
-    <row r="24" spans="2:64" ht="17.25" thickTop="1"/>
+    <row r="24" spans="2:64" ht="17.25" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="B2:B3"/>
@@ -5411,7 +5433,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.375" style="83" customWidth="1"/>
     <col min="2" max="2" width="9" style="83"/>
@@ -5423,7 +5445,7 @@
     <col min="15" max="16384" width="9" style="83"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="32.25" thickBot="1">
+    <row r="1" spans="1:14" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="110" t="s">
         <v>151</v>
       </c>
@@ -5434,7 +5456,7 @@
       <c r="D1" s="111"/>
       <c r="E1" s="109"/>
     </row>
-    <row r="2" spans="1:14" ht="30" customHeight="1" thickTop="1">
+    <row r="2" spans="1:14" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B2" s="133" t="s">
         <v>2</v>
       </c>
@@ -5463,7 +5485,7 @@
       <c r="M2" s="131"/>
       <c r="N2" s="132"/>
     </row>
-    <row r="3" spans="1:14" ht="37.5" customHeight="1" thickBot="1">
+    <row r="3" spans="1:14" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="134"/>
       <c r="C3" s="138"/>
       <c r="D3" s="138"/>
@@ -5496,7 +5518,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="108">
+    <row r="4" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B4" s="84" t="s">
         <v>120</v>
       </c>
@@ -5531,7 +5553,7 @@
       <c r="M4" s="107"/>
       <c r="N4" s="94"/>
     </row>
-    <row r="5" spans="1:14" ht="108">
+    <row r="5" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B5" s="85" t="s">
         <v>126</v>
       </c>
@@ -5566,7 +5588,7 @@
       <c r="M5" s="107"/>
       <c r="N5" s="95"/>
     </row>
-    <row r="6" spans="1:14" ht="108">
+    <row r="6" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B6" s="85" t="s">
         <v>127</v>
       </c>
@@ -5601,7 +5623,7 @@
       <c r="M6" s="107"/>
       <c r="N6" s="95"/>
     </row>
-    <row r="7" spans="1:14" ht="108">
+    <row r="7" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B7" s="85" t="s">
         <v>128</v>
       </c>
@@ -5636,7 +5658,7 @@
       <c r="M7" s="107"/>
       <c r="N7" s="95"/>
     </row>
-    <row r="8" spans="1:14" ht="108">
+    <row r="8" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B8" s="86" t="s">
         <v>3</v>
       </c>
@@ -5671,7 +5693,7 @@
       <c r="M8" s="107"/>
       <c r="N8" s="95"/>
     </row>
-    <row r="9" spans="1:14" ht="175.5">
+    <row r="9" spans="1:14" ht="175.5" x14ac:dyDescent="0.3">
       <c r="B9" s="86" t="s">
         <v>46</v>
       </c>
@@ -5706,7 +5728,7 @@
       <c r="M9" s="107"/>
       <c r="N9" s="95"/>
     </row>
-    <row r="10" spans="1:14" ht="121.5">
+    <row r="10" spans="1:14" ht="121.5" x14ac:dyDescent="0.3">
       <c r="B10" s="86" t="s">
         <v>56</v>
       </c>
@@ -5741,7 +5763,7 @@
       <c r="M10" s="107"/>
       <c r="N10" s="95"/>
     </row>
-    <row r="11" spans="1:14" ht="108">
+    <row r="11" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B11" s="85" t="s">
         <v>63</v>
       </c>
@@ -5776,7 +5798,7 @@
       <c r="M11" s="107"/>
       <c r="N11" s="95"/>
     </row>
-    <row r="12" spans="1:14" ht="57" customHeight="1">
+    <row r="12" spans="1:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="86" t="s">
         <v>74</v>
       </c>
@@ -5811,7 +5833,7 @@
       <c r="M12" s="107"/>
       <c r="N12" s="95"/>
     </row>
-    <row r="13" spans="1:14" ht="347.25" customHeight="1">
+    <row r="13" spans="1:14" ht="347.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="86" t="s">
         <v>121</v>
       </c>
@@ -5846,7 +5868,7 @@
       <c r="M13" s="107"/>
       <c r="N13" s="95"/>
     </row>
-    <row r="14" spans="1:14" ht="175.5">
+    <row r="14" spans="1:14" ht="175.5" x14ac:dyDescent="0.3">
       <c r="B14" s="87" t="s">
         <v>184</v>
       </c>
@@ -5875,7 +5897,7 @@
       <c r="M14" s="107"/>
       <c r="N14" s="95"/>
     </row>
-    <row r="15" spans="1:14" ht="57" customHeight="1">
+    <row r="15" spans="1:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="87" t="s">
         <v>76</v>
       </c>
@@ -5908,7 +5930,7 @@
       <c r="M15" s="107"/>
       <c r="N15" s="95"/>
     </row>
-    <row r="16" spans="1:14" ht="121.5">
+    <row r="16" spans="1:14" ht="121.5" x14ac:dyDescent="0.3">
       <c r="B16" s="86" t="s">
         <v>86</v>
       </c>
@@ -5941,7 +5963,7 @@
       <c r="M16" s="107"/>
       <c r="N16" s="95"/>
     </row>
-    <row r="17" spans="2:14" ht="57" customHeight="1">
+    <row r="17" spans="2:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="88" t="s">
         <v>144</v>
       </c>
@@ -5974,7 +5996,7 @@
       <c r="M17" s="91"/>
       <c r="N17" s="95"/>
     </row>
-    <row r="18" spans="2:14" ht="162">
+    <row r="18" spans="2:14" ht="162" x14ac:dyDescent="0.3">
       <c r="B18" s="88" t="s">
         <v>109</v>
       </c>
@@ -6009,7 +6031,7 @@
       <c r="M18" s="107"/>
       <c r="N18" s="95"/>
     </row>
-    <row r="19" spans="2:14" ht="57" customHeight="1">
+    <row r="19" spans="2:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="87" t="s">
         <v>112</v>
       </c>
@@ -6044,7 +6066,7 @@
       <c r="M19" s="107"/>
       <c r="N19" s="95"/>
     </row>
-    <row r="20" spans="2:14" ht="57" customHeight="1">
+    <row r="20" spans="2:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="87" t="s">
         <v>171</v>
       </c>
@@ -6079,7 +6101,7 @@
       <c r="M20" s="107"/>
       <c r="N20" s="114"/>
     </row>
-    <row r="21" spans="2:14" ht="57" customHeight="1" thickBot="1">
+    <row r="21" spans="2:14" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="89" t="s">
         <v>111</v>
       </c>
@@ -6114,7 +6136,7 @@
       <c r="M21" s="122"/>
       <c r="N21" s="97"/>
     </row>
-    <row r="22" spans="2:14" ht="14.25" thickTop="1"/>
+    <row r="22" spans="2:14" ht="14.25" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="K2:N2"/>
@@ -6187,7 +6209,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.375" style="83" customWidth="1"/>
     <col min="2" max="2" width="9" style="83"/>
@@ -6198,7 +6220,7 @@
     <col min="10" max="16384" width="9" style="83"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.25" thickBot="1">
+    <row r="1" spans="1:9" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="110" t="s">
         <v>0</v>
       </c>
@@ -6209,7 +6231,7 @@
       <c r="D1" s="111"/>
       <c r="E1" s="109"/>
     </row>
-    <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1">
+    <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B2" s="133" t="s">
         <v>2</v>
       </c>
@@ -6229,7 +6251,7 @@
       <c r="H2" s="131"/>
       <c r="I2" s="132"/>
     </row>
-    <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1">
+    <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="134"/>
       <c r="C3" s="138"/>
       <c r="D3" s="138"/>
@@ -6247,7 +6269,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="57" customHeight="1">
+    <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="84" t="s">
         <v>120</v>
       </c>
@@ -6265,7 +6287,7 @@
       <c r="H4" s="90"/>
       <c r="I4" s="94"/>
     </row>
-    <row r="5" spans="1:9" ht="57" customHeight="1">
+    <row r="5" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="85" t="s">
         <v>126</v>
       </c>
@@ -6283,7 +6305,7 @@
       <c r="H5" s="91"/>
       <c r="I5" s="95"/>
     </row>
-    <row r="6" spans="1:9" ht="57" customHeight="1">
+    <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="85" t="s">
         <v>127</v>
       </c>
@@ -6301,7 +6323,7 @@
       <c r="H6" s="91"/>
       <c r="I6" s="95"/>
     </row>
-    <row r="7" spans="1:9" ht="57" customHeight="1">
+    <row r="7" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="85" t="s">
         <v>128</v>
       </c>
@@ -6319,7 +6341,7 @@
       <c r="H7" s="91"/>
       <c r="I7" s="95"/>
     </row>
-    <row r="8" spans="1:9" ht="57" customHeight="1">
+    <row r="8" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="86" t="s">
         <v>3</v>
       </c>
@@ -6337,7 +6359,7 @@
       <c r="H8" s="91"/>
       <c r="I8" s="95"/>
     </row>
-    <row r="9" spans="1:9" ht="27">
+    <row r="9" spans="1:9" ht="27" x14ac:dyDescent="0.3">
       <c r="B9" s="86" t="s">
         <v>46</v>
       </c>
@@ -6355,7 +6377,7 @@
       <c r="H9" s="91"/>
       <c r="I9" s="95"/>
     </row>
-    <row r="10" spans="1:9" ht="57" customHeight="1">
+    <row r="10" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="86" t="s">
         <v>56</v>
       </c>
@@ -6373,7 +6395,7 @@
       <c r="H10" s="91"/>
       <c r="I10" s="95"/>
     </row>
-    <row r="11" spans="1:9" ht="40.5">
+    <row r="11" spans="1:9" ht="40.5" x14ac:dyDescent="0.3">
       <c r="B11" s="85" t="s">
         <v>63</v>
       </c>
@@ -6391,7 +6413,7 @@
       <c r="H11" s="91"/>
       <c r="I11" s="95"/>
     </row>
-    <row r="12" spans="1:9" ht="57" customHeight="1">
+    <row r="12" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="86" t="s">
         <v>74</v>
       </c>
@@ -6409,7 +6431,7 @@
       <c r="H12" s="91"/>
       <c r="I12" s="95"/>
     </row>
-    <row r="13" spans="1:9" ht="347.25" customHeight="1">
+    <row r="13" spans="1:9" ht="347.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="86" t="s">
         <v>121</v>
       </c>
@@ -6427,7 +6449,7 @@
       <c r="H13" s="91"/>
       <c r="I13" s="95"/>
     </row>
-    <row r="14" spans="1:9" ht="409.5">
+    <row r="14" spans="1:9" ht="409.5" x14ac:dyDescent="0.3">
       <c r="B14" s="87" t="s">
         <v>184</v>
       </c>
@@ -6441,11 +6463,11 @@
       <c r="F14" s="116"/>
       <c r="G14" s="107"/>
       <c r="H14" s="91"/>
-      <c r="I14" s="107" t="s">
+      <c r="I14" s="139" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="57" customHeight="1">
+    <row r="15" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="87" t="s">
         <v>76</v>
       </c>
@@ -6463,7 +6485,7 @@
       <c r="H15" s="91"/>
       <c r="I15" s="95"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B16" s="86" t="s">
         <v>86</v>
       </c>
@@ -6481,7 +6503,7 @@
       <c r="H16" s="91"/>
       <c r="I16" s="95"/>
     </row>
-    <row r="17" spans="2:9" ht="57" customHeight="1">
+    <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="88" t="s">
         <v>144</v>
       </c>
@@ -6499,7 +6521,7 @@
       <c r="H17" s="91"/>
       <c r="I17" s="95"/>
     </row>
-    <row r="18" spans="2:9" ht="27">
+    <row r="18" spans="2:9" ht="27" x14ac:dyDescent="0.3">
       <c r="B18" s="88" t="s">
         <v>109</v>
       </c>
@@ -6517,7 +6539,7 @@
       <c r="H18" s="91"/>
       <c r="I18" s="95"/>
     </row>
-    <row r="19" spans="2:9" ht="57" customHeight="1">
+    <row r="19" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="87" t="s">
         <v>112</v>
       </c>
@@ -6535,7 +6557,7 @@
       <c r="H19" s="91"/>
       <c r="I19" s="95"/>
     </row>
-    <row r="20" spans="2:9" ht="57" customHeight="1">
+    <row r="20" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="87" t="s">
         <v>170</v>
       </c>
@@ -6553,7 +6575,7 @@
       <c r="H20" s="113"/>
       <c r="I20" s="114"/>
     </row>
-    <row r="21" spans="2:9" ht="57" customHeight="1" thickBot="1">
+    <row r="21" spans="2:9" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="89" t="s">
         <v>111</v>
       </c>
@@ -6571,7 +6593,7 @@
       <c r="H21" s="96"/>
       <c r="I21" s="97"/>
     </row>
-    <row r="22" spans="2:9" ht="14.25" thickTop="1"/>
+    <row r="22" spans="2:9" ht="14.25" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="B2:B3"/>
@@ -6588,7 +6610,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.375" style="83" customWidth="1"/>
     <col min="2" max="2" width="9" style="83"/>
@@ -6599,7 +6621,7 @@
     <col min="10" max="16384" width="9" style="83"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.25" thickBot="1">
+    <row r="1" spans="1:9" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="110" t="s">
         <v>0</v>
       </c>
@@ -6610,7 +6632,7 @@
       <c r="D1" s="111"/>
       <c r="E1" s="109"/>
     </row>
-    <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1">
+    <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B2" s="133" t="s">
         <v>2</v>
       </c>
@@ -6630,7 +6652,7 @@
       <c r="H2" s="131"/>
       <c r="I2" s="132"/>
     </row>
-    <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1">
+    <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="134"/>
       <c r="C3" s="138"/>
       <c r="D3" s="138"/>
@@ -6648,7 +6670,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="57" customHeight="1">
+    <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="84" t="s">
         <v>120</v>
       </c>
@@ -6666,7 +6688,7 @@
       <c r="H4" s="90"/>
       <c r="I4" s="94"/>
     </row>
-    <row r="5" spans="1:9" ht="57" customHeight="1">
+    <row r="5" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="85" t="s">
         <v>126</v>
       </c>
@@ -6684,7 +6706,7 @@
       <c r="H5" s="91"/>
       <c r="I5" s="95"/>
     </row>
-    <row r="6" spans="1:9" ht="57" customHeight="1">
+    <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="85" t="s">
         <v>127</v>
       </c>
@@ -6702,7 +6724,7 @@
       <c r="H6" s="91"/>
       <c r="I6" s="95"/>
     </row>
-    <row r="7" spans="1:9" ht="57" customHeight="1">
+    <row r="7" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="85" t="s">
         <v>128</v>
       </c>
@@ -6720,7 +6742,7 @@
       <c r="H7" s="91"/>
       <c r="I7" s="95"/>
     </row>
-    <row r="8" spans="1:9" ht="57" customHeight="1">
+    <row r="8" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="86" t="s">
         <v>3</v>
       </c>
@@ -6738,7 +6760,7 @@
       <c r="H8" s="91"/>
       <c r="I8" s="95"/>
     </row>
-    <row r="9" spans="1:9" ht="27">
+    <row r="9" spans="1:9" ht="27" x14ac:dyDescent="0.3">
       <c r="B9" s="86" t="s">
         <v>46</v>
       </c>
@@ -6756,7 +6778,7 @@
       <c r="H9" s="91"/>
       <c r="I9" s="95"/>
     </row>
-    <row r="10" spans="1:9" ht="57" customHeight="1">
+    <row r="10" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="86" t="s">
         <v>56</v>
       </c>
@@ -6774,7 +6796,7 @@
       <c r="H10" s="91"/>
       <c r="I10" s="95"/>
     </row>
-    <row r="11" spans="1:9" ht="40.5">
+    <row r="11" spans="1:9" ht="40.5" x14ac:dyDescent="0.3">
       <c r="B11" s="85" t="s">
         <v>63</v>
       </c>
@@ -6792,7 +6814,7 @@
       <c r="H11" s="91"/>
       <c r="I11" s="95"/>
     </row>
-    <row r="12" spans="1:9" ht="57" customHeight="1">
+    <row r="12" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="86" t="s">
         <v>74</v>
       </c>
@@ -6810,7 +6832,7 @@
       <c r="H12" s="91"/>
       <c r="I12" s="95"/>
     </row>
-    <row r="13" spans="1:9" ht="347.25" customHeight="1">
+    <row r="13" spans="1:9" ht="347.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="86" t="s">
         <v>121</v>
       </c>
@@ -6828,7 +6850,7 @@
       <c r="H13" s="91"/>
       <c r="I13" s="95"/>
     </row>
-    <row r="14" spans="1:9" ht="409.5">
+    <row r="14" spans="1:9" ht="229.5" x14ac:dyDescent="0.3">
       <c r="B14" s="87" t="s">
         <v>184</v>
       </c>
@@ -6839,14 +6861,14 @@
         <v>183</v>
       </c>
       <c r="E14" s="102"/>
-      <c r="F14" s="116"/>
+      <c r="F14" s="140" t="s">
+        <v>231</v>
+      </c>
       <c r="G14" s="107"/>
       <c r="H14" s="91"/>
-      <c r="I14" s="107" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="57" customHeight="1">
+      <c r="I14" s="139"/>
+    </row>
+    <row r="15" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="87" t="s">
         <v>76</v>
       </c>
@@ -6864,7 +6886,7 @@
       <c r="H15" s="91"/>
       <c r="I15" s="95"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B16" s="86" t="s">
         <v>86</v>
       </c>
@@ -6882,7 +6904,7 @@
       <c r="H16" s="91"/>
       <c r="I16" s="95"/>
     </row>
-    <row r="17" spans="2:9" ht="57" customHeight="1">
+    <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="88" t="s">
         <v>144</v>
       </c>
@@ -6900,7 +6922,7 @@
       <c r="H17" s="91"/>
       <c r="I17" s="95"/>
     </row>
-    <row r="18" spans="2:9" ht="27">
+    <row r="18" spans="2:9" ht="27" x14ac:dyDescent="0.3">
       <c r="B18" s="88" t="s">
         <v>109</v>
       </c>
@@ -6918,7 +6940,7 @@
       <c r="H18" s="91"/>
       <c r="I18" s="95"/>
     </row>
-    <row r="19" spans="2:9" ht="57" customHeight="1">
+    <row r="19" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="87" t="s">
         <v>112</v>
       </c>
@@ -6936,7 +6958,7 @@
       <c r="H19" s="91"/>
       <c r="I19" s="95"/>
     </row>
-    <row r="20" spans="2:9" ht="57" customHeight="1">
+    <row r="20" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="87" t="s">
         <v>170</v>
       </c>
@@ -6954,7 +6976,7 @@
       <c r="H20" s="113"/>
       <c r="I20" s="114"/>
     </row>
-    <row r="21" spans="2:9" ht="57" customHeight="1" thickBot="1">
+    <row r="21" spans="2:9" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="89" t="s">
         <v>111</v>
       </c>
@@ -6972,7 +6994,7 @@
       <c r="H21" s="96"/>
       <c r="I21" s="97"/>
     </row>
-    <row r="22" spans="2:9" ht="14.25" thickTop="1"/>
+    <row r="22" spans="2:9" ht="14.25" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="B2:B3"/>

</xml_diff>

<commit_message>
2025. 7. 16. Weekly Plan 작성 완료
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\1. doc\HKMC_AIR_PTC\일정\PTC_HEATER_DOC (250626 Repo 변경, 해당 Repo 사용)\ptc_heater_doc\1. 일정\1. Weekly Plan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\일정\ptc_heater_doc\1. 일정\1. Weekly Plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="17685" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="17685" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="대일정" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="235">
   <si>
     <t>■</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1346,18 +1346,82 @@
   </si>
   <si>
     <t>[조현진 전임, 임제훈 사원]
-- SWE.1 SRS 작성 완료 : ~ 6/30
-   : 3.1 Hardware - Software Interface
-   : 3.2 CAN Communication - Software Interface
-   : 4.1 Software State Transition Requirements
-   : 4.2.1.1 LV Sensor Fault / LV Over Voltage_Under Voltage Fault
-   : 4.2.1.2 HV Sensor Fault / HV Over Voltage_Under Voltage Fault
-- SWE.2 SADS 작성 계획
-   : Component 다이어그램 작성
-   : LV Sensor Fault / LV Over Voltage_Under Voltage Fault 정적, 동적 작성
-   : HV Sensor Fault / HV Over Voltage_Under Voltage Fault 정적, 동적 작성
-- SWE.3 SDDS 작성 계획
-   : LV Sensor Fault 작성</t>
+- SWE.1 SRS 작성
+   : PCB Sensor Protection 작성
+   : PCB Temp Over Fault Detection 작성
+- SWE.2 SADS 작성
+   : PCB Sensor Protection 작성
+   : PCB Temp Over Fault Detection 작성
+- SWE.3 SDDS 작성
+   : HV Over Current Fault Detection Static Design, Dynamic Behavior 작성
+   : Current Sensor Protection Static Design, Dynamic Behavior 작성</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[조현진 전임, 임제훈 사원]
+- SWE.1 SRS 작성
+   : Hardware - Software Interface 작성
+   : CAN Communication - Software Interface 작성
+   : LV Sensor Protection 작성
+   : Low Voltage Battery Protection 작성
+   : HV Sensor Protection 작성
+   : High Voltage Battery Protection 작성
+- SWE.2 SADS 작성
+   : Software Component Overview Diagram 작성
+   : Software Component Overview Description 작성
+   : Protection Composition Diagram 작성
+   : Protection Composition attributes 작성
+   : Protection Component Diagram 작성</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[조현진 전임, 임제훈 사원]
+- SWE.1 SRS 작성
+   : Hardware - Software Interface (6/30)
+   : CAN Communication - Software Interface (6/30)
+   : Software State Transition Requirements (6/30)
+   : LV Sensor Protection (6/30)
+   : Low Voltage Battery Protection (6/30)
+   : HV Sensor Protection (6/30)
+   : High Voltage Battery Protection (6/30)
+   : Review Report 결과를 토대로 개선점 반영
+- SWE.2 SADS 작성
+   : Software Component Overview Diagram (7/1)
+   : Software Component Overview Description (7/2)
+   : Protection Composition Diagram (7/3)
+   : Protection Composition attributes (7/4)
+   : Protection Component Diagram (7/4)
+   : Structure Specification 작성
+   : Software Composition Design 작성
+   : Software Composition Attributes 작성
+   : LV Sensor Protection Static Design, Dynamic Behavior 작성
+   : Low Voltage Battery Protection Static Design, Dynamic Behavior 작성
+   : HV Sensor Protection Static Design, Dynamic Behavior 작성
+   : High Voltage Battery Protection Static Design, Dynamic Behavior 작성</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[조현진 전임, 임제훈 사원]
+- SWE.1 SRS 작성
+   : Review Report 결과를 토대로 개선점 반영 (7/11)
+   : Hardware - Software Interface의 SW Description 재작성
+   : HV Over Current Fault Detection 작성
+   : Current Sensor Protection 작성
+- SWE.2 SADS 작성
+   : Structure Specification (7/7)
+   : Software Composition Design (7/7)
+   : Software Composition Attributes (7/7)
+   : LV Sensor Protection Static Design, Dynamic Behavior (7/8)
+   : Low Voltage Battery Protection Static Design, Dynamic Behavior (7/8)
+   : HV Sensor Protection Static Design, Dynamic Behavior (7/11)
+   : High Voltage Battery Protection Static Design, Dynamic Behavior (7/11)
+   : HV Over Current Fault Detection 작성
+   : Current Sensor Protection 작성
+- SWE.3 SDDS 작성
+   : LV Sensor Protection Static Design, Dynamic Behavior 작성
+   : Low Voltage Battery Protection Static Design, Dynamic Behavior 작성
+   : HV Sensor Protection Static Design, Dynamic Behavior 작성
+   : High Voltage Battery Protection Static Design, Dynamic Behavior 작성</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2886,6 +2950,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="57" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2930,12 +3000,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="57" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3548,90 +3612,90 @@
       <c r="D1" s="21"/>
     </row>
     <row r="2" spans="1:64" ht="31.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="124" t="s">
+      <c r="B2" s="126" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="126" t="s">
+      <c r="C2" s="128" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="126" t="s">
+      <c r="D2" s="128" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="130">
+      <c r="E2" s="132">
         <v>23</v>
       </c>
-      <c r="F2" s="128"/>
-      <c r="G2" s="128"/>
-      <c r="H2" s="128"/>
-      <c r="I2" s="128"/>
-      <c r="J2" s="128"/>
-      <c r="K2" s="128"/>
-      <c r="L2" s="128"/>
-      <c r="M2" s="128"/>
-      <c r="N2" s="128"/>
-      <c r="O2" s="128"/>
-      <c r="P2" s="128"/>
-      <c r="Q2" s="128">
+      <c r="F2" s="130"/>
+      <c r="G2" s="130"/>
+      <c r="H2" s="130"/>
+      <c r="I2" s="130"/>
+      <c r="J2" s="130"/>
+      <c r="K2" s="130"/>
+      <c r="L2" s="130"/>
+      <c r="M2" s="130"/>
+      <c r="N2" s="130"/>
+      <c r="O2" s="130"/>
+      <c r="P2" s="130"/>
+      <c r="Q2" s="130">
         <v>24</v>
       </c>
-      <c r="R2" s="128"/>
-      <c r="S2" s="128"/>
-      <c r="T2" s="128"/>
-      <c r="U2" s="128"/>
-      <c r="V2" s="128"/>
-      <c r="W2" s="128"/>
-      <c r="X2" s="128"/>
-      <c r="Y2" s="128"/>
-      <c r="Z2" s="128"/>
-      <c r="AA2" s="128"/>
-      <c r="AB2" s="128"/>
-      <c r="AC2" s="128">
+      <c r="R2" s="130"/>
+      <c r="S2" s="130"/>
+      <c r="T2" s="130"/>
+      <c r="U2" s="130"/>
+      <c r="V2" s="130"/>
+      <c r="W2" s="130"/>
+      <c r="X2" s="130"/>
+      <c r="Y2" s="130"/>
+      <c r="Z2" s="130"/>
+      <c r="AA2" s="130"/>
+      <c r="AB2" s="130"/>
+      <c r="AC2" s="130">
         <v>25</v>
       </c>
-      <c r="AD2" s="128"/>
-      <c r="AE2" s="128"/>
-      <c r="AF2" s="128"/>
-      <c r="AG2" s="128"/>
-      <c r="AH2" s="128"/>
-      <c r="AI2" s="128"/>
-      <c r="AJ2" s="128"/>
-      <c r="AK2" s="128"/>
-      <c r="AL2" s="128"/>
-      <c r="AM2" s="128"/>
-      <c r="AN2" s="128"/>
-      <c r="AO2" s="128">
+      <c r="AD2" s="130"/>
+      <c r="AE2" s="130"/>
+      <c r="AF2" s="130"/>
+      <c r="AG2" s="130"/>
+      <c r="AH2" s="130"/>
+      <c r="AI2" s="130"/>
+      <c r="AJ2" s="130"/>
+      <c r="AK2" s="130"/>
+      <c r="AL2" s="130"/>
+      <c r="AM2" s="130"/>
+      <c r="AN2" s="130"/>
+      <c r="AO2" s="130">
         <v>26</v>
       </c>
-      <c r="AP2" s="128"/>
-      <c r="AQ2" s="128"/>
-      <c r="AR2" s="128"/>
-      <c r="AS2" s="128"/>
-      <c r="AT2" s="128"/>
-      <c r="AU2" s="128"/>
-      <c r="AV2" s="128"/>
-      <c r="AW2" s="128"/>
-      <c r="AX2" s="128"/>
-      <c r="AY2" s="128"/>
-      <c r="AZ2" s="129"/>
-      <c r="BA2" s="128">
+      <c r="AP2" s="130"/>
+      <c r="AQ2" s="130"/>
+      <c r="AR2" s="130"/>
+      <c r="AS2" s="130"/>
+      <c r="AT2" s="130"/>
+      <c r="AU2" s="130"/>
+      <c r="AV2" s="130"/>
+      <c r="AW2" s="130"/>
+      <c r="AX2" s="130"/>
+      <c r="AY2" s="130"/>
+      <c r="AZ2" s="131"/>
+      <c r="BA2" s="130">
         <v>27</v>
       </c>
-      <c r="BB2" s="128"/>
-      <c r="BC2" s="128"/>
-      <c r="BD2" s="128"/>
-      <c r="BE2" s="128"/>
-      <c r="BF2" s="128"/>
-      <c r="BG2" s="128"/>
-      <c r="BH2" s="128"/>
-      <c r="BI2" s="128"/>
-      <c r="BJ2" s="128"/>
-      <c r="BK2" s="128"/>
-      <c r="BL2" s="129"/>
+      <c r="BB2" s="130"/>
+      <c r="BC2" s="130"/>
+      <c r="BD2" s="130"/>
+      <c r="BE2" s="130"/>
+      <c r="BF2" s="130"/>
+      <c r="BG2" s="130"/>
+      <c r="BH2" s="130"/>
+      <c r="BI2" s="130"/>
+      <c r="BJ2" s="130"/>
+      <c r="BK2" s="130"/>
+      <c r="BL2" s="131"/>
     </row>
     <row r="3" spans="1:64" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="125"/>
-      <c r="C3" s="127"/>
-      <c r="D3" s="127"/>
+      <c r="B3" s="127"/>
+      <c r="C3" s="129"/>
+      <c r="D3" s="129"/>
       <c r="E3" s="22">
         <v>1</v>
       </c>
@@ -5457,39 +5521,39 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="133" t="s">
+      <c r="B2" s="135" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="137" t="s">
+      <c r="C2" s="139" t="s">
         <v>179</v>
       </c>
-      <c r="D2" s="137" t="s">
+      <c r="D2" s="139" t="s">
         <v>180</v>
       </c>
-      <c r="E2" s="135" t="s">
+      <c r="E2" s="137" t="s">
         <v>129</v>
       </c>
       <c r="F2" s="98" t="s">
         <v>115</v>
       </c>
-      <c r="G2" s="131" t="s">
+      <c r="G2" s="133" t="s">
         <v>116</v>
       </c>
-      <c r="H2" s="131"/>
-      <c r="I2" s="131"/>
-      <c r="J2" s="132"/>
-      <c r="K2" s="131" t="s">
+      <c r="H2" s="133"/>
+      <c r="I2" s="133"/>
+      <c r="J2" s="134"/>
+      <c r="K2" s="133" t="s">
         <v>185</v>
       </c>
-      <c r="L2" s="131"/>
-      <c r="M2" s="131"/>
-      <c r="N2" s="132"/>
+      <c r="L2" s="133"/>
+      <c r="M2" s="133"/>
+      <c r="N2" s="134"/>
     </row>
     <row r="3" spans="1:14" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="134"/>
-      <c r="C3" s="138"/>
-      <c r="D3" s="138"/>
-      <c r="E3" s="136"/>
+      <c r="B3" s="136"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="140"/>
+      <c r="E3" s="138"/>
       <c r="F3" s="99" t="s">
         <v>114</v>
       </c>
@@ -6232,30 +6296,30 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="133" t="s">
+      <c r="B2" s="135" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="137" t="s">
+      <c r="C2" s="139" t="s">
         <v>179</v>
       </c>
-      <c r="D2" s="137" t="s">
+      <c r="D2" s="139" t="s">
         <v>180</v>
       </c>
-      <c r="E2" s="135" t="s">
+      <c r="E2" s="137" t="s">
         <v>129</v>
       </c>
-      <c r="F2" s="131" t="s">
+      <c r="F2" s="133" t="s">
         <v>185</v>
       </c>
-      <c r="G2" s="131"/>
-      <c r="H2" s="131"/>
-      <c r="I2" s="132"/>
+      <c r="G2" s="133"/>
+      <c r="H2" s="133"/>
+      <c r="I2" s="134"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="134"/>
-      <c r="C3" s="138"/>
-      <c r="D3" s="138"/>
-      <c r="E3" s="136"/>
+      <c r="B3" s="136"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="140"/>
+      <c r="E3" s="138"/>
       <c r="F3" s="99" t="s">
         <v>117</v>
       </c>
@@ -6463,7 +6527,7 @@
       <c r="F14" s="116"/>
       <c r="G14" s="107"/>
       <c r="H14" s="91"/>
-      <c r="I14" s="139" t="s">
+      <c r="I14" s="124" t="s">
         <v>223</v>
       </c>
     </row>
@@ -6633,30 +6697,30 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="133" t="s">
+      <c r="B2" s="135" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="137" t="s">
+      <c r="C2" s="139" t="s">
         <v>179</v>
       </c>
-      <c r="D2" s="137" t="s">
+      <c r="D2" s="139" t="s">
         <v>180</v>
       </c>
-      <c r="E2" s="135" t="s">
+      <c r="E2" s="137" t="s">
         <v>129</v>
       </c>
-      <c r="F2" s="131" t="s">
+      <c r="F2" s="133" t="s">
         <v>230</v>
       </c>
-      <c r="G2" s="131"/>
-      <c r="H2" s="131"/>
-      <c r="I2" s="132"/>
+      <c r="G2" s="133"/>
+      <c r="H2" s="133"/>
+      <c r="I2" s="134"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="134"/>
-      <c r="C3" s="138"/>
-      <c r="D3" s="138"/>
-      <c r="E3" s="136"/>
+      <c r="B3" s="136"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="140"/>
+      <c r="E3" s="138"/>
       <c r="F3" s="99" t="s">
         <v>117</v>
       </c>
@@ -6850,7 +6914,7 @@
       <c r="H13" s="91"/>
       <c r="I13" s="95"/>
     </row>
-    <row r="14" spans="1:9" ht="229.5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="337.5" x14ac:dyDescent="0.3">
       <c r="B14" s="87" t="s">
         <v>184</v>
       </c>
@@ -6861,12 +6925,18 @@
         <v>183</v>
       </c>
       <c r="E14" s="102"/>
-      <c r="F14" s="140" t="s">
+      <c r="F14" s="125" t="s">
+        <v>232</v>
+      </c>
+      <c r="G14" s="125" t="s">
+        <v>233</v>
+      </c>
+      <c r="H14" s="125" t="s">
+        <v>234</v>
+      </c>
+      <c r="I14" s="125" t="s">
         <v>231</v>
       </c>
-      <c r="G14" s="107"/>
-      <c r="H14" s="91"/>
-      <c r="I14" s="139"/>
     </row>
     <row r="15" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="87" t="s">

</xml_diff>

<commit_message>
25. 10. 13. Weekly Plan 내 Heater 업무 분배 작성
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\2.project\hkmc_ptc_heater\Doc\1. 일정\1. Weekly Plan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\일정\ptc_heater_doc\1. 일정\1. Weekly Plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="17685"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="17685" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="대일정" sheetId="1" r:id="rId1"/>
-    <sheet name="2025.5" sheetId="2" r:id="rId2"/>
-    <sheet name="2025.6" sheetId="3" r:id="rId3"/>
-    <sheet name="2025.7" sheetId="4" r:id="rId4"/>
+    <sheet name="업무 분배" sheetId="5" r:id="rId2"/>
+    <sheet name="2025.5" sheetId="2" r:id="rId3"/>
+    <sheet name="2025.6" sheetId="3" r:id="rId4"/>
+    <sheet name="2025.7" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="259">
   <si>
     <t>■</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1444,6 +1445,86 @@
 10/15</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>양산 중</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>진행 중</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mva</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>조현진 전임</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AY, HE1I</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>임제훈 사원</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Nea</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>QV</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mea</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SVm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cva</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BJ1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SU2I</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NX5e, NQ6e</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SX3e</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NEaW</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MX5a</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SUZUKI</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>오세영 수석</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -1452,7 +1533,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="mm&quot;월&quot;\ dd&quot;일&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1550,8 +1631,40 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1582,6 +1695,32 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="73">
     <border>
@@ -2592,12 +2731,27 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3021,8 +3175,28 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" xfId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="3">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
+    <cellStyle name="60% - 강조색3" xfId="4" builtinId="40"/>
+    <cellStyle name="강조색5" xfId="5" builtinId="45"/>
+    <cellStyle name="나쁨" xfId="2" builtinId="27"/>
+    <cellStyle name="보통" xfId="3" builtinId="28"/>
+    <cellStyle name="좋음" xfId="1" builtinId="26"/>
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3610,7 +3784,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BL24"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.375" customWidth="1"/>
     <col min="2" max="2" width="18.875" customWidth="1"/>
@@ -3621,7 +3795,7 @@
     <col min="36" max="64" width="8.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:64" s="20" customFormat="1" ht="32.25" thickBot="1">
+    <row r="1" spans="1:64" s="20" customFormat="1" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
@@ -3631,7 +3805,7 @@
       <c r="C1" s="21"/>
       <c r="D1" s="21"/>
     </row>
-    <row r="2" spans="1:64" ht="31.5" customHeight="1" thickTop="1">
+    <row r="2" spans="1:64" ht="31.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B2" s="126" t="s">
         <v>2</v>
       </c>
@@ -3712,7 +3886,7 @@
       <c r="BK2" s="130"/>
       <c r="BL2" s="131"/>
     </row>
-    <row r="3" spans="1:64" ht="31.5" customHeight="1" thickBot="1">
+    <row r="3" spans="1:64" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="127"/>
       <c r="C3" s="129"/>
       <c r="D3" s="129"/>
@@ -3897,7 +4071,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:64" ht="183" customHeight="1" thickBot="1">
+    <row r="4" spans="1:64" ht="183" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="63" t="s">
         <v>120</v>
       </c>
@@ -3978,7 +4152,7 @@
       <c r="BK4" s="2"/>
       <c r="BL4" s="5"/>
     </row>
-    <row r="5" spans="1:64" ht="81">
+    <row r="5" spans="1:64" ht="81" x14ac:dyDescent="0.3">
       <c r="B5" s="28" t="s">
         <v>121</v>
       </c>
@@ -4057,7 +4231,7 @@
       <c r="BK5" s="31"/>
       <c r="BL5" s="10"/>
     </row>
-    <row r="6" spans="1:64" ht="67.5">
+    <row r="6" spans="1:64" ht="67.5" x14ac:dyDescent="0.3">
       <c r="B6" s="28" t="s">
         <v>122</v>
       </c>
@@ -4140,7 +4314,7 @@
       <c r="BK6" s="31"/>
       <c r="BL6" s="10"/>
     </row>
-    <row r="7" spans="1:64" ht="61.5" customHeight="1">
+    <row r="7" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="28" t="s">
         <v>123</v>
       </c>
@@ -4221,7 +4395,7 @@
       <c r="BK7" s="31"/>
       <c r="BL7" s="10"/>
     </row>
-    <row r="8" spans="1:64" ht="81">
+    <row r="8" spans="1:64" ht="81" x14ac:dyDescent="0.3">
       <c r="B8" s="28" t="s">
         <v>222</v>
       </c>
@@ -4298,7 +4472,7 @@
       <c r="BK8" s="31"/>
       <c r="BL8" s="10"/>
     </row>
-    <row r="9" spans="1:64" ht="61.5" customHeight="1">
+    <row r="9" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="27" t="s">
         <v>3</v>
       </c>
@@ -4371,7 +4545,7 @@
       <c r="BK9" s="31"/>
       <c r="BL9" s="10"/>
     </row>
-    <row r="10" spans="1:64" ht="61.5" customHeight="1">
+    <row r="10" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="27" t="s">
         <v>46</v>
       </c>
@@ -4448,7 +4622,7 @@
       <c r="BK10" s="31"/>
       <c r="BL10" s="10"/>
     </row>
-    <row r="11" spans="1:64" ht="61.5" customHeight="1">
+    <row r="11" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="28" t="s">
         <v>128</v>
       </c>
@@ -4529,7 +4703,7 @@
       <c r="BK11" s="31"/>
       <c r="BL11" s="10"/>
     </row>
-    <row r="12" spans="1:64" ht="61.5" customHeight="1">
+    <row r="12" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="28" t="s">
         <v>129</v>
       </c>
@@ -4608,7 +4782,7 @@
       <c r="BK12" s="31"/>
       <c r="BL12" s="10"/>
     </row>
-    <row r="13" spans="1:64" ht="183.75" customHeight="1">
+    <row r="13" spans="1:64" ht="183.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="28" t="s">
         <v>63</v>
       </c>
@@ -4697,7 +4871,7 @@
       <c r="BK13" s="31"/>
       <c r="BL13" s="10"/>
     </row>
-    <row r="14" spans="1:64" ht="67.5">
+    <row r="14" spans="1:64" ht="67.5" x14ac:dyDescent="0.3">
       <c r="B14" s="27" t="s">
         <v>74</v>
       </c>
@@ -4786,7 +4960,7 @@
       <c r="BK14" s="31"/>
       <c r="BL14" s="10"/>
     </row>
-    <row r="15" spans="1:64" ht="61.5" customHeight="1">
+    <row r="15" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="27" t="s">
         <v>65</v>
       </c>
@@ -4867,7 +5041,7 @@
       <c r="BK15" s="31"/>
       <c r="BL15" s="10"/>
     </row>
-    <row r="16" spans="1:64" ht="61.5" customHeight="1">
+    <row r="16" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="27" t="s">
         <v>66</v>
       </c>
@@ -4956,7 +5130,7 @@
       <c r="BK16" s="31"/>
       <c r="BL16" s="10"/>
     </row>
-    <row r="17" spans="2:64" ht="61.5" customHeight="1">
+    <row r="17" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="57" t="s">
         <v>76</v>
       </c>
@@ -5043,7 +5217,7 @@
       <c r="BK17" s="71"/>
       <c r="BL17" s="48"/>
     </row>
-    <row r="18" spans="2:64" ht="76.5" customHeight="1">
+    <row r="18" spans="2:64" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="27" t="s">
         <v>86</v>
       </c>
@@ -5134,7 +5308,7 @@
       <c r="BK18" s="73"/>
       <c r="BL18" s="70"/>
     </row>
-    <row r="19" spans="2:64" ht="61.5" customHeight="1">
+    <row r="19" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="77" t="s">
         <v>142</v>
       </c>
@@ -5219,7 +5393,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="2:64" ht="61.5" customHeight="1">
+    <row r="20" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="77" t="s">
         <v>107</v>
       </c>
@@ -5288,7 +5462,7 @@
       <c r="BK20" s="73"/>
       <c r="BL20" s="70"/>
     </row>
-    <row r="21" spans="2:64" ht="61.5" customHeight="1">
+    <row r="21" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="57" t="s">
         <v>110</v>
       </c>
@@ -5369,7 +5543,7 @@
       <c r="BK21" s="73"/>
       <c r="BL21" s="70"/>
     </row>
-    <row r="22" spans="2:64" ht="61.5" customHeight="1">
+    <row r="22" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="57" t="s">
         <v>167</v>
       </c>
@@ -5438,7 +5612,7 @@
       <c r="BK22" s="73"/>
       <c r="BL22" s="70"/>
     </row>
-    <row r="23" spans="2:64" ht="61.5" customHeight="1" thickBot="1">
+    <row r="23" spans="2:64" ht="61.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="79" t="s">
         <v>168</v>
       </c>
@@ -5507,7 +5681,7 @@
       <c r="BK23" s="75"/>
       <c r="BL23" s="55"/>
     </row>
-    <row r="24" spans="2:64" ht="17.25" thickTop="1"/>
+    <row r="24" spans="2:64" ht="17.25" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="B2:B3"/>
@@ -5527,9 +5701,140 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>239</v>
+      </c>
+      <c r="C1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="141" t="s">
+        <v>241</v>
+      </c>
+      <c r="B2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C2" s="142" t="s">
+        <v>243</v>
+      </c>
+      <c r="D2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="141" t="s">
+        <v>245</v>
+      </c>
+      <c r="B3" t="s">
+        <v>242</v>
+      </c>
+      <c r="C3" s="143" t="s">
+        <v>246</v>
+      </c>
+      <c r="D3" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="141" t="s">
+        <v>247</v>
+      </c>
+      <c r="B4" t="s">
+        <v>242</v>
+      </c>
+      <c r="C4" s="143" t="s">
+        <v>248</v>
+      </c>
+      <c r="D4" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="144" t="s">
+        <v>249</v>
+      </c>
+      <c r="B5" t="s">
+        <v>242</v>
+      </c>
+      <c r="C5" s="143" t="s">
+        <v>250</v>
+      </c>
+      <c r="D5" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="142" t="s">
+        <v>251</v>
+      </c>
+      <c r="B6" t="s">
+        <v>244</v>
+      </c>
+      <c r="C6" s="145" t="s">
+        <v>252</v>
+      </c>
+      <c r="D6" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="142" t="s">
+        <v>253</v>
+      </c>
+      <c r="B7" t="s">
+        <v>244</v>
+      </c>
+      <c r="C7" s="145" t="s">
+        <v>254</v>
+      </c>
+      <c r="D7" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C8" s="141" t="s">
+        <v>255</v>
+      </c>
+      <c r="D8" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C9" s="141" t="s">
+        <v>256</v>
+      </c>
+      <c r="D9" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C10" s="145" t="s">
+        <v>257</v>
+      </c>
+      <c r="D10" t="s">
+        <v>258</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.375" style="83" customWidth="1"/>
     <col min="2" max="2" width="9" style="83"/>
@@ -5541,7 +5846,7 @@
     <col min="15" max="16384" width="9" style="83"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="32.25" thickBot="1">
+    <row r="1" spans="1:14" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="110" t="s">
         <v>149</v>
       </c>
@@ -5552,7 +5857,7 @@
       <c r="D1" s="111"/>
       <c r="E1" s="109"/>
     </row>
-    <row r="2" spans="1:14" ht="30" customHeight="1" thickTop="1">
+    <row r="2" spans="1:14" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B2" s="135" t="s">
         <v>2</v>
       </c>
@@ -5581,7 +5886,7 @@
       <c r="M2" s="133"/>
       <c r="N2" s="134"/>
     </row>
-    <row r="3" spans="1:14" ht="37.5" customHeight="1" thickBot="1">
+    <row r="3" spans="1:14" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="136"/>
       <c r="C3" s="140"/>
       <c r="D3" s="140"/>
@@ -5614,7 +5919,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="108">
+    <row r="4" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B4" s="84" t="s">
         <v>118</v>
       </c>
@@ -5649,7 +5954,7 @@
       <c r="M4" s="107"/>
       <c r="N4" s="94"/>
     </row>
-    <row r="5" spans="1:14" ht="108">
+    <row r="5" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B5" s="85" t="s">
         <v>124</v>
       </c>
@@ -5684,7 +5989,7 @@
       <c r="M5" s="107"/>
       <c r="N5" s="95"/>
     </row>
-    <row r="6" spans="1:14" ht="108">
+    <row r="6" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B6" s="85" t="s">
         <v>125</v>
       </c>
@@ -5719,7 +6024,7 @@
       <c r="M6" s="107"/>
       <c r="N6" s="95"/>
     </row>
-    <row r="7" spans="1:14" ht="108">
+    <row r="7" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B7" s="85" t="s">
         <v>126</v>
       </c>
@@ -5754,7 +6059,7 @@
       <c r="M7" s="107"/>
       <c r="N7" s="95"/>
     </row>
-    <row r="8" spans="1:14" ht="108">
+    <row r="8" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B8" s="86" t="s">
         <v>3</v>
       </c>
@@ -5789,7 +6094,7 @@
       <c r="M8" s="107"/>
       <c r="N8" s="95"/>
     </row>
-    <row r="9" spans="1:14" ht="175.5">
+    <row r="9" spans="1:14" ht="175.5" x14ac:dyDescent="0.3">
       <c r="B9" s="86" t="s">
         <v>46</v>
       </c>
@@ -5824,7 +6129,7 @@
       <c r="M9" s="107"/>
       <c r="N9" s="95"/>
     </row>
-    <row r="10" spans="1:14" ht="121.5">
+    <row r="10" spans="1:14" ht="121.5" x14ac:dyDescent="0.3">
       <c r="B10" s="86" t="s">
         <v>56</v>
       </c>
@@ -5859,7 +6164,7 @@
       <c r="M10" s="107"/>
       <c r="N10" s="95"/>
     </row>
-    <row r="11" spans="1:14" ht="108">
+    <row r="11" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B11" s="85" t="s">
         <v>63</v>
       </c>
@@ -5894,7 +6199,7 @@
       <c r="M11" s="107"/>
       <c r="N11" s="95"/>
     </row>
-    <row r="12" spans="1:14" ht="57" customHeight="1">
+    <row r="12" spans="1:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="86" t="s">
         <v>74</v>
       </c>
@@ -5929,7 +6234,7 @@
       <c r="M12" s="107"/>
       <c r="N12" s="95"/>
     </row>
-    <row r="13" spans="1:14" ht="347.25" customHeight="1">
+    <row r="13" spans="1:14" ht="347.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="86" t="s">
         <v>119</v>
       </c>
@@ -5964,7 +6269,7 @@
       <c r="M13" s="107"/>
       <c r="N13" s="95"/>
     </row>
-    <row r="14" spans="1:14" ht="175.5">
+    <row r="14" spans="1:14" ht="175.5" x14ac:dyDescent="0.3">
       <c r="B14" s="87" t="s">
         <v>182</v>
       </c>
@@ -5993,7 +6298,7 @@
       <c r="M14" s="107"/>
       <c r="N14" s="95"/>
     </row>
-    <row r="15" spans="1:14" ht="57" customHeight="1">
+    <row r="15" spans="1:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="87" t="s">
         <v>76</v>
       </c>
@@ -6026,7 +6331,7 @@
       <c r="M15" s="107"/>
       <c r="N15" s="95"/>
     </row>
-    <row r="16" spans="1:14" ht="121.5">
+    <row r="16" spans="1:14" ht="121.5" x14ac:dyDescent="0.3">
       <c r="B16" s="86" t="s">
         <v>86</v>
       </c>
@@ -6059,7 +6364,7 @@
       <c r="M16" s="107"/>
       <c r="N16" s="95"/>
     </row>
-    <row r="17" spans="2:14" ht="57" customHeight="1">
+    <row r="17" spans="2:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="88" t="s">
         <v>142</v>
       </c>
@@ -6092,7 +6397,7 @@
       <c r="M17" s="91"/>
       <c r="N17" s="95"/>
     </row>
-    <row r="18" spans="2:14" ht="162">
+    <row r="18" spans="2:14" ht="162" x14ac:dyDescent="0.3">
       <c r="B18" s="88" t="s">
         <v>107</v>
       </c>
@@ -6127,7 +6432,7 @@
       <c r="M18" s="107"/>
       <c r="N18" s="95"/>
     </row>
-    <row r="19" spans="2:14" ht="57" customHeight="1">
+    <row r="19" spans="2:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="87" t="s">
         <v>110</v>
       </c>
@@ -6162,7 +6467,7 @@
       <c r="M19" s="107"/>
       <c r="N19" s="95"/>
     </row>
-    <row r="20" spans="2:14" ht="57" customHeight="1">
+    <row r="20" spans="2:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="87" t="s">
         <v>169</v>
       </c>
@@ -6197,7 +6502,7 @@
       <c r="M20" s="107"/>
       <c r="N20" s="114"/>
     </row>
-    <row r="21" spans="2:14" ht="57" customHeight="1" thickBot="1">
+    <row r="21" spans="2:14" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="89" t="s">
         <v>109</v>
       </c>
@@ -6232,7 +6537,7 @@
       <c r="M21" s="122"/>
       <c r="N21" s="97"/>
     </row>
-    <row r="22" spans="2:14" ht="14.25" thickTop="1"/>
+    <row r="22" spans="2:14" ht="14.25" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="K2:N2"/>
@@ -6302,10 +6607,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.375" style="83" customWidth="1"/>
     <col min="2" max="2" width="9" style="83"/>
@@ -6316,7 +6621,7 @@
     <col min="10" max="16384" width="9" style="83"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.25" thickBot="1">
+    <row r="1" spans="1:9" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="110" t="s">
         <v>0</v>
       </c>
@@ -6327,7 +6632,7 @@
       <c r="D1" s="111"/>
       <c r="E1" s="109"/>
     </row>
-    <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1">
+    <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B2" s="135" t="s">
         <v>2</v>
       </c>
@@ -6347,7 +6652,7 @@
       <c r="H2" s="133"/>
       <c r="I2" s="134"/>
     </row>
-    <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1">
+    <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="136"/>
       <c r="C3" s="140"/>
       <c r="D3" s="140"/>
@@ -6365,7 +6670,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="57" customHeight="1">
+    <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="84" t="s">
         <v>118</v>
       </c>
@@ -6383,7 +6688,7 @@
       <c r="H4" s="90"/>
       <c r="I4" s="94"/>
     </row>
-    <row r="5" spans="1:9" ht="57" customHeight="1">
+    <row r="5" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="85" t="s">
         <v>124</v>
       </c>
@@ -6401,7 +6706,7 @@
       <c r="H5" s="91"/>
       <c r="I5" s="95"/>
     </row>
-    <row r="6" spans="1:9" ht="57" customHeight="1">
+    <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="85" t="s">
         <v>125</v>
       </c>
@@ -6419,7 +6724,7 @@
       <c r="H6" s="91"/>
       <c r="I6" s="95"/>
     </row>
-    <row r="7" spans="1:9" ht="57" customHeight="1">
+    <row r="7" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="85" t="s">
         <v>126</v>
       </c>
@@ -6437,7 +6742,7 @@
       <c r="H7" s="91"/>
       <c r="I7" s="95"/>
     </row>
-    <row r="8" spans="1:9" ht="57" customHeight="1">
+    <row r="8" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="86" t="s">
         <v>3</v>
       </c>
@@ -6455,7 +6760,7 @@
       <c r="H8" s="91"/>
       <c r="I8" s="95"/>
     </row>
-    <row r="9" spans="1:9" ht="27">
+    <row r="9" spans="1:9" ht="27" x14ac:dyDescent="0.3">
       <c r="B9" s="86" t="s">
         <v>46</v>
       </c>
@@ -6473,7 +6778,7 @@
       <c r="H9" s="91"/>
       <c r="I9" s="95"/>
     </row>
-    <row r="10" spans="1:9" ht="57" customHeight="1">
+    <row r="10" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="86" t="s">
         <v>56</v>
       </c>
@@ -6491,7 +6796,7 @@
       <c r="H10" s="91"/>
       <c r="I10" s="95"/>
     </row>
-    <row r="11" spans="1:9" ht="40.5">
+    <row r="11" spans="1:9" ht="40.5" x14ac:dyDescent="0.3">
       <c r="B11" s="85" t="s">
         <v>63</v>
       </c>
@@ -6509,7 +6814,7 @@
       <c r="H11" s="91"/>
       <c r="I11" s="95"/>
     </row>
-    <row r="12" spans="1:9" ht="57" customHeight="1">
+    <row r="12" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="86" t="s">
         <v>74</v>
       </c>
@@ -6527,7 +6832,7 @@
       <c r="H12" s="91"/>
       <c r="I12" s="95"/>
     </row>
-    <row r="13" spans="1:9" ht="347.25" customHeight="1">
+    <row r="13" spans="1:9" ht="347.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="86" t="s">
         <v>119</v>
       </c>
@@ -6545,7 +6850,7 @@
       <c r="H13" s="91"/>
       <c r="I13" s="95"/>
     </row>
-    <row r="14" spans="1:9" ht="409.5">
+    <row r="14" spans="1:9" ht="409.5" x14ac:dyDescent="0.3">
       <c r="B14" s="87" t="s">
         <v>182</v>
       </c>
@@ -6563,7 +6868,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="57" customHeight="1">
+    <row r="15" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="87" t="s">
         <v>76</v>
       </c>
@@ -6581,7 +6886,7 @@
       <c r="H15" s="91"/>
       <c r="I15" s="95"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B16" s="86" t="s">
         <v>86</v>
       </c>
@@ -6599,7 +6904,7 @@
       <c r="H16" s="91"/>
       <c r="I16" s="95"/>
     </row>
-    <row r="17" spans="2:9" ht="57" customHeight="1">
+    <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="88" t="s">
         <v>142</v>
       </c>
@@ -6617,7 +6922,7 @@
       <c r="H17" s="91"/>
       <c r="I17" s="95"/>
     </row>
-    <row r="18" spans="2:9" ht="27">
+    <row r="18" spans="2:9" ht="27" x14ac:dyDescent="0.3">
       <c r="B18" s="88" t="s">
         <v>107</v>
       </c>
@@ -6635,7 +6940,7 @@
       <c r="H18" s="91"/>
       <c r="I18" s="95"/>
     </row>
-    <row r="19" spans="2:9" ht="57" customHeight="1">
+    <row r="19" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="87" t="s">
         <v>110</v>
       </c>
@@ -6653,7 +6958,7 @@
       <c r="H19" s="91"/>
       <c r="I19" s="95"/>
     </row>
-    <row r="20" spans="2:9" ht="57" customHeight="1">
+    <row r="20" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="87" t="s">
         <v>168</v>
       </c>
@@ -6671,7 +6976,7 @@
       <c r="H20" s="113"/>
       <c r="I20" s="114"/>
     </row>
-    <row r="21" spans="2:9" ht="57" customHeight="1" thickBot="1">
+    <row r="21" spans="2:9" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="89" t="s">
         <v>109</v>
       </c>
@@ -6689,7 +6994,7 @@
       <c r="H21" s="96"/>
       <c r="I21" s="97"/>
     </row>
-    <row r="22" spans="2:9" ht="14.25" thickTop="1"/>
+    <row r="22" spans="2:9" ht="14.25" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="B2:B3"/>
@@ -6703,10 +7008,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.375" style="83" customWidth="1"/>
     <col min="2" max="2" width="9" style="83"/>
@@ -6717,7 +7022,7 @@
     <col min="10" max="16384" width="9" style="83"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.25" thickBot="1">
+    <row r="1" spans="1:9" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="110" t="s">
         <v>0</v>
       </c>
@@ -6728,7 +7033,7 @@
       <c r="D1" s="111"/>
       <c r="E1" s="109"/>
     </row>
-    <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1">
+    <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B2" s="135" t="s">
         <v>2</v>
       </c>
@@ -6748,7 +7053,7 @@
       <c r="H2" s="133"/>
       <c r="I2" s="134"/>
     </row>
-    <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1">
+    <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="136"/>
       <c r="C3" s="140"/>
       <c r="D3" s="140"/>
@@ -6766,7 +7071,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="57" customHeight="1">
+    <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="84" t="s">
         <v>118</v>
       </c>
@@ -6784,7 +7089,7 @@
       <c r="H4" s="90"/>
       <c r="I4" s="94"/>
     </row>
-    <row r="5" spans="1:9" ht="57" customHeight="1">
+    <row r="5" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="85" t="s">
         <v>124</v>
       </c>
@@ -6802,7 +7107,7 @@
       <c r="H5" s="91"/>
       <c r="I5" s="95"/>
     </row>
-    <row r="6" spans="1:9" ht="57" customHeight="1">
+    <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="85" t="s">
         <v>125</v>
       </c>
@@ -6820,7 +7125,7 @@
       <c r="H6" s="91"/>
       <c r="I6" s="95"/>
     </row>
-    <row r="7" spans="1:9" ht="57" customHeight="1">
+    <row r="7" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="85" t="s">
         <v>126</v>
       </c>
@@ -6838,7 +7143,7 @@
       <c r="H7" s="91"/>
       <c r="I7" s="95"/>
     </row>
-    <row r="8" spans="1:9" ht="57" customHeight="1">
+    <row r="8" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="86" t="s">
         <v>3</v>
       </c>
@@ -6856,7 +7161,7 @@
       <c r="H8" s="91"/>
       <c r="I8" s="95"/>
     </row>
-    <row r="9" spans="1:9" ht="27">
+    <row r="9" spans="1:9" ht="27" x14ac:dyDescent="0.3">
       <c r="B9" s="86" t="s">
         <v>46</v>
       </c>
@@ -6874,7 +7179,7 @@
       <c r="H9" s="91"/>
       <c r="I9" s="95"/>
     </row>
-    <row r="10" spans="1:9" ht="57" customHeight="1">
+    <row r="10" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="86" t="s">
         <v>56</v>
       </c>
@@ -6892,7 +7197,7 @@
       <c r="H10" s="91"/>
       <c r="I10" s="95"/>
     </row>
-    <row r="11" spans="1:9" ht="40.5">
+    <row r="11" spans="1:9" ht="40.5" x14ac:dyDescent="0.3">
       <c r="B11" s="85" t="s">
         <v>63</v>
       </c>
@@ -6910,7 +7215,7 @@
       <c r="H11" s="91"/>
       <c r="I11" s="95"/>
     </row>
-    <row r="12" spans="1:9" ht="57" customHeight="1">
+    <row r="12" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="86" t="s">
         <v>74</v>
       </c>
@@ -6928,7 +7233,7 @@
       <c r="H12" s="91"/>
       <c r="I12" s="95"/>
     </row>
-    <row r="13" spans="1:9" ht="347.25" customHeight="1">
+    <row r="13" spans="1:9" ht="347.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="86" t="s">
         <v>119</v>
       </c>
@@ -6946,7 +7251,7 @@
       <c r="H13" s="91"/>
       <c r="I13" s="95"/>
     </row>
-    <row r="14" spans="1:9" ht="337.5">
+    <row r="14" spans="1:9" ht="337.5" x14ac:dyDescent="0.3">
       <c r="B14" s="87" t="s">
         <v>182</v>
       </c>
@@ -6970,7 +7275,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="57" customHeight="1">
+    <row r="15" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="87" t="s">
         <v>76</v>
       </c>
@@ -6988,7 +7293,7 @@
       <c r="H15" s="91"/>
       <c r="I15" s="95"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B16" s="86" t="s">
         <v>86</v>
       </c>
@@ -7006,7 +7311,7 @@
       <c r="H16" s="91"/>
       <c r="I16" s="95"/>
     </row>
-    <row r="17" spans="2:9" ht="57" customHeight="1">
+    <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="88" t="s">
         <v>142</v>
       </c>
@@ -7024,7 +7329,7 @@
       <c r="H17" s="91"/>
       <c r="I17" s="95"/>
     </row>
-    <row r="18" spans="2:9" ht="27">
+    <row r="18" spans="2:9" ht="27" x14ac:dyDescent="0.3">
       <c r="B18" s="88" t="s">
         <v>107</v>
       </c>
@@ -7042,7 +7347,7 @@
       <c r="H18" s="91"/>
       <c r="I18" s="95"/>
     </row>
-    <row r="19" spans="2:9" ht="57" customHeight="1">
+    <row r="19" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="87" t="s">
         <v>110</v>
       </c>
@@ -7060,7 +7365,7 @@
       <c r="H19" s="91"/>
       <c r="I19" s="95"/>
     </row>
-    <row r="20" spans="2:9" ht="57" customHeight="1">
+    <row r="20" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="87" t="s">
         <v>168</v>
       </c>
@@ -7078,7 +7383,7 @@
       <c r="H20" s="113"/>
       <c r="I20" s="114"/>
     </row>
-    <row r="21" spans="2:9" ht="57" customHeight="1" thickBot="1">
+    <row r="21" spans="2:9" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="89" t="s">
         <v>109</v>
       </c>
@@ -7096,7 +7401,7 @@
       <c r="H21" s="96"/>
       <c r="I21" s="97"/>
     </row>
-    <row r="22" spans="2:9" ht="14.25" thickTop="1"/>
+    <row r="22" spans="2:9" ht="14.25" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="B2:B3"/>

</xml_diff>

<commit_message>
Weeklty Plan, NX5e ESIR P/NO 작성 완료
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="17685" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="17685"/>
   </bookViews>
   <sheets>
     <sheet name="대일정" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="260">
   <si>
     <t>■</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1523,6 +1523,10 @@
   </si>
   <si>
     <t>오세영 수석</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>97191NU000(LHD)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3130,6 +3134,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="57" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" xfId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="3">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3174,21 +3193,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" xfId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="3">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -3806,90 +3810,90 @@
       <c r="D1" s="21"/>
     </row>
     <row r="2" spans="1:64" ht="31.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="126" t="s">
+      <c r="B2" s="131" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="128" t="s">
+      <c r="C2" s="133" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="128" t="s">
+      <c r="D2" s="133" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="132">
+      <c r="E2" s="137">
         <v>23</v>
       </c>
-      <c r="F2" s="130"/>
-      <c r="G2" s="130"/>
-      <c r="H2" s="130"/>
-      <c r="I2" s="130"/>
-      <c r="J2" s="130"/>
-      <c r="K2" s="130"/>
-      <c r="L2" s="130"/>
-      <c r="M2" s="130"/>
-      <c r="N2" s="130"/>
-      <c r="O2" s="130"/>
-      <c r="P2" s="130"/>
-      <c r="Q2" s="130">
+      <c r="F2" s="135"/>
+      <c r="G2" s="135"/>
+      <c r="H2" s="135"/>
+      <c r="I2" s="135"/>
+      <c r="J2" s="135"/>
+      <c r="K2" s="135"/>
+      <c r="L2" s="135"/>
+      <c r="M2" s="135"/>
+      <c r="N2" s="135"/>
+      <c r="O2" s="135"/>
+      <c r="P2" s="135"/>
+      <c r="Q2" s="135">
         <v>24</v>
       </c>
-      <c r="R2" s="130"/>
-      <c r="S2" s="130"/>
-      <c r="T2" s="130"/>
-      <c r="U2" s="130"/>
-      <c r="V2" s="130"/>
-      <c r="W2" s="130"/>
-      <c r="X2" s="130"/>
-      <c r="Y2" s="130"/>
-      <c r="Z2" s="130"/>
-      <c r="AA2" s="130"/>
-      <c r="AB2" s="130"/>
-      <c r="AC2" s="130">
+      <c r="R2" s="135"/>
+      <c r="S2" s="135"/>
+      <c r="T2" s="135"/>
+      <c r="U2" s="135"/>
+      <c r="V2" s="135"/>
+      <c r="W2" s="135"/>
+      <c r="X2" s="135"/>
+      <c r="Y2" s="135"/>
+      <c r="Z2" s="135"/>
+      <c r="AA2" s="135"/>
+      <c r="AB2" s="135"/>
+      <c r="AC2" s="135">
         <v>25</v>
       </c>
-      <c r="AD2" s="130"/>
-      <c r="AE2" s="130"/>
-      <c r="AF2" s="130"/>
-      <c r="AG2" s="130"/>
-      <c r="AH2" s="130"/>
-      <c r="AI2" s="130"/>
-      <c r="AJ2" s="130"/>
-      <c r="AK2" s="130"/>
-      <c r="AL2" s="130"/>
-      <c r="AM2" s="130"/>
-      <c r="AN2" s="130"/>
-      <c r="AO2" s="130">
+      <c r="AD2" s="135"/>
+      <c r="AE2" s="135"/>
+      <c r="AF2" s="135"/>
+      <c r="AG2" s="135"/>
+      <c r="AH2" s="135"/>
+      <c r="AI2" s="135"/>
+      <c r="AJ2" s="135"/>
+      <c r="AK2" s="135"/>
+      <c r="AL2" s="135"/>
+      <c r="AM2" s="135"/>
+      <c r="AN2" s="135"/>
+      <c r="AO2" s="135">
         <v>26</v>
       </c>
-      <c r="AP2" s="130"/>
-      <c r="AQ2" s="130"/>
-      <c r="AR2" s="130"/>
-      <c r="AS2" s="130"/>
-      <c r="AT2" s="130"/>
-      <c r="AU2" s="130"/>
-      <c r="AV2" s="130"/>
-      <c r="AW2" s="130"/>
-      <c r="AX2" s="130"/>
-      <c r="AY2" s="130"/>
-      <c r="AZ2" s="131"/>
-      <c r="BA2" s="130">
+      <c r="AP2" s="135"/>
+      <c r="AQ2" s="135"/>
+      <c r="AR2" s="135"/>
+      <c r="AS2" s="135"/>
+      <c r="AT2" s="135"/>
+      <c r="AU2" s="135"/>
+      <c r="AV2" s="135"/>
+      <c r="AW2" s="135"/>
+      <c r="AX2" s="135"/>
+      <c r="AY2" s="135"/>
+      <c r="AZ2" s="136"/>
+      <c r="BA2" s="135">
         <v>27</v>
       </c>
-      <c r="BB2" s="130"/>
-      <c r="BC2" s="130"/>
-      <c r="BD2" s="130"/>
-      <c r="BE2" s="130"/>
-      <c r="BF2" s="130"/>
-      <c r="BG2" s="130"/>
-      <c r="BH2" s="130"/>
-      <c r="BI2" s="130"/>
-      <c r="BJ2" s="130"/>
-      <c r="BK2" s="130"/>
-      <c r="BL2" s="131"/>
+      <c r="BB2" s="135"/>
+      <c r="BC2" s="135"/>
+      <c r="BD2" s="135"/>
+      <c r="BE2" s="135"/>
+      <c r="BF2" s="135"/>
+      <c r="BG2" s="135"/>
+      <c r="BH2" s="135"/>
+      <c r="BI2" s="135"/>
+      <c r="BJ2" s="135"/>
+      <c r="BK2" s="135"/>
+      <c r="BL2" s="136"/>
     </row>
     <row r="3" spans="1:64" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="127"/>
-      <c r="C3" s="129"/>
-      <c r="D3" s="129"/>
+      <c r="B3" s="132"/>
+      <c r="C3" s="134"/>
+      <c r="D3" s="134"/>
       <c r="E3" s="22">
         <v>1</v>
       </c>
@@ -5222,7 +5226,7 @@
         <v>86</v>
       </c>
       <c r="C18" s="59" t="s">
-        <v>106</v>
+        <v>259</v>
       </c>
       <c r="D18" s="33"/>
       <c r="E18" s="64"/>
@@ -5718,13 +5722,13 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="141" t="s">
+      <c r="A2" s="126" t="s">
         <v>241</v>
       </c>
       <c r="B2" t="s">
         <v>242</v>
       </c>
-      <c r="C2" s="142" t="s">
+      <c r="C2" s="127" t="s">
         <v>243</v>
       </c>
       <c r="D2" t="s">
@@ -5732,13 +5736,13 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="141" t="s">
+      <c r="A3" s="126" t="s">
         <v>245</v>
       </c>
       <c r="B3" t="s">
         <v>242</v>
       </c>
-      <c r="C3" s="143" t="s">
+      <c r="C3" s="128" t="s">
         <v>246</v>
       </c>
       <c r="D3" t="s">
@@ -5746,13 +5750,13 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="141" t="s">
+      <c r="A4" s="126" t="s">
         <v>247</v>
       </c>
       <c r="B4" t="s">
         <v>242</v>
       </c>
-      <c r="C4" s="143" t="s">
+      <c r="C4" s="128" t="s">
         <v>248</v>
       </c>
       <c r="D4" t="s">
@@ -5760,13 +5764,13 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="144" t="s">
+      <c r="A5" s="129" t="s">
         <v>249</v>
       </c>
       <c r="B5" t="s">
         <v>242</v>
       </c>
-      <c r="C5" s="143" t="s">
+      <c r="C5" s="128" t="s">
         <v>250</v>
       </c>
       <c r="D5" t="s">
@@ -5774,13 +5778,13 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="142" t="s">
+      <c r="A6" s="127" t="s">
         <v>251</v>
       </c>
       <c r="B6" t="s">
         <v>244</v>
       </c>
-      <c r="C6" s="145" t="s">
+      <c r="C6" s="130" t="s">
         <v>252</v>
       </c>
       <c r="D6" t="s">
@@ -5788,13 +5792,13 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="142" t="s">
+      <c r="A7" s="127" t="s">
         <v>253</v>
       </c>
       <c r="B7" t="s">
         <v>244</v>
       </c>
-      <c r="C7" s="145" t="s">
+      <c r="C7" s="130" t="s">
         <v>254</v>
       </c>
       <c r="D7" t="s">
@@ -5802,7 +5806,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C8" s="141" t="s">
+      <c r="C8" s="126" t="s">
         <v>255</v>
       </c>
       <c r="D8" t="s">
@@ -5810,7 +5814,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C9" s="141" t="s">
+      <c r="C9" s="126" t="s">
         <v>256</v>
       </c>
       <c r="D9" t="s">
@@ -5818,7 +5822,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C10" s="145" t="s">
+      <c r="C10" s="130" t="s">
         <v>257</v>
       </c>
       <c r="D10" t="s">
@@ -5858,39 +5862,39 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="135" t="s">
+      <c r="B2" s="140" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="139" t="s">
+      <c r="C2" s="144" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="139" t="s">
+      <c r="D2" s="144" t="s">
         <v>178</v>
       </c>
-      <c r="E2" s="137" t="s">
+      <c r="E2" s="142" t="s">
         <v>127</v>
       </c>
       <c r="F2" s="98" t="s">
         <v>113</v>
       </c>
-      <c r="G2" s="133" t="s">
+      <c r="G2" s="138" t="s">
         <v>114</v>
       </c>
-      <c r="H2" s="133"/>
-      <c r="I2" s="133"/>
-      <c r="J2" s="134"/>
-      <c r="K2" s="133" t="s">
+      <c r="H2" s="138"/>
+      <c r="I2" s="138"/>
+      <c r="J2" s="139"/>
+      <c r="K2" s="138" t="s">
         <v>183</v>
       </c>
-      <c r="L2" s="133"/>
-      <c r="M2" s="133"/>
-      <c r="N2" s="134"/>
+      <c r="L2" s="138"/>
+      <c r="M2" s="138"/>
+      <c r="N2" s="139"/>
     </row>
     <row r="3" spans="1:14" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="136"/>
-      <c r="C3" s="140"/>
-      <c r="D3" s="140"/>
-      <c r="E3" s="138"/>
+      <c r="B3" s="141"/>
+      <c r="C3" s="145"/>
+      <c r="D3" s="145"/>
+      <c r="E3" s="143"/>
       <c r="F3" s="99" t="s">
         <v>112</v>
       </c>
@@ -6633,30 +6637,30 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="135" t="s">
+      <c r="B2" s="140" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="139" t="s">
+      <c r="C2" s="144" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="139" t="s">
+      <c r="D2" s="144" t="s">
         <v>178</v>
       </c>
-      <c r="E2" s="137" t="s">
+      <c r="E2" s="142" t="s">
         <v>127</v>
       </c>
-      <c r="F2" s="133" t="s">
+      <c r="F2" s="138" t="s">
         <v>183</v>
       </c>
-      <c r="G2" s="133"/>
-      <c r="H2" s="133"/>
-      <c r="I2" s="134"/>
+      <c r="G2" s="138"/>
+      <c r="H2" s="138"/>
+      <c r="I2" s="139"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="136"/>
-      <c r="C3" s="140"/>
-      <c r="D3" s="140"/>
-      <c r="E3" s="138"/>
+      <c r="B3" s="141"/>
+      <c r="C3" s="145"/>
+      <c r="D3" s="145"/>
+      <c r="E3" s="143"/>
       <c r="F3" s="99" t="s">
         <v>115</v>
       </c>
@@ -7034,30 +7038,30 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="135" t="s">
+      <c r="B2" s="140" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="139" t="s">
+      <c r="C2" s="144" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="139" t="s">
+      <c r="D2" s="144" t="s">
         <v>178</v>
       </c>
-      <c r="E2" s="137" t="s">
+      <c r="E2" s="142" t="s">
         <v>127</v>
       </c>
-      <c r="F2" s="133" t="s">
+      <c r="F2" s="138" t="s">
         <v>228</v>
       </c>
-      <c r="G2" s="133"/>
-      <c r="H2" s="133"/>
-      <c r="I2" s="134"/>
+      <c r="G2" s="138"/>
+      <c r="H2" s="138"/>
+      <c r="I2" s="139"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="136"/>
-      <c r="C3" s="140"/>
-      <c r="D3" s="140"/>
-      <c r="E3" s="138"/>
+      <c r="B3" s="141"/>
+      <c r="C3" s="145"/>
+      <c r="D3" s="145"/>
+      <c r="E3" s="143"/>
       <c r="F3" s="99" t="s">
         <v>115</v>
       </c>

</xml_diff>

<commit_message>
25. 10. 20. Weekly Plan 일정 및 업무 현황 작성 완료
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="17685"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="17685" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="대일정" sheetId="1" r:id="rId1"/>
@@ -17,6 +17,7 @@
     <sheet name="2025.5" sheetId="2" r:id="rId3"/>
     <sheet name="2025.6" sheetId="3" r:id="rId4"/>
     <sheet name="2025.7" sheetId="4" r:id="rId5"/>
+    <sheet name="2025.10" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="285">
   <si>
     <t>■</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1529,6 +1530,212 @@
     <t>97191NU000(LHD)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>10월</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>5주차</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>4주차</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>오세영
+임제훈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>오세영
+임제훈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>오세영
+임제훈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>오세영
+임제훈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>오세영
+임제훈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- SWE.3 SDDS 후속 작업 (진행률 : 90%)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- 온도 정합성 테스트 (10/20)
+- 제어기 선행품질 검증 현황 작성
+- 제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 (10/23)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- LHD R로직 튜닝
+- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- ESIR 계획서 등록
+- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신
+- Core Temp 튜닝 결과 확인
+- 최신 승인도 확인
+- R로직 튜닝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[임제훈 사원]
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>최신 승인도 확인 (10/16)</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">[임제훈 사원]
+- </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>양산 중 (25/07/15)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RHD P1 (진행 중)
+RHD P2 (26/02/01)
+LHD Proto (진행 중)
+LHD MCAR (25/11/15)
+LHD P1 (26/02/15)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1 (진행 중)
+P2 (26/03/30)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1 (진행 중)
+LP2 (26/04/15)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Proto (진행 중)
+MCAR (확인 필요)
+P1 (26/02/15)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SU2i CARRY OVER
+Proto (25/10/15)
+P1 (06/05/15)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- AY 회의 진행 (25/10/20)
+- LHD ESIR
+- R로직 튜닝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- AY 회의 진행 (25/10/20)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>- 이슈 없음</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[임제훈 사원]
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SU2i 고품 접수 (25/10/14)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  : 원인 - SU2i 인도 생산 라인에서 EOL 95% Duty로 측정 중, Fail 발생.
+            Timerout Fault 발생으로 인해 고품 접수
+    분석 - HW 신지훈 전임, SW 임제훈 사원
+    결과 - SW 확인 결과, Timeout Fault 발생하지 않음, HALT State 발생
+            과전류 PIN Scope 측정 결과 과전류 발생
+            → 이후 진행 HW 신지훈 전임</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[임제훈 사원]
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AY 회의 진행 (25/10/13)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  : HVAC 4대 수령, 2대는 안받아도 된다고 하여 안건 종료
+    ESIR 내부 일정 9월 30일 → 10월 말 변경, 고객사 공식 일정 아직 없음</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -1537,7 +1744,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="mm&quot;월&quot;\ dd&quot;일&quot;"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1667,8 +1874,17 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1725,8 +1941,14 @@
         <fgColor theme="8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="73">
+  <borders count="78">
     <border>
       <left/>
       <right/>
@@ -2734,6 +2956,69 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="hair">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="hair">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom style="hair">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -2755,7 +3040,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="146">
+  <cellXfs count="158">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3193,6 +3478,42 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -7417,4 +7738,447 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J22"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.375" style="83" customWidth="1"/>
+    <col min="2" max="2" width="9" style="83"/>
+    <col min="3" max="4" width="14.75" style="83" customWidth="1"/>
+    <col min="5" max="5" width="43" style="83" customWidth="1"/>
+    <col min="6" max="6" width="61.875" style="83" customWidth="1"/>
+    <col min="7" max="10" width="62.125" style="83" customWidth="1"/>
+    <col min="11" max="16384" width="9" style="83"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="110" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="111" t="s">
+        <v>150</v>
+      </c>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="109"/>
+    </row>
+    <row r="2" spans="1:10" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="140" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="144" t="s">
+        <v>177</v>
+      </c>
+      <c r="D2" s="144" t="s">
+        <v>178</v>
+      </c>
+      <c r="E2" s="142" t="s">
+        <v>127</v>
+      </c>
+      <c r="F2" s="138" t="s">
+        <v>260</v>
+      </c>
+      <c r="G2" s="138"/>
+      <c r="H2" s="138"/>
+      <c r="I2" s="146"/>
+      <c r="J2" s="139"/>
+    </row>
+    <row r="3" spans="1:10" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="141"/>
+      <c r="C3" s="145"/>
+      <c r="D3" s="145"/>
+      <c r="E3" s="143"/>
+      <c r="F3" s="99" t="s">
+        <v>115</v>
+      </c>
+      <c r="G3" s="99" t="s">
+        <v>116</v>
+      </c>
+      <c r="H3" s="99" t="s">
+        <v>117</v>
+      </c>
+      <c r="I3" s="99" t="s">
+        <v>262</v>
+      </c>
+      <c r="J3" s="100" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="84" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="118" t="s">
+        <v>176</v>
+      </c>
+      <c r="D4" s="118" t="s">
+        <v>179</v>
+      </c>
+      <c r="E4" s="92" t="s">
+        <v>153</v>
+      </c>
+      <c r="F4" s="116"/>
+      <c r="G4" s="107"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="147"/>
+      <c r="J4" s="94"/>
+    </row>
+    <row r="5" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="85" t="s">
+        <v>124</v>
+      </c>
+      <c r="C5" s="119" t="s">
+        <v>176</v>
+      </c>
+      <c r="D5" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E5" s="93" t="s">
+        <v>154</v>
+      </c>
+      <c r="F5" s="116"/>
+      <c r="G5" s="107"/>
+      <c r="H5" s="91"/>
+      <c r="I5" s="148"/>
+      <c r="J5" s="95"/>
+    </row>
+    <row r="6" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="85" t="s">
+        <v>125</v>
+      </c>
+      <c r="C6" s="119" t="s">
+        <v>176</v>
+      </c>
+      <c r="D6" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E6" s="93" t="s">
+        <v>155</v>
+      </c>
+      <c r="F6" s="116"/>
+      <c r="G6" s="107"/>
+      <c r="H6" s="91"/>
+      <c r="I6" s="148"/>
+      <c r="J6" s="95"/>
+    </row>
+    <row r="7" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="85" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" s="119" t="s">
+        <v>176</v>
+      </c>
+      <c r="D7" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E7" s="93" t="s">
+        <v>156</v>
+      </c>
+      <c r="F7" s="116"/>
+      <c r="G7" s="107"/>
+      <c r="H7" s="91"/>
+      <c r="I7" s="148"/>
+      <c r="J7" s="95"/>
+    </row>
+    <row r="8" spans="1:10" ht="108" x14ac:dyDescent="0.3">
+      <c r="B8" s="153" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="119" t="s">
+        <v>263</v>
+      </c>
+      <c r="D8" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E8" s="93" t="s">
+        <v>157</v>
+      </c>
+      <c r="F8" s="116"/>
+      <c r="G8" s="107"/>
+      <c r="H8" s="156" t="s">
+        <v>283</v>
+      </c>
+      <c r="I8" s="148"/>
+      <c r="J8" s="95"/>
+    </row>
+    <row r="9" spans="1:10" ht="27" x14ac:dyDescent="0.3">
+      <c r="B9" s="153" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="119" t="s">
+        <v>264</v>
+      </c>
+      <c r="D9" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E9" s="102" t="s">
+        <v>274</v>
+      </c>
+      <c r="F9" s="116"/>
+      <c r="G9" s="107"/>
+      <c r="H9" s="106" t="s">
+        <v>282</v>
+      </c>
+      <c r="I9" s="148"/>
+      <c r="J9" s="95"/>
+    </row>
+    <row r="10" spans="1:10" ht="67.5" x14ac:dyDescent="0.3">
+      <c r="B10" s="153" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="119" t="s">
+        <v>265</v>
+      </c>
+      <c r="D10" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E10" s="102" t="s">
+        <v>275</v>
+      </c>
+      <c r="F10" s="116"/>
+      <c r="G10" s="107"/>
+      <c r="H10" s="156" t="s">
+        <v>284</v>
+      </c>
+      <c r="I10" s="150" t="s">
+        <v>280</v>
+      </c>
+      <c r="J10" s="157" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="54" x14ac:dyDescent="0.3">
+      <c r="B11" s="155" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="119" t="s">
+        <v>263</v>
+      </c>
+      <c r="D11" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E11" s="102" t="s">
+        <v>276</v>
+      </c>
+      <c r="F11" s="116"/>
+      <c r="G11" s="107"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="150" t="s">
+        <v>269</v>
+      </c>
+      <c r="J11" s="95"/>
+    </row>
+    <row r="12" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="153" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="119" t="s">
+        <v>180</v>
+      </c>
+      <c r="D12" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E12" s="102" t="s">
+        <v>277</v>
+      </c>
+      <c r="F12" s="116"/>
+      <c r="G12" s="107"/>
+      <c r="H12" s="91"/>
+      <c r="I12" s="150" t="s">
+        <v>270</v>
+      </c>
+      <c r="J12" s="95"/>
+    </row>
+    <row r="13" spans="1:10" ht="347.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="86" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" s="119" t="s">
+        <v>176</v>
+      </c>
+      <c r="D13" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E13" s="102" t="s">
+        <v>162</v>
+      </c>
+      <c r="F13" s="116"/>
+      <c r="G13" s="107"/>
+      <c r="H13" s="91"/>
+      <c r="I13" s="148"/>
+      <c r="J13" s="95"/>
+    </row>
+    <row r="14" spans="1:10" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="B14" s="87" t="s">
+        <v>182</v>
+      </c>
+      <c r="C14" s="119" t="s">
+        <v>180</v>
+      </c>
+      <c r="D14" s="119" t="s">
+        <v>181</v>
+      </c>
+      <c r="E14" s="102"/>
+      <c r="F14" s="125"/>
+      <c r="G14" s="125"/>
+      <c r="H14" s="125"/>
+      <c r="I14" s="125" t="s">
+        <v>268</v>
+      </c>
+      <c r="J14" s="95"/>
+    </row>
+    <row r="15" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="87" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="119" t="s">
+        <v>176</v>
+      </c>
+      <c r="D15" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E15" s="102" t="s">
+        <v>163</v>
+      </c>
+      <c r="F15" s="116"/>
+      <c r="G15" s="107"/>
+      <c r="H15" s="91"/>
+      <c r="I15" s="148"/>
+      <c r="J15" s="95"/>
+    </row>
+    <row r="16" spans="1:10" ht="81" x14ac:dyDescent="0.3">
+      <c r="B16" s="153" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" s="119" t="s">
+        <v>266</v>
+      </c>
+      <c r="D16" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E16" s="102" t="s">
+        <v>278</v>
+      </c>
+      <c r="F16" s="116"/>
+      <c r="G16" s="107"/>
+      <c r="H16" s="91"/>
+      <c r="I16" s="150" t="s">
+        <v>271</v>
+      </c>
+      <c r="J16" s="95"/>
+    </row>
+    <row r="17" spans="2:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="154" t="s">
+        <v>142</v>
+      </c>
+      <c r="C17" s="119" t="s">
+        <v>180</v>
+      </c>
+      <c r="D17" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E17" s="93" t="s">
+        <v>106</v>
+      </c>
+      <c r="F17" s="116"/>
+      <c r="G17" s="91"/>
+      <c r="H17" s="91"/>
+      <c r="I17" s="148"/>
+      <c r="J17" s="95"/>
+    </row>
+    <row r="18" spans="2:10" ht="27" x14ac:dyDescent="0.3">
+      <c r="B18" s="88" t="s">
+        <v>107</v>
+      </c>
+      <c r="C18" s="119" t="s">
+        <v>176</v>
+      </c>
+      <c r="D18" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E18" s="102" t="s">
+        <v>165</v>
+      </c>
+      <c r="F18" s="116"/>
+      <c r="G18" s="107"/>
+      <c r="H18" s="91"/>
+      <c r="I18" s="148"/>
+      <c r="J18" s="95"/>
+    </row>
+    <row r="19" spans="2:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="87" t="s">
+        <v>110</v>
+      </c>
+      <c r="C19" s="119" t="s">
+        <v>176</v>
+      </c>
+      <c r="D19" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E19" s="93" t="s">
+        <v>140</v>
+      </c>
+      <c r="F19" s="116"/>
+      <c r="G19" s="106"/>
+      <c r="H19" s="91"/>
+      <c r="I19" s="148"/>
+      <c r="J19" s="95"/>
+    </row>
+    <row r="20" spans="2:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="152" t="s">
+        <v>168</v>
+      </c>
+      <c r="C20" s="119" t="s">
+        <v>267</v>
+      </c>
+      <c r="D20" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E20" s="115" t="s">
+        <v>279</v>
+      </c>
+      <c r="F20" s="116"/>
+      <c r="G20" s="112"/>
+      <c r="H20" s="151" t="s">
+        <v>272</v>
+      </c>
+      <c r="I20" s="151" t="s">
+        <v>273</v>
+      </c>
+      <c r="J20" s="114"/>
+    </row>
+    <row r="21" spans="2:10" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="89" t="s">
+        <v>109</v>
+      </c>
+      <c r="C21" s="120" t="s">
+        <v>176</v>
+      </c>
+      <c r="D21" s="120" t="s">
+        <v>179</v>
+      </c>
+      <c r="E21" s="105" t="s">
+        <v>141</v>
+      </c>
+      <c r="F21" s="117"/>
+      <c r="G21" s="108"/>
+      <c r="H21" s="96"/>
+      <c r="I21" s="149"/>
+      <c r="J21" s="97"/>
+    </row>
+    <row r="22" spans="2:10" ht="14.25" thickTop="1" x14ac:dyDescent="0.3"/>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:J2"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly Plan SVm 업무 현황 항목 추가
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -1570,13 +1570,6 @@
   <si>
     <t>[임제훈 사원]
 - SWE.3 SDDS 후속 작업 (진행률 : 90%)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- 온도 정합성 테스트 (10/20)
-- 제어기 선행품질 검증 현황 작성
-- 제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 (10/23)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1734,6 +1727,14 @@
   : HVAC 4대 수령, 2대는 안받아도 된다고 하여 안건 종료
     ESIR 내부 일정 9월 30일 → 10월 말 변경, 고객사 공식 일정 아직 없음</t>
     </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- 온도 정합성 테스트 (10/20)
+- 제어기 선행품질 검증 현황 작성
+- 제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 (10/23)
+- 설계 변경 진행</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3434,6 +3435,39 @@
     <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="3">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3481,39 +3515,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -4131,90 +4132,90 @@
       <c r="D1" s="21"/>
     </row>
     <row r="2" spans="1:64" ht="31.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="131" t="s">
+      <c r="B2" s="142" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="133" t="s">
+      <c r="C2" s="144" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="133" t="s">
+      <c r="D2" s="144" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="137">
+      <c r="E2" s="148">
         <v>23</v>
       </c>
-      <c r="F2" s="135"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="135"/>
-      <c r="I2" s="135"/>
-      <c r="J2" s="135"/>
-      <c r="K2" s="135"/>
-      <c r="L2" s="135"/>
-      <c r="M2" s="135"/>
-      <c r="N2" s="135"/>
-      <c r="O2" s="135"/>
-      <c r="P2" s="135"/>
-      <c r="Q2" s="135">
+      <c r="F2" s="146"/>
+      <c r="G2" s="146"/>
+      <c r="H2" s="146"/>
+      <c r="I2" s="146"/>
+      <c r="J2" s="146"/>
+      <c r="K2" s="146"/>
+      <c r="L2" s="146"/>
+      <c r="M2" s="146"/>
+      <c r="N2" s="146"/>
+      <c r="O2" s="146"/>
+      <c r="P2" s="146"/>
+      <c r="Q2" s="146">
         <v>24</v>
       </c>
-      <c r="R2" s="135"/>
-      <c r="S2" s="135"/>
-      <c r="T2" s="135"/>
-      <c r="U2" s="135"/>
-      <c r="V2" s="135"/>
-      <c r="W2" s="135"/>
-      <c r="X2" s="135"/>
-      <c r="Y2" s="135"/>
-      <c r="Z2" s="135"/>
-      <c r="AA2" s="135"/>
-      <c r="AB2" s="135"/>
-      <c r="AC2" s="135">
+      <c r="R2" s="146"/>
+      <c r="S2" s="146"/>
+      <c r="T2" s="146"/>
+      <c r="U2" s="146"/>
+      <c r="V2" s="146"/>
+      <c r="W2" s="146"/>
+      <c r="X2" s="146"/>
+      <c r="Y2" s="146"/>
+      <c r="Z2" s="146"/>
+      <c r="AA2" s="146"/>
+      <c r="AB2" s="146"/>
+      <c r="AC2" s="146">
         <v>25</v>
       </c>
-      <c r="AD2" s="135"/>
-      <c r="AE2" s="135"/>
-      <c r="AF2" s="135"/>
-      <c r="AG2" s="135"/>
-      <c r="AH2" s="135"/>
-      <c r="AI2" s="135"/>
-      <c r="AJ2" s="135"/>
-      <c r="AK2" s="135"/>
-      <c r="AL2" s="135"/>
-      <c r="AM2" s="135"/>
-      <c r="AN2" s="135"/>
-      <c r="AO2" s="135">
+      <c r="AD2" s="146"/>
+      <c r="AE2" s="146"/>
+      <c r="AF2" s="146"/>
+      <c r="AG2" s="146"/>
+      <c r="AH2" s="146"/>
+      <c r="AI2" s="146"/>
+      <c r="AJ2" s="146"/>
+      <c r="AK2" s="146"/>
+      <c r="AL2" s="146"/>
+      <c r="AM2" s="146"/>
+      <c r="AN2" s="146"/>
+      <c r="AO2" s="146">
         <v>26</v>
       </c>
-      <c r="AP2" s="135"/>
-      <c r="AQ2" s="135"/>
-      <c r="AR2" s="135"/>
-      <c r="AS2" s="135"/>
-      <c r="AT2" s="135"/>
-      <c r="AU2" s="135"/>
-      <c r="AV2" s="135"/>
-      <c r="AW2" s="135"/>
-      <c r="AX2" s="135"/>
-      <c r="AY2" s="135"/>
-      <c r="AZ2" s="136"/>
-      <c r="BA2" s="135">
+      <c r="AP2" s="146"/>
+      <c r="AQ2" s="146"/>
+      <c r="AR2" s="146"/>
+      <c r="AS2" s="146"/>
+      <c r="AT2" s="146"/>
+      <c r="AU2" s="146"/>
+      <c r="AV2" s="146"/>
+      <c r="AW2" s="146"/>
+      <c r="AX2" s="146"/>
+      <c r="AY2" s="146"/>
+      <c r="AZ2" s="147"/>
+      <c r="BA2" s="146">
         <v>27</v>
       </c>
-      <c r="BB2" s="135"/>
-      <c r="BC2" s="135"/>
-      <c r="BD2" s="135"/>
-      <c r="BE2" s="135"/>
-      <c r="BF2" s="135"/>
-      <c r="BG2" s="135"/>
-      <c r="BH2" s="135"/>
-      <c r="BI2" s="135"/>
-      <c r="BJ2" s="135"/>
-      <c r="BK2" s="135"/>
-      <c r="BL2" s="136"/>
+      <c r="BB2" s="146"/>
+      <c r="BC2" s="146"/>
+      <c r="BD2" s="146"/>
+      <c r="BE2" s="146"/>
+      <c r="BF2" s="146"/>
+      <c r="BG2" s="146"/>
+      <c r="BH2" s="146"/>
+      <c r="BI2" s="146"/>
+      <c r="BJ2" s="146"/>
+      <c r="BK2" s="146"/>
+      <c r="BL2" s="147"/>
     </row>
     <row r="3" spans="1:64" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="132"/>
-      <c r="C3" s="134"/>
-      <c r="D3" s="134"/>
+      <c r="B3" s="143"/>
+      <c r="C3" s="145"/>
+      <c r="D3" s="145"/>
       <c r="E3" s="22">
         <v>1</v>
       </c>
@@ -6183,39 +6184,39 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="140" t="s">
+      <c r="B2" s="151" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="144" t="s">
+      <c r="C2" s="155" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="144" t="s">
+      <c r="D2" s="155" t="s">
         <v>178</v>
       </c>
-      <c r="E2" s="142" t="s">
+      <c r="E2" s="153" t="s">
         <v>127</v>
       </c>
       <c r="F2" s="98" t="s">
         <v>113</v>
       </c>
-      <c r="G2" s="138" t="s">
+      <c r="G2" s="149" t="s">
         <v>114</v>
       </c>
-      <c r="H2" s="138"/>
-      <c r="I2" s="138"/>
-      <c r="J2" s="139"/>
-      <c r="K2" s="138" t="s">
+      <c r="H2" s="149"/>
+      <c r="I2" s="149"/>
+      <c r="J2" s="150"/>
+      <c r="K2" s="149" t="s">
         <v>183</v>
       </c>
-      <c r="L2" s="138"/>
-      <c r="M2" s="138"/>
-      <c r="N2" s="139"/>
+      <c r="L2" s="149"/>
+      <c r="M2" s="149"/>
+      <c r="N2" s="150"/>
     </row>
     <row r="3" spans="1:14" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="141"/>
-      <c r="C3" s="145"/>
-      <c r="D3" s="145"/>
-      <c r="E3" s="143"/>
+      <c r="B3" s="152"/>
+      <c r="C3" s="156"/>
+      <c r="D3" s="156"/>
+      <c r="E3" s="154"/>
       <c r="F3" s="99" t="s">
         <v>112</v>
       </c>
@@ -6958,30 +6959,30 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="140" t="s">
+      <c r="B2" s="151" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="144" t="s">
+      <c r="C2" s="155" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="144" t="s">
+      <c r="D2" s="155" t="s">
         <v>178</v>
       </c>
-      <c r="E2" s="142" t="s">
+      <c r="E2" s="153" t="s">
         <v>127</v>
       </c>
-      <c r="F2" s="138" t="s">
+      <c r="F2" s="149" t="s">
         <v>183</v>
       </c>
-      <c r="G2" s="138"/>
-      <c r="H2" s="138"/>
-      <c r="I2" s="139"/>
+      <c r="G2" s="149"/>
+      <c r="H2" s="149"/>
+      <c r="I2" s="150"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="141"/>
-      <c r="C3" s="145"/>
-      <c r="D3" s="145"/>
-      <c r="E3" s="143"/>
+      <c r="B3" s="152"/>
+      <c r="C3" s="156"/>
+      <c r="D3" s="156"/>
+      <c r="E3" s="154"/>
       <c r="F3" s="99" t="s">
         <v>115</v>
       </c>
@@ -7359,30 +7360,30 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="140" t="s">
+      <c r="B2" s="151" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="144" t="s">
+      <c r="C2" s="155" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="144" t="s">
+      <c r="D2" s="155" t="s">
         <v>178</v>
       </c>
-      <c r="E2" s="142" t="s">
+      <c r="E2" s="153" t="s">
         <v>127</v>
       </c>
-      <c r="F2" s="138" t="s">
+      <c r="F2" s="149" t="s">
         <v>228</v>
       </c>
-      <c r="G2" s="138"/>
-      <c r="H2" s="138"/>
-      <c r="I2" s="139"/>
+      <c r="G2" s="149"/>
+      <c r="H2" s="149"/>
+      <c r="I2" s="150"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="141"/>
-      <c r="C3" s="145"/>
-      <c r="D3" s="145"/>
-      <c r="E3" s="143"/>
+      <c r="B3" s="152"/>
+      <c r="C3" s="156"/>
+      <c r="D3" s="156"/>
+      <c r="E3" s="154"/>
       <c r="F3" s="99" t="s">
         <v>115</v>
       </c>
@@ -7766,31 +7767,31 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="140" t="s">
+      <c r="B2" s="151" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="144" t="s">
+      <c r="C2" s="155" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="144" t="s">
+      <c r="D2" s="155" t="s">
         <v>178</v>
       </c>
-      <c r="E2" s="142" t="s">
+      <c r="E2" s="153" t="s">
         <v>127</v>
       </c>
-      <c r="F2" s="138" t="s">
+      <c r="F2" s="149" t="s">
         <v>260</v>
       </c>
-      <c r="G2" s="138"/>
-      <c r="H2" s="138"/>
-      <c r="I2" s="146"/>
-      <c r="J2" s="139"/>
+      <c r="G2" s="149"/>
+      <c r="H2" s="149"/>
+      <c r="I2" s="157"/>
+      <c r="J2" s="150"/>
     </row>
     <row r="3" spans="1:10" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="141"/>
-      <c r="C3" s="145"/>
-      <c r="D3" s="145"/>
-      <c r="E3" s="143"/>
+      <c r="B3" s="152"/>
+      <c r="C3" s="156"/>
+      <c r="D3" s="156"/>
+      <c r="E3" s="154"/>
       <c r="F3" s="99" t="s">
         <v>115</v>
       </c>
@@ -7823,7 +7824,7 @@
       <c r="F4" s="116"/>
       <c r="G4" s="107"/>
       <c r="H4" s="90"/>
-      <c r="I4" s="147"/>
+      <c r="I4" s="131"/>
       <c r="J4" s="94"/>
     </row>
     <row r="5" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -7842,7 +7843,7 @@
       <c r="F5" s="116"/>
       <c r="G5" s="107"/>
       <c r="H5" s="91"/>
-      <c r="I5" s="148"/>
+      <c r="I5" s="132"/>
       <c r="J5" s="95"/>
     </row>
     <row r="6" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -7861,7 +7862,7 @@
       <c r="F6" s="116"/>
       <c r="G6" s="107"/>
       <c r="H6" s="91"/>
-      <c r="I6" s="148"/>
+      <c r="I6" s="132"/>
       <c r="J6" s="95"/>
     </row>
     <row r="7" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -7880,11 +7881,11 @@
       <c r="F7" s="116"/>
       <c r="G7" s="107"/>
       <c r="H7" s="91"/>
-      <c r="I7" s="148"/>
+      <c r="I7" s="132"/>
       <c r="J7" s="95"/>
     </row>
     <row r="8" spans="1:10" ht="108" x14ac:dyDescent="0.3">
-      <c r="B8" s="153" t="s">
+      <c r="B8" s="137" t="s">
         <v>3</v>
       </c>
       <c r="C8" s="119" t="s">
@@ -7898,14 +7899,14 @@
       </c>
       <c r="F8" s="116"/>
       <c r="G8" s="107"/>
-      <c r="H8" s="156" t="s">
-        <v>283</v>
-      </c>
-      <c r="I8" s="148"/>
+      <c r="H8" s="140" t="s">
+        <v>282</v>
+      </c>
+      <c r="I8" s="132"/>
       <c r="J8" s="95"/>
     </row>
     <row r="9" spans="1:10" ht="27" x14ac:dyDescent="0.3">
-      <c r="B9" s="153" t="s">
+      <c r="B9" s="137" t="s">
         <v>46</v>
       </c>
       <c r="C9" s="119" t="s">
@@ -7915,18 +7916,18 @@
         <v>179</v>
       </c>
       <c r="E9" s="102" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F9" s="116"/>
       <c r="G9" s="107"/>
       <c r="H9" s="106" t="s">
-        <v>282</v>
-      </c>
-      <c r="I9" s="148"/>
+        <v>281</v>
+      </c>
+      <c r="I9" s="132"/>
       <c r="J9" s="95"/>
     </row>
     <row r="10" spans="1:10" ht="67.5" x14ac:dyDescent="0.3">
-      <c r="B10" s="153" t="s">
+      <c r="B10" s="137" t="s">
         <v>56</v>
       </c>
       <c r="C10" s="119" t="s">
@@ -7936,22 +7937,22 @@
         <v>179</v>
       </c>
       <c r="E10" s="102" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F10" s="116"/>
       <c r="G10" s="107"/>
-      <c r="H10" s="156" t="s">
-        <v>284</v>
-      </c>
-      <c r="I10" s="150" t="s">
+      <c r="H10" s="140" t="s">
+        <v>283</v>
+      </c>
+      <c r="I10" s="134" t="s">
+        <v>279</v>
+      </c>
+      <c r="J10" s="141" t="s">
         <v>280</v>
       </c>
-      <c r="J10" s="157" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="54" x14ac:dyDescent="0.3">
-      <c r="B11" s="155" t="s">
+    </row>
+    <row r="11" spans="1:10" ht="67.5" x14ac:dyDescent="0.3">
+      <c r="B11" s="139" t="s">
         <v>63</v>
       </c>
       <c r="C11" s="119" t="s">
@@ -7961,18 +7962,18 @@
         <v>179</v>
       </c>
       <c r="E11" s="102" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F11" s="116"/>
       <c r="G11" s="107"/>
       <c r="H11" s="91"/>
-      <c r="I11" s="150" t="s">
-        <v>269</v>
+      <c r="I11" s="134" t="s">
+        <v>284</v>
       </c>
       <c r="J11" s="95"/>
     </row>
     <row r="12" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="153" t="s">
+      <c r="B12" s="137" t="s">
         <v>74</v>
       </c>
       <c r="C12" s="119" t="s">
@@ -7982,13 +7983,13 @@
         <v>179</v>
       </c>
       <c r="E12" s="102" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F12" s="116"/>
       <c r="G12" s="107"/>
       <c r="H12" s="91"/>
-      <c r="I12" s="150" t="s">
-        <v>270</v>
+      <c r="I12" s="134" t="s">
+        <v>269</v>
       </c>
       <c r="J12" s="95"/>
     </row>
@@ -8008,7 +8009,7 @@
       <c r="F13" s="116"/>
       <c r="G13" s="107"/>
       <c r="H13" s="91"/>
-      <c r="I13" s="148"/>
+      <c r="I13" s="132"/>
       <c r="J13" s="95"/>
     </row>
     <row r="14" spans="1:10" ht="40.5" x14ac:dyDescent="0.3">
@@ -8046,11 +8047,11 @@
       <c r="F15" s="116"/>
       <c r="G15" s="107"/>
       <c r="H15" s="91"/>
-      <c r="I15" s="148"/>
+      <c r="I15" s="132"/>
       <c r="J15" s="95"/>
     </row>
     <row r="16" spans="1:10" ht="81" x14ac:dyDescent="0.3">
-      <c r="B16" s="153" t="s">
+      <c r="B16" s="137" t="s">
         <v>86</v>
       </c>
       <c r="C16" s="119" t="s">
@@ -8060,18 +8061,18 @@
         <v>179</v>
       </c>
       <c r="E16" s="102" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F16" s="116"/>
       <c r="G16" s="107"/>
       <c r="H16" s="91"/>
-      <c r="I16" s="150" t="s">
-        <v>271</v>
+      <c r="I16" s="134" t="s">
+        <v>270</v>
       </c>
       <c r="J16" s="95"/>
     </row>
     <row r="17" spans="2:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="154" t="s">
+      <c r="B17" s="138" t="s">
         <v>142</v>
       </c>
       <c r="C17" s="119" t="s">
@@ -8086,7 +8087,7 @@
       <c r="F17" s="116"/>
       <c r="G17" s="91"/>
       <c r="H17" s="91"/>
-      <c r="I17" s="148"/>
+      <c r="I17" s="132"/>
       <c r="J17" s="95"/>
     </row>
     <row r="18" spans="2:10" ht="27" x14ac:dyDescent="0.3">
@@ -8105,7 +8106,7 @@
       <c r="F18" s="116"/>
       <c r="G18" s="107"/>
       <c r="H18" s="91"/>
-      <c r="I18" s="148"/>
+      <c r="I18" s="132"/>
       <c r="J18" s="95"/>
     </row>
     <row r="19" spans="2:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -8124,11 +8125,11 @@
       <c r="F19" s="116"/>
       <c r="G19" s="106"/>
       <c r="H19" s="91"/>
-      <c r="I19" s="148"/>
+      <c r="I19" s="132"/>
       <c r="J19" s="95"/>
     </row>
     <row r="20" spans="2:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="152" t="s">
+      <c r="B20" s="136" t="s">
         <v>168</v>
       </c>
       <c r="C20" s="119" t="s">
@@ -8138,15 +8139,15 @@
         <v>179</v>
       </c>
       <c r="E20" s="115" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F20" s="116"/>
       <c r="G20" s="112"/>
-      <c r="H20" s="151" t="s">
+      <c r="H20" s="135" t="s">
+        <v>271</v>
+      </c>
+      <c r="I20" s="135" t="s">
         <v>272</v>
-      </c>
-      <c r="I20" s="151" t="s">
-        <v>273</v>
       </c>
       <c r="J20" s="114"/>
     </row>
@@ -8166,7 +8167,7 @@
       <c r="F21" s="117"/>
       <c r="G21" s="108"/>
       <c r="H21" s="96"/>
-      <c r="I21" s="149"/>
+      <c r="I21" s="133"/>
       <c r="J21" s="97"/>
     </row>
     <row r="22" spans="2:10" ht="14.25" thickTop="1" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Heater Weekly Plan 10월 양식 작성 완료
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -18,6 +18,7 @@
     <sheet name="2025.6" sheetId="3" r:id="rId4"/>
     <sheet name="2025.7" sheetId="4" r:id="rId5"/>
     <sheet name="2025.10" sheetId="6" r:id="rId6"/>
+    <sheet name="2025.11" sheetId="8" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="302">
   <si>
     <t>■</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1535,59 +1536,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>5주차</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>4주차</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>오세영
-임제훈</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>오세영
-임제훈</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>오세영
-임제훈</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>오세영
-임제훈</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>오세영
-임제훈</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- SWE.3 SDDS 후속 작업 (진행률 : 90%)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- LHD R로직 튜닝
-- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- ESIR 계획서 등록
-- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신
-- Core Temp 튜닝 결과 확인
-- 최신 승인도 확인
-- R로직 튜닝</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">[임제훈 사원]
 - </t>
@@ -1607,11 +1555,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">[임제훈 사원]
-- </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>양산 중 (25/07/15)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1637,18 +1580,6 @@
     <t>Proto (진행 중)
 MCAR (확인 필요)
 P1 (26/02/15)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- AY 회의 진행 (25/10/20)
-- LHD ESIR
-- R로직 튜닝</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- AY 회의 진행 (25/10/20)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1724,6 +1655,38 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>SU2i CARRY OVER
+Proto (25/10/15)
+P1 (26/05/15)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2주차 (10/10 ~ 10/15)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3주차 (10/16 ~ 10/22)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>4주차 (10/23 ~ 10/29)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- AY 회의 진행 (25/10/20)
+- LHD ESIR
+- R로직 튜닝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- AY 회의 진행 (25/10/20)
+- LHD ESIR
+- R로직 튜닝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>[임제훈 사원]
 - 온도 정합성 테스트 (10/20)
 - 제어기 선행품질 검증 현황 작성
@@ -1732,9 +1695,130 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>SU2i CARRY OVER
-Proto (25/10/15)
-P1 (26/05/15)</t>
+    <t>[임제훈 사원]
+- 온도 정합성 테스트 (10/20)
+- 제어기 선행품질 검증 현황 작성
+- 제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 (10/23)
+- 설계 변경 진행</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- LHD R로직 튜닝
+- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- LHD R로직 튜닝
+- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- SWE.3 SDDS 후속 작업 (진행률 : 90%)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- SWE.3 SDDS 후속 작업 (진행률 : 90%)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- ESIR 계획서 등록
+- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신
+- Core Temp 튜닝 결과 확인
+- 최신 승인도 확인
+- R로직 튜닝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">[임제훈 사원]
+- </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>오세영
+조현진
+임제훈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>조현진</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>조현진</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>임제훈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>임제훈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>임제훈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>임제훈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>임제훈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>QV</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>11월</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1주차 (10/30 ~ 11/05)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1주차 (10/02)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2주차 (11/06 ~ 11/12)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3주차 (11/13 ~ 11/19)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>4주차 (11/20 ~ 11/26)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- LHD ESIR
+- R로직 튜닝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- ESIR 계획서 등록 (~10/21)
+- Core Temp 튜닝 결과 확인 (~10/21)
+- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/24)
+- R로직 튜닝 (~10/24)
+- 최신 승인도 확인</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>출도 (26/02/01)
+Proto (26/04/06)
+정확한 일정인지 확인 필요</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1885,7 +1969,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1948,8 +2032,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="78">
+  <borders count="80">
     <border>
       <left/>
       <right/>
@@ -2962,45 +3058,6 @@
         <color auto="1"/>
       </left>
       <right/>
-      <top style="thick">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="hair">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
       <top style="hair">
         <color auto="1"/>
       </top>
@@ -3008,14 +3065,81 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="thick">
         <color auto="1"/>
       </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="hair">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="hair">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right/>
-      <top style="hair">
-        <color auto="1"/>
-      </top>
-      <bottom style="thick">
+      <top/>
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -3041,7 +3165,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="158">
+  <cellXfs count="172">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3435,19 +3559,7 @@
     <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="3">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3456,9 +3568,6 @@
     <xf numFmtId="0" fontId="8" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3513,8 +3622,65 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="53" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="53" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="54" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="54" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="79" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="74" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -4132,90 +4298,90 @@
       <c r="D1" s="21"/>
     </row>
     <row r="2" spans="1:64" ht="31.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="142" t="s">
+      <c r="B2" s="137" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="144" t="s">
+      <c r="C2" s="139" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="144" t="s">
+      <c r="D2" s="139" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="148">
+      <c r="E2" s="143">
         <v>23</v>
       </c>
-      <c r="F2" s="146"/>
-      <c r="G2" s="146"/>
-      <c r="H2" s="146"/>
-      <c r="I2" s="146"/>
-      <c r="J2" s="146"/>
-      <c r="K2" s="146"/>
-      <c r="L2" s="146"/>
-      <c r="M2" s="146"/>
-      <c r="N2" s="146"/>
-      <c r="O2" s="146"/>
-      <c r="P2" s="146"/>
-      <c r="Q2" s="146">
+      <c r="F2" s="141"/>
+      <c r="G2" s="141"/>
+      <c r="H2" s="141"/>
+      <c r="I2" s="141"/>
+      <c r="J2" s="141"/>
+      <c r="K2" s="141"/>
+      <c r="L2" s="141"/>
+      <c r="M2" s="141"/>
+      <c r="N2" s="141"/>
+      <c r="O2" s="141"/>
+      <c r="P2" s="141"/>
+      <c r="Q2" s="141">
         <v>24</v>
       </c>
-      <c r="R2" s="146"/>
-      <c r="S2" s="146"/>
-      <c r="T2" s="146"/>
-      <c r="U2" s="146"/>
-      <c r="V2" s="146"/>
-      <c r="W2" s="146"/>
-      <c r="X2" s="146"/>
-      <c r="Y2" s="146"/>
-      <c r="Z2" s="146"/>
-      <c r="AA2" s="146"/>
-      <c r="AB2" s="146"/>
-      <c r="AC2" s="146">
+      <c r="R2" s="141"/>
+      <c r="S2" s="141"/>
+      <c r="T2" s="141"/>
+      <c r="U2" s="141"/>
+      <c r="V2" s="141"/>
+      <c r="W2" s="141"/>
+      <c r="X2" s="141"/>
+      <c r="Y2" s="141"/>
+      <c r="Z2" s="141"/>
+      <c r="AA2" s="141"/>
+      <c r="AB2" s="141"/>
+      <c r="AC2" s="141">
         <v>25</v>
       </c>
-      <c r="AD2" s="146"/>
-      <c r="AE2" s="146"/>
-      <c r="AF2" s="146"/>
-      <c r="AG2" s="146"/>
-      <c r="AH2" s="146"/>
-      <c r="AI2" s="146"/>
-      <c r="AJ2" s="146"/>
-      <c r="AK2" s="146"/>
-      <c r="AL2" s="146"/>
-      <c r="AM2" s="146"/>
-      <c r="AN2" s="146"/>
-      <c r="AO2" s="146">
+      <c r="AD2" s="141"/>
+      <c r="AE2" s="141"/>
+      <c r="AF2" s="141"/>
+      <c r="AG2" s="141"/>
+      <c r="AH2" s="141"/>
+      <c r="AI2" s="141"/>
+      <c r="AJ2" s="141"/>
+      <c r="AK2" s="141"/>
+      <c r="AL2" s="141"/>
+      <c r="AM2" s="141"/>
+      <c r="AN2" s="141"/>
+      <c r="AO2" s="141">
         <v>26</v>
       </c>
-      <c r="AP2" s="146"/>
-      <c r="AQ2" s="146"/>
-      <c r="AR2" s="146"/>
-      <c r="AS2" s="146"/>
-      <c r="AT2" s="146"/>
-      <c r="AU2" s="146"/>
-      <c r="AV2" s="146"/>
-      <c r="AW2" s="146"/>
-      <c r="AX2" s="146"/>
-      <c r="AY2" s="146"/>
-      <c r="AZ2" s="147"/>
-      <c r="BA2" s="146">
+      <c r="AP2" s="141"/>
+      <c r="AQ2" s="141"/>
+      <c r="AR2" s="141"/>
+      <c r="AS2" s="141"/>
+      <c r="AT2" s="141"/>
+      <c r="AU2" s="141"/>
+      <c r="AV2" s="141"/>
+      <c r="AW2" s="141"/>
+      <c r="AX2" s="141"/>
+      <c r="AY2" s="141"/>
+      <c r="AZ2" s="142"/>
+      <c r="BA2" s="141">
         <v>27</v>
       </c>
-      <c r="BB2" s="146"/>
-      <c r="BC2" s="146"/>
-      <c r="BD2" s="146"/>
-      <c r="BE2" s="146"/>
-      <c r="BF2" s="146"/>
-      <c r="BG2" s="146"/>
-      <c r="BH2" s="146"/>
-      <c r="BI2" s="146"/>
-      <c r="BJ2" s="146"/>
-      <c r="BK2" s="146"/>
-      <c r="BL2" s="147"/>
+      <c r="BB2" s="141"/>
+      <c r="BC2" s="141"/>
+      <c r="BD2" s="141"/>
+      <c r="BE2" s="141"/>
+      <c r="BF2" s="141"/>
+      <c r="BG2" s="141"/>
+      <c r="BH2" s="141"/>
+      <c r="BI2" s="141"/>
+      <c r="BJ2" s="141"/>
+      <c r="BK2" s="141"/>
+      <c r="BL2" s="142"/>
     </row>
     <row r="3" spans="1:64" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="143"/>
-      <c r="C3" s="145"/>
-      <c r="D3" s="145"/>
+      <c r="B3" s="138"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="140"/>
       <c r="E3" s="22">
         <v>1</v>
       </c>
@@ -6184,39 +6350,39 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="151" t="s">
+      <c r="B2" s="146" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="155" t="s">
+      <c r="C2" s="150" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="155" t="s">
+      <c r="D2" s="150" t="s">
         <v>178</v>
       </c>
-      <c r="E2" s="153" t="s">
+      <c r="E2" s="148" t="s">
         <v>127</v>
       </c>
       <c r="F2" s="98" t="s">
         <v>113</v>
       </c>
-      <c r="G2" s="149" t="s">
+      <c r="G2" s="144" t="s">
         <v>114</v>
       </c>
-      <c r="H2" s="149"/>
-      <c r="I2" s="149"/>
-      <c r="J2" s="150"/>
-      <c r="K2" s="149" t="s">
+      <c r="H2" s="144"/>
+      <c r="I2" s="144"/>
+      <c r="J2" s="145"/>
+      <c r="K2" s="144" t="s">
         <v>183</v>
       </c>
-      <c r="L2" s="149"/>
-      <c r="M2" s="149"/>
-      <c r="N2" s="150"/>
+      <c r="L2" s="144"/>
+      <c r="M2" s="144"/>
+      <c r="N2" s="145"/>
     </row>
     <row r="3" spans="1:14" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="152"/>
-      <c r="C3" s="156"/>
-      <c r="D3" s="156"/>
-      <c r="E3" s="154"/>
+      <c r="B3" s="147"/>
+      <c r="C3" s="151"/>
+      <c r="D3" s="151"/>
+      <c r="E3" s="149"/>
       <c r="F3" s="99" t="s">
         <v>112</v>
       </c>
@@ -6959,30 +7125,30 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="151" t="s">
+      <c r="B2" s="146" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="155" t="s">
+      <c r="C2" s="150" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="155" t="s">
+      <c r="D2" s="150" t="s">
         <v>178</v>
       </c>
-      <c r="E2" s="153" t="s">
+      <c r="E2" s="148" t="s">
         <v>127</v>
       </c>
-      <c r="F2" s="149" t="s">
+      <c r="F2" s="144" t="s">
         <v>183</v>
       </c>
-      <c r="G2" s="149"/>
-      <c r="H2" s="149"/>
-      <c r="I2" s="150"/>
+      <c r="G2" s="144"/>
+      <c r="H2" s="144"/>
+      <c r="I2" s="145"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="152"/>
-      <c r="C3" s="156"/>
-      <c r="D3" s="156"/>
-      <c r="E3" s="154"/>
+      <c r="B3" s="147"/>
+      <c r="C3" s="151"/>
+      <c r="D3" s="151"/>
+      <c r="E3" s="149"/>
       <c r="F3" s="99" t="s">
         <v>115</v>
       </c>
@@ -7360,30 +7526,30 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="151" t="s">
+      <c r="B2" s="146" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="155" t="s">
+      <c r="C2" s="150" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="155" t="s">
+      <c r="D2" s="150" t="s">
         <v>178</v>
       </c>
-      <c r="E2" s="153" t="s">
+      <c r="E2" s="148" t="s">
         <v>127</v>
       </c>
-      <c r="F2" s="149" t="s">
+      <c r="F2" s="144" t="s">
         <v>228</v>
       </c>
-      <c r="G2" s="149"/>
-      <c r="H2" s="149"/>
-      <c r="I2" s="150"/>
+      <c r="G2" s="144"/>
+      <c r="H2" s="144"/>
+      <c r="I2" s="145"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="152"/>
-      <c r="C3" s="156"/>
-      <c r="D3" s="156"/>
-      <c r="E3" s="154"/>
+      <c r="B3" s="147"/>
+      <c r="C3" s="151"/>
+      <c r="D3" s="151"/>
+      <c r="E3" s="149"/>
       <c r="F3" s="99" t="s">
         <v>115</v>
       </c>
@@ -7743,7 +7909,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.375" style="83" customWidth="1"/>
@@ -7751,11 +7917,11 @@
     <col min="3" max="4" width="14.75" style="83" customWidth="1"/>
     <col min="5" max="5" width="43" style="83" customWidth="1"/>
     <col min="6" max="6" width="61.875" style="83" customWidth="1"/>
-    <col min="7" max="10" width="62.125" style="83" customWidth="1"/>
-    <col min="11" max="16384" width="9" style="83"/>
+    <col min="7" max="9" width="62.125" style="83" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="83"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="110" t="s">
         <v>0</v>
       </c>
@@ -7766,51 +7932,47 @@
       <c r="D1" s="111"/>
       <c r="E1" s="109"/>
     </row>
-    <row r="2" spans="1:10" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="151" t="s">
+    <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="146" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="155" t="s">
+      <c r="C2" s="150" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="155" t="s">
+      <c r="D2" s="150" t="s">
         <v>178</v>
       </c>
-      <c r="E2" s="153" t="s">
+      <c r="E2" s="148" t="s">
         <v>127</v>
       </c>
-      <c r="F2" s="149" t="s">
+      <c r="F2" s="144" t="s">
         <v>260</v>
       </c>
-      <c r="G2" s="149"/>
-      <c r="H2" s="149"/>
-      <c r="I2" s="157"/>
-      <c r="J2" s="150"/>
-    </row>
-    <row r="3" spans="1:10" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="152"/>
-      <c r="C3" s="156"/>
-      <c r="D3" s="156"/>
-      <c r="E3" s="154"/>
+      <c r="G2" s="144"/>
+      <c r="H2" s="144"/>
+      <c r="I2" s="145"/>
+    </row>
+    <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="147"/>
+      <c r="C3" s="151"/>
+      <c r="D3" s="151"/>
+      <c r="E3" s="149"/>
       <c r="F3" s="99" t="s">
-        <v>115</v>
+        <v>295</v>
       </c>
       <c r="G3" s="99" t="s">
-        <v>116</v>
+        <v>271</v>
       </c>
       <c r="H3" s="99" t="s">
-        <v>117</v>
-      </c>
-      <c r="I3" s="99" t="s">
-        <v>262</v>
-      </c>
-      <c r="J3" s="100" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="84" t="s">
-        <v>118</v>
+        <v>272</v>
+      </c>
+      <c r="I3" s="100" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="168" t="s">
+        <v>109</v>
       </c>
       <c r="C4" s="118" t="s">
         <v>176</v>
@@ -7818,366 +7980,737 @@
       <c r="D4" s="118" t="s">
         <v>179</v>
       </c>
-      <c r="E4" s="92" t="s">
-        <v>153</v>
-      </c>
-      <c r="F4" s="116"/>
-      <c r="G4" s="107"/>
+      <c r="E4" s="157" t="s">
+        <v>141</v>
+      </c>
+      <c r="F4" s="158"/>
+      <c r="G4" s="159"/>
       <c r="H4" s="90"/>
-      <c r="I4" s="131"/>
-      <c r="J4" s="94"/>
-    </row>
-    <row r="5" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="85" t="s">
-        <v>124</v>
+      <c r="I4" s="94"/>
+    </row>
+    <row r="5" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="171" t="s">
+        <v>182</v>
       </c>
       <c r="C5" s="119" t="s">
-        <v>176</v>
+        <v>284</v>
       </c>
       <c r="D5" s="119" t="s">
-        <v>179</v>
-      </c>
-      <c r="E5" s="93" t="s">
-        <v>154</v>
+        <v>181</v>
+      </c>
+      <c r="E5" s="102" t="s">
+        <v>162</v>
       </c>
       <c r="F5" s="116"/>
       <c r="G5" s="107"/>
-      <c r="H5" s="91"/>
-      <c r="I5" s="132"/>
-      <c r="J5" s="95"/>
-    </row>
-    <row r="6" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="85" t="s">
-        <v>125</v>
+      <c r="H5" s="125" t="s">
+        <v>281</v>
+      </c>
+      <c r="I5" s="152" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="169" t="s">
+        <v>292</v>
       </c>
       <c r="C6" s="119" t="s">
-        <v>176</v>
+        <v>285</v>
       </c>
       <c r="D6" s="119" t="s">
         <v>179</v>
       </c>
-      <c r="E6" s="93" t="s">
-        <v>155</v>
-      </c>
-      <c r="F6" s="116"/>
-      <c r="G6" s="107"/>
-      <c r="H6" s="91"/>
-      <c r="I6" s="132"/>
-      <c r="J6" s="95"/>
-    </row>
-    <row r="7" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="85" t="s">
-        <v>126</v>
+      <c r="E6" s="102" t="s">
+        <v>162</v>
+      </c>
+      <c r="F6" s="125"/>
+      <c r="G6" s="125"/>
+      <c r="H6" s="125"/>
+      <c r="I6" s="152"/>
+    </row>
+    <row r="7" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="169" t="s">
+        <v>76</v>
       </c>
       <c r="C7" s="119" t="s">
-        <v>176</v>
+        <v>286</v>
       </c>
       <c r="D7" s="119" t="s">
         <v>179</v>
       </c>
-      <c r="E7" s="93" t="s">
-        <v>156</v>
+      <c r="E7" s="102" t="s">
+        <v>163</v>
       </c>
       <c r="F7" s="116"/>
       <c r="G7" s="107"/>
       <c r="H7" s="91"/>
-      <c r="I7" s="132"/>
-      <c r="J7" s="95"/>
-    </row>
-    <row r="8" spans="1:10" ht="108" x14ac:dyDescent="0.3">
-      <c r="B8" s="137" t="s">
-        <v>3</v>
+      <c r="I7" s="95"/>
+    </row>
+    <row r="8" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="169" t="s">
+        <v>110</v>
       </c>
       <c r="C8" s="119" t="s">
-        <v>263</v>
+        <v>285</v>
       </c>
       <c r="D8" s="119" t="s">
         <v>179</v>
       </c>
       <c r="E8" s="93" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="F8" s="116"/>
-      <c r="G8" s="107"/>
-      <c r="H8" s="140" t="s">
-        <v>281</v>
-      </c>
-      <c r="I8" s="132"/>
-      <c r="J8" s="95"/>
-    </row>
-    <row r="9" spans="1:10" ht="27" x14ac:dyDescent="0.3">
-      <c r="B9" s="137" t="s">
-        <v>46</v>
+      <c r="G8" s="106"/>
+      <c r="H8" s="91"/>
+      <c r="I8" s="95"/>
+    </row>
+    <row r="9" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="170" t="s">
+        <v>118</v>
       </c>
       <c r="C9" s="119" t="s">
-        <v>264</v>
+        <v>285</v>
       </c>
       <c r="D9" s="119" t="s">
         <v>179</v>
       </c>
-      <c r="E9" s="102" t="s">
-        <v>273</v>
+      <c r="E9" s="93" t="s">
+        <v>153</v>
       </c>
       <c r="F9" s="116"/>
       <c r="G9" s="107"/>
-      <c r="H9" s="106" t="s">
-        <v>280</v>
-      </c>
-      <c r="I9" s="132"/>
-      <c r="J9" s="95"/>
-    </row>
-    <row r="10" spans="1:10" ht="67.5" x14ac:dyDescent="0.3">
-      <c r="B10" s="137" t="s">
-        <v>56</v>
+      <c r="H9" s="155"/>
+      <c r="I9" s="95"/>
+    </row>
+    <row r="10" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="170" t="s">
+        <v>124</v>
       </c>
       <c r="C10" s="119" t="s">
-        <v>265</v>
+        <v>285</v>
       </c>
       <c r="D10" s="119" t="s">
         <v>179</v>
       </c>
-      <c r="E10" s="102" t="s">
-        <v>274</v>
+      <c r="E10" s="93" t="s">
+        <v>154</v>
       </c>
       <c r="F10" s="116"/>
       <c r="G10" s="107"/>
-      <c r="H10" s="140" t="s">
-        <v>282</v>
-      </c>
-      <c r="I10" s="134" t="s">
-        <v>278</v>
-      </c>
-      <c r="J10" s="141" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="67.5" x14ac:dyDescent="0.3">
-      <c r="B11" s="139" t="s">
-        <v>63</v>
+      <c r="H10" s="155"/>
+      <c r="I10" s="95"/>
+    </row>
+    <row r="11" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="170" t="s">
+        <v>125</v>
       </c>
       <c r="C11" s="119" t="s">
-        <v>263</v>
+        <v>285</v>
       </c>
       <c r="D11" s="119" t="s">
         <v>179</v>
       </c>
-      <c r="E11" s="102" t="s">
-        <v>275</v>
+      <c r="E11" s="93" t="s">
+        <v>155</v>
       </c>
       <c r="F11" s="116"/>
       <c r="G11" s="107"/>
-      <c r="H11" s="91"/>
-      <c r="I11" s="134" t="s">
-        <v>283</v>
-      </c>
-      <c r="J11" s="95"/>
-    </row>
-    <row r="12" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="137" t="s">
-        <v>74</v>
+      <c r="H11" s="155"/>
+      <c r="I11" s="95"/>
+    </row>
+    <row r="12" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="170" t="s">
+        <v>126</v>
       </c>
       <c r="C12" s="119" t="s">
-        <v>180</v>
+        <v>285</v>
       </c>
       <c r="D12" s="119" t="s">
         <v>179</v>
       </c>
-      <c r="E12" s="102" t="s">
-        <v>276</v>
+      <c r="E12" s="93" t="s">
+        <v>156</v>
       </c>
       <c r="F12" s="116"/>
       <c r="G12" s="107"/>
-      <c r="H12" s="91"/>
-      <c r="I12" s="134" t="s">
-        <v>269</v>
-      </c>
-      <c r="J12" s="95"/>
-    </row>
-    <row r="13" spans="1:10" ht="347.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="86" t="s">
-        <v>119</v>
+      <c r="H12" s="155"/>
+      <c r="I12" s="95"/>
+    </row>
+    <row r="13" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
+      <c r="B13" s="134" t="s">
+        <v>63</v>
       </c>
       <c r="C13" s="119" t="s">
-        <v>176</v>
+        <v>287</v>
       </c>
       <c r="D13" s="119" t="s">
         <v>179</v>
       </c>
       <c r="E13" s="102" t="s">
-        <v>162</v>
+        <v>264</v>
       </c>
       <c r="F13" s="116"/>
       <c r="G13" s="107"/>
-      <c r="H13" s="91"/>
-      <c r="I13" s="132"/>
-      <c r="J13" s="95"/>
-    </row>
-    <row r="14" spans="1:10" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="B14" s="87" t="s">
-        <v>182</v>
+      <c r="H13" s="135" t="s">
+        <v>277</v>
+      </c>
+      <c r="I13" s="136"/>
+    </row>
+    <row r="14" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="133" t="s">
+        <v>74</v>
       </c>
       <c r="C14" s="119" t="s">
-        <v>180</v>
+        <v>287</v>
       </c>
       <c r="D14" s="119" t="s">
-        <v>181</v>
-      </c>
-      <c r="E14" s="102"/>
-      <c r="F14" s="125"/>
-      <c r="G14" s="125"/>
-      <c r="H14" s="125"/>
-      <c r="I14" s="125" t="s">
-        <v>268</v>
-      </c>
-      <c r="J14" s="95"/>
-    </row>
-    <row r="15" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="87" t="s">
-        <v>76</v>
+        <v>179</v>
+      </c>
+      <c r="E14" s="102" t="s">
+        <v>265</v>
+      </c>
+      <c r="F14" s="116"/>
+      <c r="G14" s="107"/>
+      <c r="H14" s="135" t="s">
+        <v>279</v>
+      </c>
+      <c r="I14" s="136"/>
+    </row>
+    <row r="15" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
+      <c r="B15" s="133" t="s">
+        <v>56</v>
       </c>
       <c r="C15" s="119" t="s">
-        <v>176</v>
+        <v>288</v>
       </c>
       <c r="D15" s="119" t="s">
         <v>179</v>
       </c>
       <c r="E15" s="102" t="s">
-        <v>163</v>
+        <v>263</v>
       </c>
       <c r="F15" s="116"/>
-      <c r="G15" s="107"/>
-      <c r="H15" s="91"/>
-      <c r="I15" s="132"/>
-      <c r="J15" s="95"/>
-    </row>
-    <row r="16" spans="1:10" ht="81" x14ac:dyDescent="0.3">
-      <c r="B16" s="137" t="s">
+      <c r="G15" s="135" t="s">
+        <v>269</v>
+      </c>
+      <c r="H15" s="154" t="s">
+        <v>299</v>
+      </c>
+      <c r="I15" s="136"/>
+    </row>
+    <row r="16" spans="1:9" ht="81" x14ac:dyDescent="0.3">
+      <c r="B16" s="133" t="s">
         <v>86</v>
       </c>
       <c r="C16" s="119" t="s">
-        <v>266</v>
+        <v>289</v>
       </c>
       <c r="D16" s="119" t="s">
         <v>179</v>
       </c>
       <c r="E16" s="102" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="F16" s="116"/>
       <c r="G16" s="107"/>
-      <c r="H16" s="91"/>
-      <c r="I16" s="134" t="s">
-        <v>270</v>
-      </c>
-      <c r="J16" s="95"/>
-    </row>
-    <row r="17" spans="2:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="138" t="s">
-        <v>142</v>
+      <c r="H16" s="135" t="s">
+        <v>300</v>
+      </c>
+      <c r="I16" s="136"/>
+    </row>
+    <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="132" t="s">
+        <v>168</v>
       </c>
       <c r="C17" s="119" t="s">
-        <v>180</v>
+        <v>287</v>
       </c>
       <c r="D17" s="119" t="s">
         <v>179</v>
       </c>
-      <c r="E17" s="93" t="s">
-        <v>106</v>
+      <c r="E17" s="115" t="s">
+        <v>270</v>
       </c>
       <c r="F17" s="116"/>
-      <c r="G17" s="91"/>
-      <c r="H17" s="91"/>
-      <c r="I17" s="132"/>
-      <c r="J17" s="95"/>
-    </row>
-    <row r="18" spans="2:10" ht="27" x14ac:dyDescent="0.3">
-      <c r="B18" s="88" t="s">
-        <v>107</v>
+      <c r="G17" s="131" t="s">
+        <v>261</v>
+      </c>
+      <c r="H17" s="154" t="s">
+        <v>283</v>
+      </c>
+      <c r="I17" s="153"/>
+    </row>
+    <row r="18" spans="2:9" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="133" t="s">
+        <v>142</v>
       </c>
       <c r="C18" s="119" t="s">
-        <v>176</v>
+        <v>290</v>
       </c>
       <c r="D18" s="119" t="s">
         <v>179</v>
       </c>
-      <c r="E18" s="102" t="s">
-        <v>165</v>
+      <c r="E18" s="115" t="s">
+        <v>301</v>
       </c>
       <c r="F18" s="116"/>
-      <c r="G18" s="107"/>
-      <c r="H18" s="91"/>
-      <c r="I18" s="132"/>
-      <c r="J18" s="95"/>
-    </row>
-    <row r="19" spans="2:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="87" t="s">
-        <v>110</v>
-      </c>
-      <c r="C19" s="119" t="s">
-        <v>176</v>
-      </c>
-      <c r="D19" s="119" t="s">
+      <c r="G18" s="131"/>
+      <c r="H18" s="154"/>
+      <c r="I18" s="153"/>
+    </row>
+    <row r="19" spans="2:9" ht="108" x14ac:dyDescent="0.3">
+      <c r="B19" s="167" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" s="156" t="s">
+        <v>287</v>
+      </c>
+      <c r="D19" s="156" t="s">
         <v>179</v>
       </c>
       <c r="E19" s="93" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="F19" s="116"/>
-      <c r="G19" s="106"/>
-      <c r="H19" s="91"/>
-      <c r="I19" s="132"/>
-      <c r="J19" s="95"/>
-    </row>
-    <row r="20" spans="2:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="136" t="s">
-        <v>168</v>
-      </c>
-      <c r="C20" s="119" t="s">
+      <c r="G19" s="135" t="s">
+        <v>268</v>
+      </c>
+      <c r="I19" s="95"/>
+    </row>
+    <row r="20" spans="2:9" ht="14.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="160" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" s="161" t="s">
+        <v>291</v>
+      </c>
+      <c r="D20" s="161" t="s">
+        <v>179</v>
+      </c>
+      <c r="E20" s="162" t="s">
+        <v>262</v>
+      </c>
+      <c r="F20" s="163"/>
+      <c r="G20" s="164" t="s">
         <v>267</v>
       </c>
-      <c r="D20" s="119" t="s">
-        <v>179</v>
-      </c>
-      <c r="E20" s="115" t="s">
-        <v>284</v>
-      </c>
-      <c r="F20" s="116"/>
-      <c r="G20" s="112"/>
-      <c r="H20" s="135" t="s">
-        <v>271</v>
-      </c>
-      <c r="I20" s="135" t="s">
-        <v>272</v>
-      </c>
-      <c r="J20" s="114"/>
-    </row>
-    <row r="21" spans="2:10" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="89" t="s">
-        <v>109</v>
-      </c>
-      <c r="C21" s="120" t="s">
-        <v>176</v>
-      </c>
-      <c r="D21" s="120" t="s">
-        <v>179</v>
-      </c>
-      <c r="E21" s="105" t="s">
-        <v>141</v>
-      </c>
-      <c r="F21" s="117"/>
-      <c r="G21" s="108"/>
-      <c r="H21" s="96"/>
-      <c r="I21" s="133"/>
-      <c r="J21" s="97"/>
-    </row>
-    <row r="22" spans="2:10" ht="14.25" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="H20" s="165"/>
+      <c r="I20" s="166"/>
+    </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="F2:I2"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.375" style="83" customWidth="1"/>
+    <col min="2" max="2" width="9" style="83"/>
+    <col min="3" max="4" width="14.75" style="83" customWidth="1"/>
+    <col min="5" max="5" width="43" style="83" customWidth="1"/>
+    <col min="6" max="6" width="61.875" style="83" customWidth="1"/>
+    <col min="7" max="9" width="62.125" style="83" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="83"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="110" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="111" t="s">
+        <v>150</v>
+      </c>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="109"/>
+    </row>
+    <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="146" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="150" t="s">
+        <v>177</v>
+      </c>
+      <c r="D2" s="150" t="s">
+        <v>178</v>
+      </c>
+      <c r="E2" s="148" t="s">
+        <v>127</v>
+      </c>
+      <c r="F2" s="144" t="s">
+        <v>293</v>
+      </c>
+      <c r="G2" s="144"/>
+      <c r="H2" s="144"/>
+      <c r="I2" s="145"/>
+    </row>
+    <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="147"/>
+      <c r="C3" s="151"/>
+      <c r="D3" s="151"/>
+      <c r="E3" s="149"/>
+      <c r="F3" s="99" t="s">
+        <v>294</v>
+      </c>
+      <c r="G3" s="99" t="s">
+        <v>296</v>
+      </c>
+      <c r="H3" s="99" t="s">
+        <v>297</v>
+      </c>
+      <c r="I3" s="100" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="168" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" s="118" t="s">
+        <v>176</v>
+      </c>
+      <c r="D4" s="118" t="s">
+        <v>179</v>
+      </c>
+      <c r="E4" s="157" t="s">
+        <v>141</v>
+      </c>
+      <c r="F4" s="158"/>
+      <c r="G4" s="159"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="94"/>
+    </row>
+    <row r="5" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="171" t="s">
+        <v>182</v>
+      </c>
+      <c r="C5" s="119" t="s">
+        <v>284</v>
+      </c>
+      <c r="D5" s="119" t="s">
+        <v>181</v>
+      </c>
+      <c r="E5" s="102" t="s">
+        <v>162</v>
+      </c>
+      <c r="F5" s="116"/>
+      <c r="G5" s="107"/>
+      <c r="H5" s="125" t="s">
+        <v>281</v>
+      </c>
+      <c r="I5" s="152" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="169" t="s">
+        <v>292</v>
+      </c>
+      <c r="C6" s="119" t="s">
+        <v>285</v>
+      </c>
+      <c r="D6" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E6" s="102" t="s">
+        <v>162</v>
+      </c>
+      <c r="F6" s="125"/>
+      <c r="G6" s="125"/>
+      <c r="H6" s="125"/>
+      <c r="I6" s="152"/>
+    </row>
+    <row r="7" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="169" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="119" t="s">
+        <v>286</v>
+      </c>
+      <c r="D7" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E7" s="102" t="s">
+        <v>163</v>
+      </c>
+      <c r="F7" s="116"/>
+      <c r="G7" s="107"/>
+      <c r="H7" s="91"/>
+      <c r="I7" s="95"/>
+    </row>
+    <row r="8" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="169" t="s">
+        <v>110</v>
+      </c>
+      <c r="C8" s="119" t="s">
+        <v>285</v>
+      </c>
+      <c r="D8" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E8" s="93" t="s">
+        <v>140</v>
+      </c>
+      <c r="F8" s="116"/>
+      <c r="G8" s="106"/>
+      <c r="H8" s="91"/>
+      <c r="I8" s="95"/>
+    </row>
+    <row r="9" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="170" t="s">
+        <v>118</v>
+      </c>
+      <c r="C9" s="119" t="s">
+        <v>285</v>
+      </c>
+      <c r="D9" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E9" s="93" t="s">
+        <v>153</v>
+      </c>
+      <c r="F9" s="116"/>
+      <c r="G9" s="107"/>
+      <c r="H9" s="155"/>
+      <c r="I9" s="95"/>
+    </row>
+    <row r="10" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="170" t="s">
+        <v>124</v>
+      </c>
+      <c r="C10" s="119" t="s">
+        <v>285</v>
+      </c>
+      <c r="D10" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E10" s="93" t="s">
+        <v>154</v>
+      </c>
+      <c r="F10" s="116"/>
+      <c r="G10" s="107"/>
+      <c r="H10" s="155"/>
+      <c r="I10" s="95"/>
+    </row>
+    <row r="11" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="170" t="s">
+        <v>125</v>
+      </c>
+      <c r="C11" s="119" t="s">
+        <v>285</v>
+      </c>
+      <c r="D11" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E11" s="93" t="s">
+        <v>155</v>
+      </c>
+      <c r="F11" s="116"/>
+      <c r="G11" s="107"/>
+      <c r="H11" s="155"/>
+      <c r="I11" s="95"/>
+    </row>
+    <row r="12" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="170" t="s">
+        <v>126</v>
+      </c>
+      <c r="C12" s="119" t="s">
+        <v>285</v>
+      </c>
+      <c r="D12" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E12" s="93" t="s">
+        <v>156</v>
+      </c>
+      <c r="F12" s="116"/>
+      <c r="G12" s="107"/>
+      <c r="H12" s="155"/>
+      <c r="I12" s="95"/>
+    </row>
+    <row r="13" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
+      <c r="B13" s="134" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="119" t="s">
+        <v>287</v>
+      </c>
+      <c r="D13" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E13" s="102" t="s">
+        <v>264</v>
+      </c>
+      <c r="F13" s="116"/>
+      <c r="G13" s="107"/>
+      <c r="H13" s="135" t="s">
+        <v>277</v>
+      </c>
+      <c r="I13" s="136" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="133" t="s">
+        <v>74</v>
+      </c>
+      <c r="C14" s="119" t="s">
+        <v>287</v>
+      </c>
+      <c r="D14" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E14" s="102" t="s">
+        <v>265</v>
+      </c>
+      <c r="F14" s="116"/>
+      <c r="G14" s="107"/>
+      <c r="H14" s="135" t="s">
+        <v>279</v>
+      </c>
+      <c r="I14" s="136" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
+      <c r="B15" s="133" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="119" t="s">
+        <v>288</v>
+      </c>
+      <c r="D15" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E15" s="102" t="s">
+        <v>263</v>
+      </c>
+      <c r="F15" s="116"/>
+      <c r="G15" s="135" t="s">
+        <v>269</v>
+      </c>
+      <c r="H15" s="154" t="s">
+        <v>275</v>
+      </c>
+      <c r="I15" s="136" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="81" x14ac:dyDescent="0.3">
+      <c r="B16" s="133" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" s="119" t="s">
+        <v>289</v>
+      </c>
+      <c r="D16" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E16" s="102" t="s">
+        <v>266</v>
+      </c>
+      <c r="F16" s="116"/>
+      <c r="G16" s="107"/>
+      <c r="H16" s="135" t="s">
+        <v>282</v>
+      </c>
+      <c r="I16" s="136"/>
+    </row>
+    <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="132" t="s">
+        <v>168</v>
+      </c>
+      <c r="C17" s="119" t="s">
+        <v>287</v>
+      </c>
+      <c r="D17" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E17" s="115" t="s">
+        <v>270</v>
+      </c>
+      <c r="F17" s="116"/>
+      <c r="G17" s="131" t="s">
+        <v>261</v>
+      </c>
+      <c r="H17" s="154" t="s">
+        <v>283</v>
+      </c>
+      <c r="I17" s="153"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B18" s="133" t="s">
+        <v>142</v>
+      </c>
+      <c r="C18" s="119" t="s">
+        <v>290</v>
+      </c>
+      <c r="D18" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="E18" s="115"/>
+      <c r="F18" s="116"/>
+      <c r="G18" s="131"/>
+      <c r="H18" s="154"/>
+      <c r="I18" s="153"/>
+    </row>
+    <row r="19" spans="2:9" ht="108" x14ac:dyDescent="0.3">
+      <c r="B19" s="167" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" s="156" t="s">
+        <v>287</v>
+      </c>
+      <c r="D19" s="156" t="s">
+        <v>179</v>
+      </c>
+      <c r="E19" s="93" t="s">
+        <v>157</v>
+      </c>
+      <c r="F19" s="116"/>
+      <c r="G19" s="135" t="s">
+        <v>268</v>
+      </c>
+      <c r="I19" s="95"/>
+    </row>
+    <row r="20" spans="2:9" ht="14.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="160" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" s="161" t="s">
+        <v>291</v>
+      </c>
+      <c r="D20" s="161" t="s">
+        <v>179</v>
+      </c>
+      <c r="E20" s="162" t="s">
+        <v>262</v>
+      </c>
+      <c r="F20" s="163"/>
+      <c r="G20" s="164" t="s">
+        <v>267</v>
+      </c>
+      <c r="H20" s="165"/>
+      <c r="I20" s="166"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:I2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Weekly Plan 작성 완료
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\2.project\hkmc_ptc_heater\Doc\1. 일정\1. Weekly Plan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\일정\ptc_heater_doc\1. 일정\1. Weekly Plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="309">
   <si>
     <t>■</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1819,21 +1819,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>[임제훈 사원]
-- LHD ESIR 계획서 작성
-- R로직 튜닝</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- Core Temp 튜닝 결과 확인 (~10/21)
-- ESIR 계획서 등록 (~10/24)
-- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/24)
-- R로직 튜닝 (~10/24)
-- 최신 승인도 확인</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve">[우리산업]
 PM : 유정호, 기구 : 공준석, HW : 신지훈, 
 제조 : 전진호, 품질 : 박상철, 일렉스 : 남시온, 류상근, 박철수, 슬로박법인 : 김예현
@@ -1842,6 +1827,48 @@
 freshair@hyundai.com
 [신차 품질팀]
 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- LHD, RHD 사양 3D 모델링 수령 (10/21)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- LHD R로직 튜닝
+- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- LHD ESIR 계획서 작성
+- R로직 튜닝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- 최소 작동 전압 범위 수정 후, EV HTR 개발팀 김민수 선임에게 전달 (~10/24)
+  : 0℃, -30℃ 환경에서 QV Air PTC와 160V, 170V 출력 비교 필요로 인한 요청</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- 온도 정합성 테스트 (10/20)
+- 제어기 선행품질 검증 현황 작성 (10/21)
+- 제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 (10/23)
+- 설계 변경 진행</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- Core Temp 튜닝 결과 확인 (~10/22)
+- HVAC RPM 확인 (~10/22)
+- 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (~10/22)
+- R로직 튜닝 (~10/22)
+- ESIR 계획서 등록 (~10/24)
+- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/24)
+- 최신 승인도 확인 (~10/31)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3188,7 +3215,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="172">
+  <cellXfs count="173">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3704,6 +3731,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -5488,7 +5518,7 @@
         <v>85</v>
       </c>
       <c r="D15" s="34" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E15" s="6"/>
       <c r="F15" s="7"/>
@@ -8127,7 +8157,7 @@
       </c>
       <c r="F10" s="116"/>
       <c r="G10" s="107"/>
-      <c r="H10" s="140"/>
+      <c r="H10" s="91"/>
       <c r="I10" s="95"/>
     </row>
     <row r="11" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -8145,7 +8175,7 @@
       </c>
       <c r="F11" s="116"/>
       <c r="G11" s="107"/>
-      <c r="H11" s="140"/>
+      <c r="H11" s="91"/>
       <c r="I11" s="95"/>
     </row>
     <row r="12" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -8182,7 +8212,7 @@
       <c r="F13" s="116"/>
       <c r="G13" s="107"/>
       <c r="H13" s="135" t="s">
-        <v>277</v>
+        <v>307</v>
       </c>
       <c r="I13" s="136"/>
     </row>
@@ -8202,7 +8232,7 @@
       <c r="F14" s="116"/>
       <c r="G14" s="107"/>
       <c r="H14" s="135" t="s">
-        <v>279</v>
+        <v>304</v>
       </c>
       <c r="I14" s="136"/>
     </row>
@@ -8224,11 +8254,11 @@
         <v>269</v>
       </c>
       <c r="H15" s="139" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="I15" s="136"/>
     </row>
-    <row r="16" spans="1:9" ht="81" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="108" x14ac:dyDescent="0.3">
       <c r="B16" s="133" t="s">
         <v>86</v>
       </c>
@@ -8244,7 +8274,7 @@
       <c r="F16" s="116"/>
       <c r="G16" s="107"/>
       <c r="H16" s="135" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="I16" s="136"/>
     </row>
@@ -8265,8 +8295,8 @@
       <c r="G17" s="131" t="s">
         <v>261</v>
       </c>
-      <c r="H17" s="139" t="s">
-        <v>283</v>
+      <c r="H17" s="172" t="s">
+        <v>303</v>
       </c>
       <c r="I17" s="138"/>
     </row>
@@ -8285,7 +8315,7 @@
       </c>
       <c r="F18" s="116"/>
       <c r="G18" s="131"/>
-      <c r="H18" s="139"/>
+      <c r="H18" s="135"/>
       <c r="I18" s="138"/>
     </row>
     <row r="19" spans="2:9" ht="108" x14ac:dyDescent="0.3">
@@ -8304,6 +8334,9 @@
       <c r="F19" s="116"/>
       <c r="G19" s="135" t="s">
         <v>268</v>
+      </c>
+      <c r="H19" s="135" t="s">
+        <v>306</v>
       </c>
       <c r="I19" s="95"/>
     </row>

</xml_diff>

<commit_message>
Weekly Plan 4주차 작성 완료
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="316">
   <si>
     <t>■</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1836,8 +1836,32 @@
   </si>
   <si>
     <t>[임제훈 사원]
+- SWE.3 SDDS 후속 작업 (진행률 : 95%)
+- SPQA 프로세스 절차를 따라 ALM 등록 (~10/31)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
 - LHD R로직 튜닝
 - RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- LHD R로직 튜닝
+- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- LHD ESIR 계획서 작성 (~10/24)
+- R로직 튜닝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- LHD ESIR 계획서 작성 (~10/24)
+- R로직 튜닝</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1848,26 +1872,100 @@
   </si>
   <si>
     <t>[임제훈 사원]
-- LHD ESIR 계획서 작성 (~10/24)
-- R로직 튜닝</t>
+- 최소 작동 전압 범위 수정 후, EV HTR 개발팀 김민수 선임에게 전달 (~10/24)
+  : 0℃, -30℃ 환경에서 QV Air PTC와 160V, 170V 출력 비교 필요로 인한 요청</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>[임제훈 사원]
-- Core Temp 튜닝 결과 확인 (~10/22)
-- HVAC RPM 확인 (~10/22)
-- R로직 튜닝 (~10/22)
-- 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (~10/24)
-- ESIR 계획서 등록 (~10/24)
-- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/24)
-- 최신 승인도 확인 (~10/31)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- 온도 정합성 테스트 (10/20)
-- 제어기 선행품질 검증 현황 작성 (10/21)
-- 제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 (10/23)
+- 설계 변경 진행 (~10/24)
+- 제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 후 자료 회신 (~10/29)
+  : 1. P2 단계 전까지 매 월 1회 제어기 검증 현황 관련 회의 진행 예정
+    2. 진행 단계 별로 이력 및 변경점 꾸준히 업데이트 해서 자료 회신 요청
+    3. Fail Safety 항목 공유 요청
+    4. 제어기 검증 프로세스 관련 자료 공유 요청
+    5. 컨버전 룰이 무엇인지에 대한 자료 공유 요청
+    6. S/W 검증 현황의 검증 항목별 LIST 자료 공유 요청
+    7. CPU / 메모리 부하율 관리 방안 재확인 요청
+    8. 고장 진단 로그 저장 가능 개수 재확인 요청
+- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/31)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[임제훈 사원]
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>온도 정합성 테스트 (10/20)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>제어기 선행품질 검증 현황 작성 (10/21)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 (10/23)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
   : 1. P2 단계 전까지 매 월 1회 제어기 검증 현황 관련 회의 진행 예정
     2. 진행 단계 별로 이력 및 변경점 꾸준히 업데이트 해서 자료 회신 요청
     3. Fail Safety 항목 공유 요청
@@ -1878,11 +1976,80 @@
     8. 고장 진단 로그 저장 가능 개수 재확인 요청
 - 설계 변경 진행 (~10/24)
 - 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/31)</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[임제훈 사원]
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Core Temp 튜닝 결과 확인 (~10/22)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>HVAC RPM 확인 (~10/22)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- R로직 튜닝 (~10/22)
+- 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (~10/24)
+- ESIR 계획서 등록 (~10/24)
+- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/24)
+- 최신 승인도 확인 (~10/31)</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>[임제훈 사원]
-- SWE.3 SDDS 후속 작업 (진행률 : 95%)
+- 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (~10/24)
+- R로직 튜닝 (~10/28)
+- ESIR 계획서 등록 (~10/28)
+- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/28)
+- 최신 승인도 확인 (~10/31)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- SWE.3 SDDS 후속 작업 (진행률 : 100%)
 - SPQA 프로세스 절차를 따라 ALM 등록 (~10/31)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -8079,10 +8246,10 @@
       <c r="F5" s="116"/>
       <c r="G5" s="107"/>
       <c r="H5" s="125" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="I5" s="137" t="s">
-        <v>280</v>
+        <v>315</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -8227,9 +8394,11 @@
       <c r="F13" s="116"/>
       <c r="G13" s="107"/>
       <c r="H13" s="135" t="s">
-        <v>308</v>
-      </c>
-      <c r="I13" s="136"/>
+        <v>312</v>
+      </c>
+      <c r="I13" s="136" t="s">
+        <v>311</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="133" t="s">
@@ -8247,9 +8416,11 @@
       <c r="F14" s="116"/>
       <c r="G14" s="107"/>
       <c r="H14" s="135" t="s">
-        <v>304</v>
-      </c>
-      <c r="I14" s="136"/>
+        <v>305</v>
+      </c>
+      <c r="I14" s="136" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="15" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
       <c r="B15" s="133" t="s">
@@ -8269,9 +8440,11 @@
         <v>269</v>
       </c>
       <c r="H15" s="139" t="s">
-        <v>306</v>
-      </c>
-      <c r="I15" s="136"/>
+        <v>307</v>
+      </c>
+      <c r="I15" s="136" t="s">
+        <v>308</v>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="108" x14ac:dyDescent="0.3">
       <c r="B16" s="133" t="s">
@@ -8289,9 +8462,11 @@
       <c r="F16" s="116"/>
       <c r="G16" s="107"/>
       <c r="H16" s="135" t="s">
-        <v>307</v>
-      </c>
-      <c r="I16" s="136"/>
+        <v>313</v>
+      </c>
+      <c r="I16" s="136" t="s">
+        <v>314</v>
+      </c>
     </row>
     <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="132" t="s">
@@ -8351,9 +8526,11 @@
         <v>268</v>
       </c>
       <c r="H19" s="135" t="s">
-        <v>305</v>
-      </c>
-      <c r="I19" s="95"/>
+        <v>309</v>
+      </c>
+      <c r="I19" s="136" t="s">
+        <v>310</v>
+      </c>
     </row>
     <row r="20" spans="2:9" ht="14.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="145" t="s">

</xml_diff>

<commit_message>
Weekly Plan NX5e 수정 완료
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -2040,17 +2040,18 @@
   </si>
   <si>
     <t>[임제훈 사원]
-- 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (~10/24)
+- SWE.3 SDDS 후속 작업 (진행률 : 100%)
+- SPQA 프로세스 절차를 따라 ALM 등록 (~10/31)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
 - R로직 튜닝 (~10/28)
 - ESIR 계획서 등록 (~10/28)
 - 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/28)
+- 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (10/30)
+  : 휴가 중, 목요일 출근 예정, 이 때 메일로 다시 문의
 - 최신 승인도 확인 (~10/31)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- SWE.3 SDDS 후속 작업 (진행률 : 100%)
-- SPQA 프로세스 절차를 따라 ALM 등록 (~10/31)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -8249,7 +8250,7 @@
         <v>304</v>
       </c>
       <c r="I5" s="137" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -8465,7 +8466,7 @@
         <v>313</v>
       </c>
       <c r="I16" s="136" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Weekly Plan 수정 완료
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -1874,21 +1874,6 @@
     <t>[임제훈 사원]
 - 최소 작동 전압 범위 수정 후, EV HTR 개발팀 김민수 선임에게 전달 (~10/24)
   : 0℃, -30℃ 환경에서 QV Air PTC와 160V, 170V 출력 비교 필요로 인한 요청</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- 설계 변경 진행 (~10/24)
-- 제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 후 자료 회신 (~10/29)
-  : 1. P2 단계 전까지 매 월 1회 제어기 검증 현황 관련 회의 진행 예정
-    2. 진행 단계 별로 이력 및 변경점 꾸준히 업데이트 해서 자료 회신 요청
-    3. Fail Safety 항목 공유 요청
-    4. 제어기 검증 프로세스 관련 자료 공유 요청
-    5. 컨버전 룰이 무엇인지에 대한 자료 공유 요청
-    6. S/W 검증 현황의 검증 항목별 LIST 자료 공유 요청
-    7. CPU / 메모리 부하율 관리 방안 재확인 요청
-    8. 고장 진단 로그 저장 가능 개수 재확인 요청
-- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/31)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -2046,6 +2031,24 @@
   </si>
   <si>
     <t>[임제훈 사원]
+- 설계 변경 진행 (~10/24)
+- CPU 및 메모리 부하율 관리 대책 르네사스 문의 (~10/27)
+- 사이버 보안 항목 QV와 비교 및 리스트업 후 공조시스템설계팀 회신 (~10/27)
+- 제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 후 자료 회신 (~10/29)
+  : 1. P2 단계 전까지 매 월 1회 제어기 검증 현황 관련 회의 진행 예정
+    2. 진행 단계 별로 이력 및 변경점 꾸준히 업데이트 해서 자료 회신 요청
+    3. Fail Safety 항목 공유 요청
+    4. 제어기 검증 프로세스 관련 자료 공유 요청
+    5. 컨버전 룰이 무엇인지에 대한 자료 공유 요청
+    6. S/W 검증 현황의 검증 항목별 LIST 자료 공유 요청
+    7. CPU / 메모리 부하율 관리 방안 재확인 요청
+    8. 고장 진단 로그 저장 가능 개수 재확인 요청
+- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/31)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- ESIR 일정에 맞춰서 5가지 항목 다 가능한지 파악하기 (~10/27)
 - R로직 튜닝 (~10/28)
 - ESIR 계획서 등록 (~10/28)
 - 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/28)
@@ -8250,7 +8253,7 @@
         <v>304</v>
       </c>
       <c r="I5" s="137" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -8395,10 +8398,10 @@
       <c r="F13" s="116"/>
       <c r="G13" s="107"/>
       <c r="H13" s="135" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="I13" s="136" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -8463,7 +8466,7 @@
       <c r="F16" s="116"/>
       <c r="G16" s="107"/>
       <c r="H16" s="135" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="I16" s="136" t="s">
         <v>315</v>

</xml_diff>

<commit_message>
Weekly Plan NX5e 내용 추가
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -2516,21 +2516,26 @@
   </si>
   <si>
     <t>[임제훈 사원]
+- BJ PTC HTR 벤치 시험 합동 평가 일정 (10/29 예정)
+  : SW 대응은 딱히 없을 것 같다고 했지만, 결과나 진행 사항 파악 필요
+- LHD R로직 튜닝
+- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
 - R로직 튜닝 (~10/27)
 - ESIR 일정에 맞춰서 5가지 항목 다 가능한지 파악하기 (~10/29)
 - 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (10/30)
   : 휴가 중, 목요일 출근 예정, 이 때 메일로 다시 문의
+- ES 규격 대로 15초 내로 목표 전력 도달 SW로 변경 (~10/29)
+  : Softstart enable 0으로 변경
+  : Sofftstart 0일 때, R로직 확인, 전력 구간 별 칼로리와 CAN 출력 차이 비교
 - ESIR 계획서 등록 (~10/31)
 - 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/31)
-- 최신 승인도 확인 (~10/31)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- BJ PTC HTR 벤치 시험 합동 평가 일정 (10/29 예정)
-  : SW 대응은 딱히 없을 것 같다고 했지만, 결과나 진행 사항 파악 필요
-- LHD R로직 튜닝
-- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
+- 최신 승인도 확인 (~10/31)
+- 제작사양서 배포 준비 (~10/31)
+  : SW 파일, 제어사양서</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -8907,7 +8912,7 @@
         <v>305</v>
       </c>
       <c r="I14" s="136" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
@@ -8934,7 +8939,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="108" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="175.5" x14ac:dyDescent="0.3">
       <c r="B16" s="133" t="s">
         <v>86</v>
       </c>
@@ -8953,7 +8958,7 @@
         <v>313</v>
       </c>
       <c r="I16" s="136" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
11월 Weekly Plan 작성
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="17685" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="17685" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="대일정" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="316">
   <si>
     <t>■</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -259,17 +259,6 @@
 dong3082@kia.com
 [샤시부품개발2팀]
 김현우 책임 010-8493-6493</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[전자편의개발 2팀] 
-서상기 책임 010-9311-9821
-zsskz@hyundai.com
-[공조시스템설계팀] 
-김응영 책임 010-7635-0265
-key@hyundai.com
-안성민 책임연구원 
-freshair@hyundai.com</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1661,84 +1650,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>2주차 (10/10 ~ 10/15)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>3주차 (10/16 ~ 10/22)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>4주차 (10/23 ~ 10/29)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- AY 회의 진행 (25/10/20)
-- LHD ESIR
-- R로직 튜닝</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- AY 회의 진행 (25/10/20)
-- LHD ESIR
-- R로직 튜닝</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- 온도 정합성 테스트 (10/20)
-- 제어기 선행품질 검증 현황 작성
-- 제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 (10/23)
-- 설계 변경 진행</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- 온도 정합성 테스트 (10/20)
-- 제어기 선행품질 검증 현황 작성
-- 제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 (10/23)
-- 설계 변경 진행</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- LHD R로직 튜닝
-- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- LHD R로직 튜닝
-- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- SWE.3 SDDS 후속 작업 (진행률 : 90%)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- SWE.3 SDDS 후속 작업 (진행률 : 90%)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- ESIR 계획서 등록
-- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신
-- Core Temp 튜닝 결과 확인
-- 최신 승인도 확인
-- R로직 튜닝</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">[임제훈 사원]
-- </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>오세영
 조현진
 임제훈</t>
@@ -1781,23 +1692,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>1주차 (10/30 ~ 11/05)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>1주차 (10/02)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2주차 (11/06 ~ 11/12)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>3주차 (11/13 ~ 11/19)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>4주차 (11/20 ~ 11/26)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1938,12 +1833,6 @@
 - 설계 변경 진행 (~10/24)
 - 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/31)</t>
     </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- LHD ESIR 계획서 (기구, HW 업로드 후, 행추가 예정) (~10/31)
-- R로직 튜닝</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -2487,14 +2376,6 @@
   </si>
   <si>
     <t>[임제훈 사원]
-- BJ PTC HTR 벤치 시험 합동 평가 일정 (10/29 예정)
-  : SW 대응은 딱히 없을 것 같다고 했지만, 결과나 진행 사항 파악 필요
-- LHD R로직 튜닝
-- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
 - SWE.3 SDDS 후속 작업 (진행률 : 100%)
 - SPQA 프로세스 절차를 따라 ALM 등록 (~10/31)
 [조현진 전임]
@@ -2559,22 +2440,325 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>4주차 (10/24 ~ 10/30)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3주차 (10/17 ~ 10/23)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2주차 (10/10 ~ 10/16)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1주차 (10/31 ~ 11/06)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2주차 (11/07 ~ 11/13)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3주차 (11/14 ~ 11/20)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>4주차 (11/21 ~ 11/27)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>[임제훈 사원]
-- R로직 튜닝 (~10/27)
-- ESIR 일정에 맞춰서 5가지 항목 다 가능한지 파악하기 (~10/29)
+- SWE.3 SDDS 후속 작업 (진행률 : 100%)
+- SPQA 프로세스 절차를 따라 ALM 등록 (~11/06)
+[조현진 전임]
+- SWE.1, 2, 3 등록에 맞추어 SWE. 4, 5, 6 ALM 등록</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[임제훈 사원]
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BJ PTC HTR 벤치 시험 합동 평가 일정 (10/29 예정)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  : SW 대응은 딱히 없을 것 같다고 했지만, 결과나 진행 사항 파악 필요
+- LHD R로직 튜닝
+- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[임제훈 사원]
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>R로직 튜닝 (~10/27)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ESIR 일정에 맞춰서 5가지 항목 다 가능한지 파악하기 (~10/29)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
 - 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (10/30)
   : 휴가 중, 목요일 출근 예정, 이 때 메일로 다시 문의
-- ES 규격 대로 15초 내로 목표 전력 도달 SW로 변경 (~10/29)
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ES 규격 대로 15초 내로 목표 전력 도달 SW로 변경 (~10/29)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
   : Softstart enable 0으로 변경
   : Sofftstart 0일 때, R로직 확인, 전력 구간 별 칼로리와 CAN 출력 차이 비교
 - ESIR 계획서 등록 (~10/31)
-- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/31)
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/31)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
 - 최신 승인도 확인 (~10/31)
-- 제작사양서 배포 준비 (~10/31)
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>제작사양서 배포 준비 (~10/31)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
   : SW 파일, 제어사양서
   : 10월 14일부터 tc 160℃, 스톤 기울기 변경되었음
   : 제작사양서 배포 기준, tc 160℃ 스톤 기울기 변경된 샘플 기준으로 튜닝 완료
   : P1 때 tc 165℃ 변경 협의 중</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- LHD R로직 튜닝
+- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- R로직 튜닝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">임제훈 사원]
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">LHD ESIR 계획서 (기구, HW 업로드 후, 행추가 예정) (~10/31)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  : 90700-00, 95480-00 계획서 등록 완료</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- R로직 튜닝</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (~11/03)
+  : 10/30 문의 완료, 재회신 요청 예정
+- ESIR 계획서 등록 (~11/05)
+- 최신 승인도 확인 (~11/06)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[우리산업]
+PM : 유정호, 품질 : 박상철, 기구 : 김민수, 공준석, HW : 신지훈
+[전자편의개발 2팀] 
+서상기 책임 010-9311-9821
+zsskz@hyundai.com
+[공조시스템설계팀] 
+김응영 책임 010-7635-0265
+key@hyundai.com
+이웅기 연구원 010-8427-8230
+lwg8230@hyundai.com
+[기아샤시시스템품질팀]
+김제일 매니저
+J1@kia.com</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[우리산업]
+기구 : 정우헌, HW : 신지훈
+[공조시스템설계팀]
+정재근 책임 연구원 010-9402-3594
+wjdworms1357@hyundai.com
+김동환 연구원 010-4162-2776
+kdh2776@hyundai.com</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- 사이버 보안 항목 QV와 비교 및 리스트업 후 공조시스템설계팀 회신 (~11/05)
+  : ES95489-21 빼는 것은 안됨. 업데이트에 해당하는 항목 N/A로 하자고 회신 받음
+- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~11/03)
+- 설계 변경 진행 (~11/10)
+  : 기구팀 문의 결과, QV, SVm, BJ 담당자 전부 똑같다고 함. 결재 라인 똑같이 예정
+  : 설계 변경 문서 작성</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2809,7 +2993,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="81">
+  <borders count="83">
     <border>
       <left/>
       <right/>
@@ -3921,6 +4105,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom style="hair">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -3942,7 +4148,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="174">
+  <cellXfs count="179">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -4464,6 +4670,21 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="81" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="81" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -5091,7 +5312,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="161" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D2" s="161" t="s">
         <v>39</v>
@@ -5354,10 +5575,10 @@
     </row>
     <row r="4" spans="1:64" ht="183" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="63" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C4" s="61" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D4" s="35" t="s">
         <v>42</v>
@@ -5435,10 +5656,10 @@
     </row>
     <row r="5" spans="1:64" ht="81" x14ac:dyDescent="0.3">
       <c r="B5" s="28" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C5" s="62" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>41</v>
@@ -5514,10 +5735,10 @@
     </row>
     <row r="6" spans="1:64" ht="67.5" x14ac:dyDescent="0.3">
       <c r="B6" s="28" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C6" s="58" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D6" s="34" t="s">
         <v>40</v>
@@ -5597,10 +5818,10 @@
     </row>
     <row r="7" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="28" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C7" s="58" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D7" s="33"/>
       <c r="E7" s="6"/>
@@ -5678,7 +5899,7 @@
     </row>
     <row r="8" spans="1:64" ht="81" x14ac:dyDescent="0.3">
       <c r="B8" s="28" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C8" s="58"/>
       <c r="D8" s="33"/>
@@ -5702,7 +5923,7 @@
       <c r="V8" s="30"/>
       <c r="W8" s="30"/>
       <c r="X8" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="Y8" s="31"/>
       <c r="Z8" s="30"/>
@@ -5712,22 +5933,22 @@
       <c r="AD8" s="31"/>
       <c r="AE8" s="31"/>
       <c r="AF8" s="15" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="AG8" s="31"/>
       <c r="AH8" s="31"/>
       <c r="AI8" s="17" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AJ8" s="31"/>
       <c r="AK8" s="31"/>
       <c r="AL8" s="31"/>
       <c r="AM8" s="17" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AN8" s="123"/>
       <c r="AO8" s="29" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="AP8" s="31"/>
       <c r="AQ8" s="31"/>
@@ -5758,7 +5979,7 @@
         <v>3</v>
       </c>
       <c r="C9" s="59" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D9" s="33"/>
       <c r="E9" s="6"/>
@@ -5783,11 +6004,11 @@
       <c r="X9" s="7"/>
       <c r="Y9" s="7"/>
       <c r="Z9" s="17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AA9" s="7"/>
       <c r="AB9" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AC9" s="9"/>
       <c r="AD9" s="7"/>
@@ -5828,10 +6049,10 @@
     </row>
     <row r="10" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="27" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C10" s="58" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D10" s="33"/>
       <c r="E10" s="6"/>
@@ -5854,11 +6075,11 @@
       <c r="V10" s="7"/>
       <c r="W10" s="7"/>
       <c r="X10" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Y10" s="7"/>
       <c r="Z10" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="AA10" s="7"/>
       <c r="AB10" s="8"/>
@@ -5871,7 +6092,7 @@
       </c>
       <c r="AH10" s="7"/>
       <c r="AI10" s="13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="AJ10" s="7"/>
       <c r="AK10" s="7"/>
@@ -5905,10 +6126,10 @@
     </row>
     <row r="11" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="28" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C11" s="58" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D11" s="33"/>
       <c r="E11" s="6"/>
@@ -5934,34 +6155,34 @@
       <c r="Y11" s="7"/>
       <c r="Z11" s="7"/>
       <c r="AA11" s="37" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AB11" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AC11" s="9"/>
       <c r="AD11" s="30"/>
       <c r="AE11" s="31"/>
       <c r="AF11" s="31"/>
       <c r="AG11" s="13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AH11" s="7"/>
       <c r="AI11" s="13"/>
       <c r="AJ11" s="7"/>
       <c r="AK11" s="17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AL11" s="7"/>
       <c r="AM11" s="7"/>
       <c r="AN11" s="8"/>
       <c r="AO11" s="9"/>
       <c r="AP11" s="17" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AQ11" s="7"/>
       <c r="AR11" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AS11" s="7"/>
       <c r="AT11" s="7"/>
@@ -5986,10 +6207,10 @@
     </row>
     <row r="12" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="28" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C12" s="58" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D12" s="33"/>
       <c r="E12" s="6"/>
@@ -6024,12 +6245,12 @@
       <c r="AH12" s="7"/>
       <c r="AI12" s="13"/>
       <c r="AJ12" s="101" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AK12" s="36"/>
       <c r="AL12" s="13"/>
       <c r="AM12" s="13" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AN12" s="8"/>
       <c r="AO12" s="12"/>
@@ -6046,7 +6267,7 @@
       </c>
       <c r="AW12" s="7"/>
       <c r="AX12" s="13" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AY12" s="7"/>
       <c r="AZ12" s="10"/>
@@ -6063,15 +6284,15 @@
       <c r="BK12" s="31"/>
       <c r="BL12" s="10"/>
     </row>
-    <row r="13" spans="1:64" ht="183.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:64" ht="228.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C13" s="59" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D13" s="34" t="s">
-        <v>43</v>
+        <v>313</v>
       </c>
       <c r="E13" s="6"/>
       <c r="F13" s="7"/>
@@ -6094,7 +6315,7 @@
       <c r="U13" s="7"/>
       <c r="V13" s="7"/>
       <c r="W13" s="13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="X13" s="7"/>
       <c r="Y13" s="7"/>
@@ -6107,11 +6328,11 @@
       <c r="AF13" s="7"/>
       <c r="AG13" s="7"/>
       <c r="AH13" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AI13" s="36"/>
       <c r="AJ13" s="17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AK13" s="30"/>
       <c r="AL13" s="7"/>
@@ -6119,19 +6340,19 @@
         <v>4</v>
       </c>
       <c r="AN13" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="AO13" s="9"/>
       <c r="AP13" s="7"/>
       <c r="AQ13" s="17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AR13" s="7"/>
       <c r="AS13" s="13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AT13" s="13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AU13" s="7"/>
       <c r="AV13" s="7"/>
@@ -6154,13 +6375,13 @@
     </row>
     <row r="14" spans="1:64" ht="67.5" x14ac:dyDescent="0.3">
       <c r="B14" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="59" t="s">
+        <v>83</v>
+      </c>
+      <c r="D14" s="34" t="s">
         <v>74</v>
-      </c>
-      <c r="C14" s="59" t="s">
-        <v>84</v>
-      </c>
-      <c r="D14" s="34" t="s">
-        <v>75</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="7"/>
@@ -6200,13 +6421,13 @@
       <c r="AH14" s="7"/>
       <c r="AI14" s="7"/>
       <c r="AJ14" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AK14" s="13" t="s">
         <v>13</v>
       </c>
       <c r="AL14" s="17" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="AM14" s="7"/>
       <c r="AN14" s="8"/>
@@ -6221,7 +6442,7 @@
         <v>15</v>
       </c>
       <c r="AU14" s="13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AV14" s="7"/>
       <c r="AW14" s="7"/>
@@ -6243,13 +6464,13 @@
     </row>
     <row r="15" spans="1:64" ht="285.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C15" s="59" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D15" s="34" t="s">
-        <v>302</v>
+        <v>284</v>
       </c>
       <c r="E15" s="6"/>
       <c r="F15" s="7"/>
@@ -6272,7 +6493,7 @@
       <c r="W15" s="7"/>
       <c r="X15" s="7"/>
       <c r="Y15" s="13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Z15" s="13"/>
       <c r="AA15" s="7"/>
@@ -6280,26 +6501,26 @@
       <c r="AC15" s="12"/>
       <c r="AD15" s="7"/>
       <c r="AE15" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="AF15" s="38"/>
       <c r="AG15" s="37" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AH15" s="7"/>
       <c r="AI15" s="37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AJ15" s="30"/>
       <c r="AK15" s="7"/>
       <c r="AL15" s="13"/>
       <c r="AM15" s="13"/>
       <c r="AN15" s="17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AO15" s="9"/>
       <c r="AP15" s="13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AQ15" s="13"/>
       <c r="AR15" s="7"/>
@@ -6326,10 +6547,10 @@
     </row>
     <row r="16" spans="1:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="27" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C16" s="59" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D16" s="33"/>
       <c r="E16" s="6"/>
@@ -6374,25 +6595,25 @@
       <c r="AH16" s="7"/>
       <c r="AI16" s="13"/>
       <c r="AJ16" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="AK16" s="37" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AL16" s="7"/>
       <c r="AM16" s="37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AN16" s="8"/>
       <c r="AO16" s="12"/>
       <c r="AP16" s="13"/>
       <c r="AQ16" s="13"/>
       <c r="AR16" s="17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AS16" s="7"/>
       <c r="AT16" s="13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AU16" s="7"/>
       <c r="AV16" s="7"/>
@@ -6415,13 +6636,13 @@
     </row>
     <row r="17" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="57" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C17" s="60" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D17" s="76" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E17" s="40"/>
       <c r="F17" s="41"/>
@@ -6432,13 +6653,13 @@
       <c r="K17" s="41"/>
       <c r="L17" s="41"/>
       <c r="M17" s="13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="N17" s="41"/>
       <c r="O17" s="41"/>
       <c r="P17" s="43"/>
       <c r="Q17" s="104" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="R17" s="103"/>
       <c r="S17" s="41"/>
@@ -6448,7 +6669,7 @@
       <c r="W17" s="42"/>
       <c r="X17" s="41"/>
       <c r="Y17" s="30" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="Z17" s="41"/>
       <c r="AA17" s="41"/>
@@ -6461,7 +6682,7 @@
       <c r="AH17" s="41"/>
       <c r="AI17" s="37"/>
       <c r="AJ17" s="30" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AK17" s="46"/>
       <c r="AL17" s="41"/>
@@ -6469,11 +6690,11 @@
       <c r="AN17" s="8"/>
       <c r="AO17" s="47"/>
       <c r="AP17" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AQ17" s="42"/>
       <c r="AR17" s="37" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AS17" s="41"/>
       <c r="AT17" s="42"/>
@@ -6481,7 +6702,7 @@
       <c r="AV17" s="41"/>
       <c r="AW17" s="41"/>
       <c r="AX17" s="17" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AY17" s="41"/>
       <c r="AZ17" s="48"/>
@@ -6489,7 +6710,7 @@
       <c r="BB17" s="45"/>
       <c r="BC17" s="45"/>
       <c r="BD17" s="13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="BE17" s="71"/>
       <c r="BF17" s="45"/>
@@ -6500,14 +6721,16 @@
       <c r="BK17" s="71"/>
       <c r="BL17" s="48"/>
     </row>
-    <row r="18" spans="2:64" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:64" ht="108" x14ac:dyDescent="0.3">
       <c r="B18" s="27" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C18" s="59" t="s">
-        <v>259</v>
-      </c>
-      <c r="D18" s="33"/>
+        <v>258</v>
+      </c>
+      <c r="D18" s="178" t="s">
+        <v>314</v>
+      </c>
       <c r="E18" s="64"/>
       <c r="F18" s="65"/>
       <c r="G18" s="65"/>
@@ -6535,12 +6758,12 @@
       <c r="AC18" s="67"/>
       <c r="AD18" s="65"/>
       <c r="AE18" s="68" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AF18" s="65"/>
       <c r="AG18" s="68"/>
       <c r="AH18" s="56" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AI18" s="69"/>
       <c r="AJ18" s="65"/>
@@ -6561,27 +6784,27 @@
       <c r="AU18" s="73"/>
       <c r="AV18" s="65"/>
       <c r="AW18" s="69" t="s">
+        <v>88</v>
+      </c>
+      <c r="AX18" s="69" t="s">
         <v>89</v>
       </c>
-      <c r="AX18" s="69" t="s">
+      <c r="AY18" s="69" t="s">
         <v>90</v>
       </c>
-      <c r="AY18" s="69" t="s">
+      <c r="AZ18" s="70" t="s">
         <v>91</v>
-      </c>
-      <c r="AZ18" s="70" t="s">
-        <v>92</v>
       </c>
       <c r="BA18" s="67"/>
       <c r="BB18" s="73" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="BC18" s="73"/>
       <c r="BD18" s="73" t="s">
+        <v>93</v>
+      </c>
+      <c r="BE18" s="73" t="s">
         <v>94</v>
-      </c>
-      <c r="BE18" s="73" t="s">
-        <v>95</v>
       </c>
       <c r="BF18" s="72"/>
       <c r="BG18" s="73"/>
@@ -6593,10 +6816,10 @@
     </row>
     <row r="19" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="77" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C19" s="78" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D19" s="33"/>
       <c r="E19" s="64"/>
@@ -6637,11 +6860,11 @@
       <c r="AN19" s="66"/>
       <c r="AO19" s="67"/>
       <c r="AP19" s="69" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AQ19" s="69"/>
       <c r="AR19" s="69" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AS19" s="65"/>
       <c r="AT19" s="65"/>
@@ -6651,7 +6874,7 @@
       <c r="AX19" s="65"/>
       <c r="AY19" s="69"/>
       <c r="AZ19" s="70" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="BA19" s="67"/>
       <c r="BB19" s="72"/>
@@ -6659,29 +6882,29 @@
       <c r="BD19" s="72"/>
       <c r="BE19" s="72"/>
       <c r="BF19" s="73" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="BG19" s="73"/>
       <c r="BH19" s="73" t="s">
+        <v>99</v>
+      </c>
+      <c r="BI19" s="73" t="s">
         <v>100</v>
       </c>
-      <c r="BI19" s="73" t="s">
+      <c r="BJ19" s="73" t="s">
         <v>101</v>
-      </c>
-      <c r="BJ19" s="73" t="s">
-        <v>102</v>
       </c>
       <c r="BK19" s="73"/>
       <c r="BL19" s="70" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="20" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="77" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C20" s="78" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D20" s="39"/>
       <c r="E20" s="64"/>
@@ -6747,13 +6970,13 @@
     </row>
     <row r="21" spans="2:64" ht="137.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="57" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C21" s="82" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D21" s="34" t="s">
-        <v>315</v>
+        <v>295</v>
       </c>
       <c r="E21" s="64"/>
       <c r="F21" s="65"/>
@@ -6794,14 +7017,14 @@
       <c r="AO21" s="67"/>
       <c r="AP21" s="69"/>
       <c r="AQ21" s="69" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="AR21" s="69"/>
       <c r="AS21" s="65"/>
       <c r="AT21" s="65"/>
       <c r="AU21" s="69"/>
       <c r="AV21" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AW21" s="65"/>
       <c r="AX21" s="65"/>
@@ -6809,20 +7032,20 @@
       <c r="AZ21" s="70"/>
       <c r="BA21" s="67"/>
       <c r="BB21" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="BC21" s="73"/>
       <c r="BD21" s="69" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="BE21" s="72"/>
       <c r="BF21" s="73"/>
       <c r="BG21" s="69" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="BH21" s="73"/>
       <c r="BI21" s="69" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="BJ21" s="73"/>
       <c r="BK21" s="73"/>
@@ -6830,10 +7053,10 @@
     </row>
     <row r="22" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="57" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C22" s="82" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D22" s="39"/>
       <c r="E22" s="64"/>
@@ -6899,10 +7122,10 @@
     </row>
     <row r="23" spans="2:64" ht="61.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="79" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C23" s="80" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D23" s="81"/>
       <c r="E23" s="49"/>
@@ -6996,118 +7219,118 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C1" t="s">
         <v>239</v>
-      </c>
-      <c r="C1" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="126" t="s">
+        <v>240</v>
+      </c>
+      <c r="B2" t="s">
         <v>241</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="127" t="s">
         <v>242</v>
       </c>
-      <c r="C2" s="127" t="s">
+      <c r="D2" t="s">
         <v>243</v>
-      </c>
-      <c r="D2" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="126" t="s">
+        <v>244</v>
+      </c>
+      <c r="B3" t="s">
+        <v>241</v>
+      </c>
+      <c r="C3" s="128" t="s">
         <v>245</v>
       </c>
-      <c r="B3" t="s">
-        <v>242</v>
-      </c>
-      <c r="C3" s="128" t="s">
-        <v>246</v>
-      </c>
       <c r="D3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="126" t="s">
+        <v>246</v>
+      </c>
+      <c r="B4" t="s">
+        <v>241</v>
+      </c>
+      <c r="C4" s="128" t="s">
         <v>247</v>
       </c>
-      <c r="B4" t="s">
-        <v>242</v>
-      </c>
-      <c r="C4" s="128" t="s">
-        <v>248</v>
-      </c>
       <c r="D4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="129" t="s">
+        <v>248</v>
+      </c>
+      <c r="B5" t="s">
+        <v>241</v>
+      </c>
+      <c r="C5" s="128" t="s">
         <v>249</v>
       </c>
-      <c r="B5" t="s">
-        <v>242</v>
-      </c>
-      <c r="C5" s="128" t="s">
-        <v>250</v>
-      </c>
       <c r="D5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="127" t="s">
+        <v>250</v>
+      </c>
+      <c r="B6" t="s">
+        <v>243</v>
+      </c>
+      <c r="C6" s="130" t="s">
         <v>251</v>
       </c>
-      <c r="B6" t="s">
-        <v>244</v>
-      </c>
-      <c r="C6" s="130" t="s">
-        <v>252</v>
-      </c>
       <c r="D6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="127" t="s">
+        <v>252</v>
+      </c>
+      <c r="B7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C7" s="130" t="s">
         <v>253</v>
       </c>
-      <c r="B7" t="s">
-        <v>244</v>
-      </c>
-      <c r="C7" s="130" t="s">
-        <v>254</v>
-      </c>
       <c r="D7" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C8" s="126" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D8" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C9" s="126" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C10" s="130" t="s">
+        <v>256</v>
+      </c>
+      <c r="D10" t="s">
         <v>257</v>
-      </c>
-      <c r="D10" t="s">
-        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -7133,10 +7356,10 @@
   <sheetData>
     <row r="1" spans="1:14" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="110" t="s">
+        <v>148</v>
+      </c>
+      <c r="B1" s="111" t="s">
         <v>149</v>
-      </c>
-      <c r="B1" s="111" t="s">
-        <v>150</v>
       </c>
       <c r="C1" s="111"/>
       <c r="D1" s="111"/>
@@ -7147,25 +7370,25 @@
         <v>2</v>
       </c>
       <c r="C2" s="172" t="s">
+        <v>176</v>
+      </c>
+      <c r="D2" s="172" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="172" t="s">
-        <v>178</v>
-      </c>
       <c r="E2" s="170" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F2" s="98" t="s">
+        <v>112</v>
+      </c>
+      <c r="G2" s="166" t="s">
         <v>113</v>
-      </c>
-      <c r="G2" s="166" t="s">
-        <v>114</v>
       </c>
       <c r="H2" s="166"/>
       <c r="I2" s="166"/>
       <c r="J2" s="167"/>
       <c r="K2" s="166" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="L2" s="166"/>
       <c r="M2" s="166"/>
@@ -7177,169 +7400,169 @@
       <c r="D3" s="173"/>
       <c r="E3" s="171"/>
       <c r="F3" s="99" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G3" s="99" t="s">
+        <v>114</v>
+      </c>
+      <c r="H3" s="99" t="s">
         <v>115</v>
       </c>
-      <c r="H3" s="99" t="s">
+      <c r="I3" s="99" t="s">
         <v>116</v>
       </c>
-      <c r="I3" s="99" t="s">
-        <v>117</v>
-      </c>
       <c r="J3" s="100" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K3" s="99" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="L3" s="99" t="s">
+        <v>115</v>
+      </c>
+      <c r="M3" s="99" t="s">
         <v>116</v>
       </c>
-      <c r="M3" s="99" t="s">
-        <v>117</v>
-      </c>
       <c r="N3" s="100" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B4" s="84" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C4" s="118" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D4" s="118" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E4" s="92" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F4" s="107" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G4" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H4" s="107" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I4" s="107" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="J4" s="94"/>
       <c r="K4" s="107" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="L4" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M4" s="107"/>
       <c r="N4" s="94"/>
     </row>
     <row r="5" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B5" s="85" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C5" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D5" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E5" s="93" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F5" s="107" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G5" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H5" s="107" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I5" s="107" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="J5" s="95"/>
       <c r="K5" s="107" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="L5" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M5" s="107"/>
       <c r="N5" s="95"/>
     </row>
     <row r="6" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B6" s="85" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C6" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D6" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E6" s="93" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F6" s="107" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G6" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H6" s="107" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I6" s="107" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="J6" s="95"/>
       <c r="K6" s="107" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="L6" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M6" s="107"/>
       <c r="N6" s="95"/>
     </row>
     <row r="7" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B7" s="85" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C7" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D7" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E7" s="93" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F7" s="107" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G7" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H7" s="107" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I7" s="107" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="J7" s="95"/>
       <c r="K7" s="107" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="L7" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M7" s="107"/>
       <c r="N7" s="95"/>
@@ -7349,268 +7572,268 @@
         <v>3</v>
       </c>
       <c r="C8" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D8" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E8" s="93" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F8" s="107" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G8" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H8" s="107" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I8" s="107" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="J8" s="95"/>
       <c r="K8" s="107" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="L8" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M8" s="107"/>
       <c r="N8" s="95"/>
     </row>
     <row r="9" spans="1:14" ht="175.5" x14ac:dyDescent="0.3">
       <c r="B9" s="86" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C9" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D9" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E9" s="102" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F9" s="107" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G9" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H9" s="107" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I9" s="107" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="J9" s="95"/>
       <c r="K9" s="107" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="L9" s="107" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="M9" s="107"/>
       <c r="N9" s="95"/>
     </row>
     <row r="10" spans="1:14" ht="121.5" x14ac:dyDescent="0.3">
       <c r="B10" s="86" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C10" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D10" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E10" s="102" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F10" s="107" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G10" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H10" s="107" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I10" s="107" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="J10" s="95"/>
       <c r="K10" s="107" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="L10" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M10" s="107"/>
       <c r="N10" s="95"/>
     </row>
     <row r="11" spans="1:14" ht="108" x14ac:dyDescent="0.3">
       <c r="B11" s="85" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C11" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D11" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E11" s="102" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F11" s="107" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G11" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H11" s="107" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I11" s="107" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J11" s="95"/>
       <c r="K11" s="107" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L11" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M11" s="107"/>
       <c r="N11" s="95"/>
     </row>
     <row r="12" spans="1:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="86" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C12" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D12" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E12" s="102" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F12" s="107" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G12" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H12" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I12" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J12" s="95"/>
       <c r="K12" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L12" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M12" s="107"/>
       <c r="N12" s="95"/>
     </row>
     <row r="13" spans="1:14" ht="347.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="86" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C13" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D13" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E13" s="102" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F13" s="107" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G13" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H13" s="107" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I13" s="107" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="J13" s="95"/>
       <c r="K13" s="107" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="L13" s="107" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="M13" s="107"/>
       <c r="N13" s="95"/>
     </row>
     <row r="14" spans="1:14" ht="175.5" x14ac:dyDescent="0.3">
       <c r="B14" s="87" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C14" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="D14" s="119" t="s">
         <v>180</v>
-      </c>
-      <c r="D14" s="119" t="s">
-        <v>181</v>
       </c>
       <c r="E14" s="102"/>
       <c r="F14" s="107"/>
       <c r="G14" s="116"/>
       <c r="H14" s="107" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I14" s="107" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J14" s="95"/>
       <c r="K14" s="107" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="L14" s="107" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="M14" s="107"/>
       <c r="N14" s="95"/>
     </row>
     <row r="15" spans="1:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="87" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C15" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D15" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E15" s="102" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F15" s="107" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G15" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H15" s="107" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I15" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J15" s="95"/>
       <c r="K15" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L15" s="107"/>
       <c r="M15" s="107"/>
@@ -7618,32 +7841,32 @@
     </row>
     <row r="16" spans="1:14" ht="121.5" x14ac:dyDescent="0.3">
       <c r="B16" s="86" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C16" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D16" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E16" s="93" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F16" s="107" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G16" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H16" s="107" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I16" s="107" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J16" s="95"/>
       <c r="K16" s="107" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="L16" s="107"/>
       <c r="M16" s="107"/>
@@ -7651,173 +7874,173 @@
     </row>
     <row r="17" spans="2:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="88" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C17" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D17" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E17" s="93" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F17" s="91"/>
       <c r="G17" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H17" s="91" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I17" s="91" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J17" s="95"/>
       <c r="K17" s="91" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="L17" s="91" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="M17" s="91"/>
       <c r="N17" s="95"/>
     </row>
     <row r="18" spans="2:14" ht="162" x14ac:dyDescent="0.3">
       <c r="B18" s="88" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C18" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D18" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E18" s="102" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F18" s="107" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G18" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H18" s="107" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I18" s="107" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="J18" s="95"/>
       <c r="K18" s="107" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="L18" s="107" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="M18" s="107"/>
       <c r="N18" s="95"/>
     </row>
     <row r="19" spans="2:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="87" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C19" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D19" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E19" s="93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F19" s="106" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G19" s="116" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H19" s="107" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I19" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J19" s="95"/>
       <c r="K19" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L19" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M19" s="107"/>
       <c r="N19" s="95"/>
     </row>
     <row r="20" spans="2:14" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="87" t="s">
+        <v>168</v>
+      </c>
+      <c r="C20" s="119" t="s">
+        <v>175</v>
+      </c>
+      <c r="D20" s="119" t="s">
+        <v>178</v>
+      </c>
+      <c r="E20" s="115" t="s">
         <v>169</v>
       </c>
-      <c r="C20" s="119" t="s">
-        <v>176</v>
-      </c>
-      <c r="D20" s="119" t="s">
-        <v>179</v>
-      </c>
-      <c r="E20" s="115" t="s">
+      <c r="F20" s="112" t="s">
         <v>170</v>
       </c>
-      <c r="F20" s="112" t="s">
+      <c r="G20" s="116" t="s">
         <v>171</v>
       </c>
-      <c r="G20" s="116" t="s">
-        <v>172</v>
-      </c>
       <c r="H20" s="121" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I20" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J20" s="114"/>
       <c r="K20" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L20" s="107" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M20" s="107"/>
       <c r="N20" s="114"/>
     </row>
     <row r="21" spans="2:14" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="89" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C21" s="120" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D21" s="120" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E21" s="105" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F21" s="108" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G21" s="117" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H21" s="122" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I21" s="122" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J21" s="97"/>
       <c r="K21" s="122" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L21" s="122" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M21" s="122"/>
       <c r="N21" s="97"/>
@@ -7911,7 +8134,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="111" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C1" s="111"/>
       <c r="D1" s="111"/>
@@ -7922,16 +8145,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="172" t="s">
+        <v>176</v>
+      </c>
+      <c r="D2" s="172" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="172" t="s">
-        <v>178</v>
-      </c>
       <c r="E2" s="170" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F2" s="166" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G2" s="166"/>
       <c r="H2" s="166"/>
@@ -7943,30 +8166,30 @@
       <c r="D3" s="173"/>
       <c r="E3" s="171"/>
       <c r="F3" s="99" t="s">
+        <v>114</v>
+      </c>
+      <c r="G3" s="99" t="s">
         <v>115</v>
       </c>
-      <c r="G3" s="99" t="s">
+      <c r="H3" s="99" t="s">
         <v>116</v>
       </c>
-      <c r="H3" s="99" t="s">
-        <v>117</v>
-      </c>
       <c r="I3" s="100" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="84" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C4" s="118" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D4" s="118" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E4" s="92" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F4" s="116"/>
       <c r="G4" s="107"/>
@@ -7975,16 +8198,16 @@
     </row>
     <row r="5" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="85" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C5" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D5" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E5" s="93" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F5" s="116"/>
       <c r="G5" s="107"/>
@@ -7993,16 +8216,16 @@
     </row>
     <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="85" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C6" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D6" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E6" s="93" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F6" s="116"/>
       <c r="G6" s="107"/>
@@ -8011,16 +8234,16 @@
     </row>
     <row r="7" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="85" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C7" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D7" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E7" s="93" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F7" s="116"/>
       <c r="G7" s="107"/>
@@ -8032,13 +8255,13 @@
         <v>3</v>
       </c>
       <c r="C8" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D8" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E8" s="93" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F8" s="116"/>
       <c r="G8" s="107"/>
@@ -8047,16 +8270,16 @@
     </row>
     <row r="9" spans="1:9" ht="27" x14ac:dyDescent="0.3">
       <c r="B9" s="86" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C9" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D9" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E9" s="102" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F9" s="116"/>
       <c r="G9" s="107"/>
@@ -8065,16 +8288,16 @@
     </row>
     <row r="10" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="86" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C10" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D10" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E10" s="102" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F10" s="116"/>
       <c r="G10" s="107"/>
@@ -8083,16 +8306,16 @@
     </row>
     <row r="11" spans="1:9" ht="40.5" x14ac:dyDescent="0.3">
       <c r="B11" s="85" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C11" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D11" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E11" s="102" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F11" s="116"/>
       <c r="G11" s="107"/>
@@ -8101,16 +8324,16 @@
     </row>
     <row r="12" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="86" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C12" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D12" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E12" s="102" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F12" s="116"/>
       <c r="G12" s="107"/>
@@ -8119,16 +8342,16 @@
     </row>
     <row r="13" spans="1:9" ht="347.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="86" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C13" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D13" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E13" s="102" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F13" s="116"/>
       <c r="G13" s="107"/>
@@ -8137,34 +8360,34 @@
     </row>
     <row r="14" spans="1:9" ht="409.5" x14ac:dyDescent="0.3">
       <c r="B14" s="87" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C14" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="D14" s="119" t="s">
         <v>180</v>
-      </c>
-      <c r="D14" s="119" t="s">
-        <v>181</v>
       </c>
       <c r="E14" s="102"/>
       <c r="F14" s="116"/>
       <c r="G14" s="107"/>
       <c r="H14" s="91"/>
       <c r="I14" s="124" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="87" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C15" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D15" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E15" s="102" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F15" s="116"/>
       <c r="G15" s="107"/>
@@ -8173,16 +8396,16 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B16" s="86" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C16" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D16" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E16" s="93" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F16" s="116"/>
       <c r="G16" s="107"/>
@@ -8191,16 +8414,16 @@
     </row>
     <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="88" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C17" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D17" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E17" s="93" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F17" s="116"/>
       <c r="G17" s="91"/>
@@ -8209,16 +8432,16 @@
     </row>
     <row r="18" spans="2:9" ht="27" x14ac:dyDescent="0.3">
       <c r="B18" s="88" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C18" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D18" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E18" s="102" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F18" s="116"/>
       <c r="G18" s="107"/>
@@ -8227,16 +8450,16 @@
     </row>
     <row r="19" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="87" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C19" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D19" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E19" s="93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F19" s="116"/>
       <c r="G19" s="106"/>
@@ -8245,16 +8468,16 @@
     </row>
     <row r="20" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="87" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C20" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D20" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E20" s="115" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F20" s="116"/>
       <c r="G20" s="112"/>
@@ -8263,16 +8486,16 @@
     </row>
     <row r="21" spans="2:9" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="89" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C21" s="120" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D21" s="120" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E21" s="105" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F21" s="117"/>
       <c r="G21" s="108"/>
@@ -8312,7 +8535,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="111" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C1" s="111"/>
       <c r="D1" s="111"/>
@@ -8323,16 +8546,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="172" t="s">
+        <v>176</v>
+      </c>
+      <c r="D2" s="172" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="172" t="s">
-        <v>178</v>
-      </c>
       <c r="E2" s="170" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F2" s="166" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G2" s="166"/>
       <c r="H2" s="166"/>
@@ -8344,30 +8567,30 @@
       <c r="D3" s="173"/>
       <c r="E3" s="171"/>
       <c r="F3" s="99" t="s">
+        <v>114</v>
+      </c>
+      <c r="G3" s="99" t="s">
         <v>115</v>
       </c>
-      <c r="G3" s="99" t="s">
+      <c r="H3" s="99" t="s">
         <v>116</v>
       </c>
-      <c r="H3" s="99" t="s">
-        <v>117</v>
-      </c>
       <c r="I3" s="100" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="84" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C4" s="118" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D4" s="118" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E4" s="92" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F4" s="116"/>
       <c r="G4" s="107"/>
@@ -8376,16 +8599,16 @@
     </row>
     <row r="5" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="85" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C5" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D5" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E5" s="93" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F5" s="116"/>
       <c r="G5" s="107"/>
@@ -8394,16 +8617,16 @@
     </row>
     <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="85" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C6" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D6" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E6" s="93" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F6" s="116"/>
       <c r="G6" s="107"/>
@@ -8412,16 +8635,16 @@
     </row>
     <row r="7" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="85" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C7" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D7" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E7" s="93" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F7" s="116"/>
       <c r="G7" s="107"/>
@@ -8433,13 +8656,13 @@
         <v>3</v>
       </c>
       <c r="C8" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D8" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E8" s="93" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F8" s="116"/>
       <c r="G8" s="107"/>
@@ -8448,16 +8671,16 @@
     </row>
     <row r="9" spans="1:9" ht="27" x14ac:dyDescent="0.3">
       <c r="B9" s="86" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C9" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D9" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E9" s="102" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F9" s="116"/>
       <c r="G9" s="107"/>
@@ -8466,16 +8689,16 @@
     </row>
     <row r="10" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="86" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C10" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D10" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E10" s="102" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F10" s="116"/>
       <c r="G10" s="107"/>
@@ -8484,16 +8707,16 @@
     </row>
     <row r="11" spans="1:9" ht="40.5" x14ac:dyDescent="0.3">
       <c r="B11" s="85" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C11" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D11" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E11" s="102" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F11" s="116"/>
       <c r="G11" s="107"/>
@@ -8502,16 +8725,16 @@
     </row>
     <row r="12" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="86" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C12" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D12" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E12" s="102" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F12" s="116"/>
       <c r="G12" s="107"/>
@@ -8520,16 +8743,16 @@
     </row>
     <row r="13" spans="1:9" ht="347.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="86" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C13" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D13" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E13" s="102" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F13" s="116"/>
       <c r="G13" s="107"/>
@@ -8538,40 +8761,40 @@
     </row>
     <row r="14" spans="1:9" ht="337.5" x14ac:dyDescent="0.3">
       <c r="B14" s="87" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C14" s="119" t="s">
+        <v>179</v>
+      </c>
+      <c r="D14" s="119" t="s">
         <v>180</v>
-      </c>
-      <c r="D14" s="119" t="s">
-        <v>181</v>
       </c>
       <c r="E14" s="102"/>
       <c r="F14" s="125" t="s">
+        <v>229</v>
+      </c>
+      <c r="G14" s="125" t="s">
         <v>230</v>
       </c>
-      <c r="G14" s="125" t="s">
+      <c r="H14" s="125" t="s">
         <v>231</v>
       </c>
-      <c r="H14" s="125" t="s">
-        <v>232</v>
-      </c>
       <c r="I14" s="125" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="87" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C15" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D15" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E15" s="102" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F15" s="116"/>
       <c r="G15" s="107"/>
@@ -8580,16 +8803,16 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B16" s="86" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C16" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D16" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E16" s="93" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F16" s="116"/>
       <c r="G16" s="107"/>
@@ -8598,16 +8821,16 @@
     </row>
     <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="88" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C17" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D17" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E17" s="93" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F17" s="116"/>
       <c r="G17" s="91"/>
@@ -8616,16 +8839,16 @@
     </row>
     <row r="18" spans="2:9" ht="27" x14ac:dyDescent="0.3">
       <c r="B18" s="88" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C18" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D18" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E18" s="102" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F18" s="116"/>
       <c r="G18" s="107"/>
@@ -8634,16 +8857,16 @@
     </row>
     <row r="19" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="87" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C19" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D19" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E19" s="93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F19" s="116"/>
       <c r="G19" s="106"/>
@@ -8652,16 +8875,16 @@
     </row>
     <row r="20" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="87" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C20" s="119" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D20" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E20" s="115" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F20" s="116"/>
       <c r="G20" s="112"/>
@@ -8670,16 +8893,16 @@
     </row>
     <row r="21" spans="2:9" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="89" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C21" s="120" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D21" s="120" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E21" s="105" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F21" s="117"/>
       <c r="G21" s="108"/>
@@ -8719,7 +8942,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="111" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C1" s="111"/>
       <c r="D1" s="111"/>
@@ -8730,16 +8953,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="172" t="s">
+        <v>176</v>
+      </c>
+      <c r="D2" s="172" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="172" t="s">
-        <v>178</v>
-      </c>
       <c r="E2" s="170" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F2" s="166" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G2" s="166"/>
       <c r="H2" s="166"/>
@@ -8751,30 +8974,30 @@
       <c r="D3" s="173"/>
       <c r="E3" s="171"/>
       <c r="F3" s="99" t="s">
-        <v>295</v>
+        <v>280</v>
       </c>
       <c r="G3" s="99" t="s">
-        <v>271</v>
+        <v>301</v>
       </c>
       <c r="H3" s="99" t="s">
-        <v>272</v>
+        <v>300</v>
       </c>
       <c r="I3" s="100" t="s">
-        <v>273</v>
+        <v>299</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="153" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C4" s="118" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D4" s="118" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E4" s="142" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F4" s="143"/>
       <c r="G4" s="144"/>
@@ -8783,98 +9006,98 @@
     </row>
     <row r="5" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
       <c r="B5" s="156" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C5" s="119" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="D5" s="119" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E5" s="102" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F5" s="116"/>
       <c r="G5" s="107"/>
       <c r="H5" s="125" t="s">
-        <v>314</v>
+        <v>294</v>
       </c>
       <c r="I5" s="137" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="154" t="s">
-        <v>292</v>
+        <v>278</v>
       </c>
       <c r="C6" s="119" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="D6" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E6" s="102" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F6" s="125"/>
       <c r="G6" s="125"/>
       <c r="H6" s="135" t="s">
-        <v>313</v>
+        <v>293</v>
       </c>
       <c r="I6" s="158"/>
     </row>
     <row r="7" spans="1:9" ht="93" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="154" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C7" s="119" t="s">
-        <v>286</v>
+        <v>272</v>
       </c>
       <c r="D7" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E7" s="102" t="s">
-        <v>301</v>
+        <v>283</v>
       </c>
       <c r="F7" s="116"/>
       <c r="G7" s="107"/>
       <c r="H7" s="91"/>
       <c r="I7" s="136" t="s">
-        <v>316</v>
+        <v>296</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="87.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="154" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C8" s="119" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="D8" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E8" s="102" t="s">
-        <v>300</v>
+        <v>282</v>
       </c>
       <c r="F8" s="116"/>
       <c r="G8" s="106"/>
       <c r="H8" s="91"/>
       <c r="I8" s="136" t="s">
-        <v>317</v>
+        <v>297</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="155" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C9" s="119" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="D9" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E9" s="93" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F9" s="116"/>
       <c r="G9" s="107"/>
@@ -8883,16 +9106,16 @@
     </row>
     <row r="10" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="155" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C10" s="119" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="D10" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E10" s="93" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F10" s="116"/>
       <c r="G10" s="107"/>
@@ -8901,16 +9124,16 @@
     </row>
     <row r="11" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="155" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C11" s="119" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="D11" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E11" s="93" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F11" s="116"/>
       <c r="G11" s="107"/>
@@ -8919,16 +9142,16 @@
     </row>
     <row r="12" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="155" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C12" s="119" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="D12" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E12" s="93" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F12" s="116"/>
       <c r="G12" s="107"/>
@@ -8937,128 +9160,128 @@
     </row>
     <row r="13" spans="1:9" ht="222" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="134" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C13" s="119" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
       <c r="D13" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E13" s="102" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F13" s="116"/>
       <c r="G13" s="107"/>
       <c r="H13" s="135" t="s">
-        <v>307</v>
+        <v>289</v>
       </c>
       <c r="I13" s="136" t="s">
-        <v>318</v>
+        <v>298</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
       <c r="B14" s="133" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C14" s="119" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
       <c r="D14" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E14" s="102" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F14" s="116"/>
       <c r="G14" s="107"/>
       <c r="H14" s="135" t="s">
-        <v>304</v>
+        <v>286</v>
       </c>
       <c r="I14" s="136" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
       <c r="B15" s="133" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C15" s="119" t="s">
-        <v>288</v>
+        <v>274</v>
       </c>
       <c r="D15" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E15" s="102" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F15" s="116"/>
       <c r="G15" s="135" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H15" s="139" t="s">
-        <v>305</v>
-      </c>
-      <c r="I15" s="136" t="s">
-        <v>308</v>
+        <v>287</v>
+      </c>
+      <c r="I15" s="177" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="228.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="133" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C16" s="119" t="s">
-        <v>289</v>
+        <v>275</v>
       </c>
       <c r="D16" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E16" s="102" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F16" s="116"/>
       <c r="G16" s="107"/>
       <c r="H16" s="135" t="s">
-        <v>310</v>
+        <v>291</v>
       </c>
       <c r="I16" s="136" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="132" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C17" s="119" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
       <c r="D17" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E17" s="115" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F17" s="116"/>
       <c r="G17" s="131" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="H17" s="157" t="s">
-        <v>303</v>
+        <v>285</v>
       </c>
       <c r="I17" s="138"/>
     </row>
     <row r="18" spans="2:9" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="133" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C18" s="119" t="s">
-        <v>290</v>
+        <v>276</v>
       </c>
       <c r="D18" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E18" s="115" t="s">
-        <v>299</v>
+        <v>281</v>
       </c>
       <c r="F18" s="116"/>
       <c r="G18" s="131"/>
@@ -9070,41 +9293,41 @@
         <v>3</v>
       </c>
       <c r="C19" s="141" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
       <c r="D19" s="141" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E19" s="93" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F19" s="116"/>
       <c r="G19" s="135" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="H19" s="135" t="s">
-        <v>306</v>
+        <v>288</v>
       </c>
       <c r="I19" s="136" t="s">
-        <v>309</v>
+        <v>290</v>
       </c>
     </row>
     <row r="20" spans="2:9" ht="14.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="145" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C20" s="146" t="s">
-        <v>291</v>
+        <v>277</v>
       </c>
       <c r="D20" s="146" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E20" s="147" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F20" s="148"/>
       <c r="G20" s="149" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="H20" s="150"/>
       <c r="I20" s="151"/>
@@ -9142,7 +9365,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="111" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C1" s="111"/>
       <c r="D1" s="111"/>
@@ -9153,16 +9376,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="172" t="s">
+        <v>176</v>
+      </c>
+      <c r="D2" s="172" t="s">
         <v>177</v>
       </c>
-      <c r="D2" s="172" t="s">
-        <v>178</v>
-      </c>
       <c r="E2" s="170" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F2" s="166" t="s">
-        <v>293</v>
+        <v>279</v>
       </c>
       <c r="G2" s="166"/>
       <c r="H2" s="166"/>
@@ -9174,70 +9397,68 @@
       <c r="D3" s="173"/>
       <c r="E3" s="171"/>
       <c r="F3" s="99" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="G3" s="99" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="H3" s="99" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="I3" s="100" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="153" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C4" s="118" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D4" s="118" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E4" s="142" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F4" s="143"/>
       <c r="G4" s="144"/>
       <c r="H4" s="90"/>
       <c r="I4" s="94"/>
     </row>
-    <row r="5" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
       <c r="B5" s="156" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C5" s="119" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="D5" s="119" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E5" s="102" t="s">
-        <v>162</v>
-      </c>
-      <c r="F5" s="116"/>
-      <c r="G5" s="107"/>
-      <c r="H5" s="125" t="s">
-        <v>281</v>
-      </c>
-      <c r="I5" s="137" t="s">
-        <v>280</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="F5" s="125" t="s">
+        <v>306</v>
+      </c>
+      <c r="G5" s="174"/>
+      <c r="H5" s="125"/>
+      <c r="I5" s="137"/>
     </row>
     <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="154" t="s">
-        <v>292</v>
+        <v>278</v>
       </c>
       <c r="C6" s="119" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="D6" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E6" s="102" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F6" s="125"/>
       <c r="G6" s="125"/>
@@ -9246,16 +9467,16 @@
     </row>
     <row r="7" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="154" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C7" s="119" t="s">
-        <v>286</v>
+        <v>272</v>
       </c>
       <c r="D7" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E7" s="102" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F7" s="116"/>
       <c r="G7" s="107"/>
@@ -9264,16 +9485,16 @@
     </row>
     <row r="8" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="154" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C8" s="119" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="D8" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E8" s="93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F8" s="116"/>
       <c r="G8" s="106"/>
@@ -9282,16 +9503,16 @@
     </row>
     <row r="9" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="155" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C9" s="119" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="D9" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E9" s="93" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F9" s="116"/>
       <c r="G9" s="107"/>
@@ -9300,16 +9521,16 @@
     </row>
     <row r="10" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="155" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C10" s="119" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="D10" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E10" s="93" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F10" s="116"/>
       <c r="G10" s="107"/>
@@ -9318,16 +9539,16 @@
     </row>
     <row r="11" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="155" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C11" s="119" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="D11" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E11" s="93" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F11" s="116"/>
       <c r="G11" s="107"/>
@@ -9336,184 +9557,170 @@
     </row>
     <row r="12" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="155" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C12" s="119" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="D12" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E12" s="93" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F12" s="116"/>
       <c r="G12" s="107"/>
       <c r="H12" s="140"/>
       <c r="I12" s="95"/>
     </row>
-    <row r="13" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="94.5" x14ac:dyDescent="0.3">
       <c r="B13" s="134" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C13" s="119" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
       <c r="D13" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E13" s="102" t="s">
+        <v>263</v>
+      </c>
+      <c r="F13" s="135" t="s">
+        <v>315</v>
+      </c>
+      <c r="G13" s="174"/>
+      <c r="H13" s="135"/>
+      <c r="I13" s="136"/>
+    </row>
+    <row r="14" spans="1:9" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="B14" s="133" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="119" t="s">
+        <v>273</v>
+      </c>
+      <c r="D14" s="119" t="s">
+        <v>178</v>
+      </c>
+      <c r="E14" s="102" t="s">
         <v>264</v>
       </c>
-      <c r="F13" s="116"/>
-      <c r="G13" s="107"/>
-      <c r="H13" s="135" t="s">
-        <v>277</v>
-      </c>
-      <c r="I13" s="136" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="133" t="s">
-        <v>74</v>
-      </c>
-      <c r="C14" s="119" t="s">
-        <v>287</v>
-      </c>
-      <c r="D14" s="119" t="s">
-        <v>179</v>
-      </c>
-      <c r="E14" s="102" t="s">
-        <v>265</v>
-      </c>
-      <c r="F14" s="116"/>
-      <c r="G14" s="107"/>
-      <c r="H14" s="135" t="s">
-        <v>279</v>
-      </c>
-      <c r="I14" s="136" t="s">
-        <v>278</v>
-      </c>
+      <c r="F14" s="135" t="s">
+        <v>309</v>
+      </c>
+      <c r="G14" s="174"/>
+      <c r="H14" s="135"/>
+      <c r="I14" s="136"/>
     </row>
     <row r="15" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
       <c r="B15" s="133" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C15" s="119" t="s">
-        <v>288</v>
+        <v>274</v>
       </c>
       <c r="D15" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E15" s="102" t="s">
-        <v>263</v>
-      </c>
-      <c r="F15" s="116"/>
-      <c r="G15" s="135" t="s">
-        <v>269</v>
-      </c>
-      <c r="H15" s="139" t="s">
+        <v>262</v>
+      </c>
+      <c r="F15" s="135" t="s">
+        <v>310</v>
+      </c>
+      <c r="G15" s="175"/>
+      <c r="H15" s="139"/>
+      <c r="I15" s="136"/>
+    </row>
+    <row r="16" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
+      <c r="B16" s="133" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" s="119" t="s">
         <v>275</v>
       </c>
-      <c r="I15" s="136" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="81" x14ac:dyDescent="0.3">
-      <c r="B16" s="133" t="s">
-        <v>86</v>
-      </c>
-      <c r="C16" s="119" t="s">
-        <v>289</v>
-      </c>
       <c r="D16" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E16" s="102" t="s">
-        <v>266</v>
-      </c>
-      <c r="F16" s="116"/>
-      <c r="G16" s="107"/>
-      <c r="H16" s="135" t="s">
-        <v>282</v>
-      </c>
+        <v>265</v>
+      </c>
+      <c r="F16" s="135" t="s">
+        <v>312</v>
+      </c>
+      <c r="G16" s="174"/>
+      <c r="H16" s="135"/>
       <c r="I16" s="136"/>
     </row>
     <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="132" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C17" s="119" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
       <c r="D17" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E17" s="115" t="s">
-        <v>270</v>
-      </c>
-      <c r="F17" s="116"/>
-      <c r="G17" s="131" t="s">
-        <v>261</v>
-      </c>
-      <c r="H17" s="139" t="s">
-        <v>283</v>
-      </c>
+        <v>269</v>
+      </c>
+      <c r="F17" s="157"/>
+      <c r="G17" s="176"/>
+      <c r="H17" s="139"/>
       <c r="I17" s="138"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B18" s="133" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C18" s="119" t="s">
-        <v>290</v>
+        <v>276</v>
       </c>
       <c r="D18" s="119" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E18" s="115"/>
-      <c r="F18" s="116"/>
-      <c r="G18" s="131"/>
+      <c r="F18" s="157"/>
+      <c r="G18" s="176"/>
       <c r="H18" s="139"/>
       <c r="I18" s="138"/>
     </row>
-    <row r="19" spans="2:9" ht="108" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:9" ht="54" x14ac:dyDescent="0.3">
       <c r="B19" s="152" t="s">
         <v>3</v>
       </c>
       <c r="C19" s="141" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
       <c r="D19" s="141" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E19" s="93" t="s">
-        <v>157</v>
-      </c>
-      <c r="F19" s="116"/>
-      <c r="G19" s="135" t="s">
-        <v>268</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="F19" s="135" t="s">
+        <v>290</v>
+      </c>
+      <c r="G19" s="175"/>
       <c r="I19" s="95"/>
     </row>
     <row r="20" spans="2:9" ht="14.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="145" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C20" s="146" t="s">
-        <v>291</v>
+        <v>277</v>
       </c>
       <c r="D20" s="146" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E20" s="147" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F20" s="148"/>
-      <c r="G20" s="149" t="s">
-        <v>267</v>
-      </c>
+      <c r="G20" s="149"/>
       <c r="H20" s="150"/>
       <c r="I20" s="151"/>
     </row>
@@ -9527,5 +9734,6 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly Plan 내용 수정 완료
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="318">
   <si>
     <t>■</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2422,24 +2422,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>[임제훈 사원]
-- CPU 및 메모리 부하율 관리 대책 르네사스 문의 (~10/27)
-- 사이버 보안 항목 QV와 비교 및 리스트업 후 공조시스템설계팀 회신 (~10/29)
-- 제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 후 자료 회신 (~10/29)
-  : 1. P2 단계 전까지 매 월 1회 제어기 검증 현황 관련 회의 진행 예정
-    2. 진행 단계 별로 이력 및 변경점 꾸준히 업데이트 해서 자료 회신 요청
-    3. Fail Safety 항목 공유 요청
-    4. 제어기 검증 프로세스 관련 자료 공유 요청
-    5. 컨버전 룰이 무엇인지에 대한 자료 공유 요청
-    6. S/W 검증 현황의 검증 항목별 LIST 자료 공유 요청
-    7. CPU / 메모리 부하율 관리 방안 재확인 요청
-    8. 고장 진단 로그 저장 가능 개수 재확인 요청
-- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/31)
-- 설계 변경 진행 (~11/10)
-  : 기구팀 문의 결과, QV, SVm, BJ 담당자 전부 똑같다고 함. 결재 라인 똑같이 예정</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>4주차 (10/24 ~ 10/30)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -2505,142 +2487,6 @@
   : SW 대응은 딱히 없을 것 같다고 했지만, 결과나 진행 사항 파악 필요
 - LHD R로직 튜닝
 - RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">[임제훈 사원]
-- </t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>R로직 튜닝 (~10/27)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-- </t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>ESIR 일정에 맞춰서 5가지 항목 다 가능한지 파악하기 (~10/29)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-- 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (10/30)
-  : 휴가 중, 목요일 출근 예정, 이 때 메일로 다시 문의
-- </t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>ES 규격 대로 15초 내로 목표 전력 도달 SW로 변경 (~10/29)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-  : Softstart enable 0으로 변경
-  : Sofftstart 0일 때, R로직 확인, 전력 구간 별 칼로리와 CAN 출력 차이 비교
-- ESIR 계획서 등록 (~10/31)
-- </t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/31)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-- 최신 승인도 확인 (~10/31)
-- </t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>제작사양서 배포 준비 (~10/31)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-  : SW 파일, 제어사양서
-  : 10월 14일부터 tc 160℃, 스톤 기울기 변경되었음
-  : 제작사양서 배포 기준, tc 160℃ 스톤 기울기 변경된 샘플 기준으로 튜닝 완료
-  : P1 때 tc 165℃ 변경 협의 중</t>
     </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -2718,14 +2564,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>[임제훈 사원]
-- 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (~11/03)
-  : 10/30 문의 완료, 재회신 요청 예정
-- ESIR 계획서 등록 (~11/05)
-- 최신 승인도 확인 (~11/06)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>[우리산업]
 PM : 유정호, 품질 : 박상철, 기구 : 김민수, 공준석, HW : 신지훈
 [전자편의개발 2팀] 
@@ -2755,10 +2593,267 @@
     <t>[임제훈 사원]
 - 사이버 보안 항목 QV와 비교 및 리스트업 후 공조시스템설계팀 회신 (~11/05)
   : ES95489-21 빼는 것은 안됨. 업데이트에 해당하는 항목 N/A로 하자고 회신 받음
-- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~11/03)
+- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~11/05)
 - 설계 변경 진행 (~11/10)
   : 기구팀 문의 결과, QV, SVm, BJ 담당자 전부 똑같다고 함. 결재 라인 똑같이 예정
   : 설계 변경 문서 작성</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SU2i CARRY OVER
+Proto (진행 중)
+P1 (26/05/15)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[임제훈 사원]
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>R로직 튜닝 (~10/27)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ESIR 일정에 맞춰서 5가지 항목 다 가능한지 파악하기 (~10/29)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ES 규격 대로 15초 내로 목표 전력 도달 SW로 변경 (~10/29)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  : Softstart enable 0으로 변경
+  : Sofftstart 0일 때, R로직 확인, 전력 구간 별 칼로리와 CAN 출력 차이 비교</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/31)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>제작사양서 배포 준비 (~10/31)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  : SW 파일, 제어사양서
+  : 10월 14일부터 tc 160℃, 스톤 기울기 변경되었음
+  : 제작사양서 배포 기준, tc 160℃ 스톤 기울기 변경된 샘플 기준으로 튜닝 완료
+  : P1 때 tc 165℃ 변경 협의 중
+- 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (10/30)
+  : 휴가 중, 목요일 출근 예정, 이 때 메일로 다시 문의
+- ESIR 계획서 등록 (~10/31)
+- 최신 승인도 확인 (~10/31)</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[임제훈 사원]
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CPU 및 메모리 부하율 관리 대책 르네사스 문의 (~10/27)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>사이버 보안 항목 QV와 비교 및 리스트업 후 공조시스템설계팀 회신 (~10/29)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>제어기 선행품질 검증 현황 관련 기아 오토랜드 방문 후 자료 회신 (~10/29)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  : 1. P2 단계 전까지 매 월 1회 제어기 검증 현황 관련 회의 진행 예정
+    2. 진행 단계 별로 이력 및 변경점 꾸준히 업데이트 해서 자료 회신 요청
+    3. Fail Safety 항목 공유 요청
+    4. 제어기 검증 프로세스 관련 자료 공유 요청
+    5. 컨버전 룰이 무엇인지에 대한 자료 공유 요청
+    6. S/W 검증 현황의 검증 항목별 LIST 자료 공유 요청
+    7. CPU / 메모리 부하율 관리 방안 재확인 요청
+    8. 고장 진단 로그 저장 가능 개수 재확인 요청
+- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~10/31)
+- 설계 변경 진행 (~11/10)
+  : 기구팀 문의 결과, QV, SVm, BJ 담당자 전부 똑같다고 함. 결재 라인 똑같이 예정</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- PTC 벤치 테스트 한온에서 진행 (11/12)
+  : BJ RHD HVAC 수령 예정</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (11/03)
+  : 일정 조율에 대한 사유 작성하여 재회신 예정, 조건부 승인으로 가면 된다고 함
+  : 사이버 보안팀에 시료 제출하여 선 공정 검사 진행 여부는 확인 해본다고 함
+- ESIR 계획서 등록 (~11/05)
+- 최신 승인도 확인 (~11/06)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2993,7 +3088,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="83">
+  <borders count="82">
     <border>
       <left/>
       <right/>
@@ -4118,15 +4213,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="hair">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -4148,7 +4234,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="179">
+  <cellXfs count="178">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -4626,6 +4712,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="80" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="81" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="81" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4670,21 +4768,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="81" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="81" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -5308,90 +5391,90 @@
       <c r="D1" s="21"/>
     </row>
     <row r="2" spans="1:64" ht="31.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="159" t="s">
+      <c r="B2" s="163" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="161" t="s">
+      <c r="C2" s="165" t="s">
         <v>76</v>
       </c>
-      <c r="D2" s="161" t="s">
+      <c r="D2" s="165" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="165">
+      <c r="E2" s="169">
         <v>23</v>
       </c>
-      <c r="F2" s="163"/>
-      <c r="G2" s="163"/>
-      <c r="H2" s="163"/>
-      <c r="I2" s="163"/>
-      <c r="J2" s="163"/>
-      <c r="K2" s="163"/>
-      <c r="L2" s="163"/>
-      <c r="M2" s="163"/>
-      <c r="N2" s="163"/>
-      <c r="O2" s="163"/>
-      <c r="P2" s="163"/>
-      <c r="Q2" s="163">
+      <c r="F2" s="167"/>
+      <c r="G2" s="167"/>
+      <c r="H2" s="167"/>
+      <c r="I2" s="167"/>
+      <c r="J2" s="167"/>
+      <c r="K2" s="167"/>
+      <c r="L2" s="167"/>
+      <c r="M2" s="167"/>
+      <c r="N2" s="167"/>
+      <c r="O2" s="167"/>
+      <c r="P2" s="167"/>
+      <c r="Q2" s="167">
         <v>24</v>
       </c>
-      <c r="R2" s="163"/>
-      <c r="S2" s="163"/>
-      <c r="T2" s="163"/>
-      <c r="U2" s="163"/>
-      <c r="V2" s="163"/>
-      <c r="W2" s="163"/>
-      <c r="X2" s="163"/>
-      <c r="Y2" s="163"/>
-      <c r="Z2" s="163"/>
-      <c r="AA2" s="163"/>
-      <c r="AB2" s="163"/>
-      <c r="AC2" s="163">
+      <c r="R2" s="167"/>
+      <c r="S2" s="167"/>
+      <c r="T2" s="167"/>
+      <c r="U2" s="167"/>
+      <c r="V2" s="167"/>
+      <c r="W2" s="167"/>
+      <c r="X2" s="167"/>
+      <c r="Y2" s="167"/>
+      <c r="Z2" s="167"/>
+      <c r="AA2" s="167"/>
+      <c r="AB2" s="167"/>
+      <c r="AC2" s="167">
         <v>25</v>
       </c>
-      <c r="AD2" s="163"/>
-      <c r="AE2" s="163"/>
-      <c r="AF2" s="163"/>
-      <c r="AG2" s="163"/>
-      <c r="AH2" s="163"/>
-      <c r="AI2" s="163"/>
-      <c r="AJ2" s="163"/>
-      <c r="AK2" s="163"/>
-      <c r="AL2" s="163"/>
-      <c r="AM2" s="163"/>
-      <c r="AN2" s="163"/>
-      <c r="AO2" s="163">
+      <c r="AD2" s="167"/>
+      <c r="AE2" s="167"/>
+      <c r="AF2" s="167"/>
+      <c r="AG2" s="167"/>
+      <c r="AH2" s="167"/>
+      <c r="AI2" s="167"/>
+      <c r="AJ2" s="167"/>
+      <c r="AK2" s="167"/>
+      <c r="AL2" s="167"/>
+      <c r="AM2" s="167"/>
+      <c r="AN2" s="167"/>
+      <c r="AO2" s="167">
         <v>26</v>
       </c>
-      <c r="AP2" s="163"/>
-      <c r="AQ2" s="163"/>
-      <c r="AR2" s="163"/>
-      <c r="AS2" s="163"/>
-      <c r="AT2" s="163"/>
-      <c r="AU2" s="163"/>
-      <c r="AV2" s="163"/>
-      <c r="AW2" s="163"/>
-      <c r="AX2" s="163"/>
-      <c r="AY2" s="163"/>
-      <c r="AZ2" s="164"/>
-      <c r="BA2" s="163">
+      <c r="AP2" s="167"/>
+      <c r="AQ2" s="167"/>
+      <c r="AR2" s="167"/>
+      <c r="AS2" s="167"/>
+      <c r="AT2" s="167"/>
+      <c r="AU2" s="167"/>
+      <c r="AV2" s="167"/>
+      <c r="AW2" s="167"/>
+      <c r="AX2" s="167"/>
+      <c r="AY2" s="167"/>
+      <c r="AZ2" s="168"/>
+      <c r="BA2" s="167">
         <v>27</v>
       </c>
-      <c r="BB2" s="163"/>
-      <c r="BC2" s="163"/>
-      <c r="BD2" s="163"/>
-      <c r="BE2" s="163"/>
-      <c r="BF2" s="163"/>
-      <c r="BG2" s="163"/>
-      <c r="BH2" s="163"/>
-      <c r="BI2" s="163"/>
-      <c r="BJ2" s="163"/>
-      <c r="BK2" s="163"/>
-      <c r="BL2" s="164"/>
+      <c r="BB2" s="167"/>
+      <c r="BC2" s="167"/>
+      <c r="BD2" s="167"/>
+      <c r="BE2" s="167"/>
+      <c r="BF2" s="167"/>
+      <c r="BG2" s="167"/>
+      <c r="BH2" s="167"/>
+      <c r="BI2" s="167"/>
+      <c r="BJ2" s="167"/>
+      <c r="BK2" s="167"/>
+      <c r="BL2" s="168"/>
     </row>
     <row r="3" spans="1:64" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="160"/>
-      <c r="C3" s="162"/>
-      <c r="D3" s="162"/>
+      <c r="B3" s="164"/>
+      <c r="C3" s="166"/>
+      <c r="D3" s="166"/>
       <c r="E3" s="22">
         <v>1</v>
       </c>
@@ -6292,7 +6375,7 @@
         <v>82</v>
       </c>
       <c r="D13" s="34" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="E13" s="6"/>
       <c r="F13" s="7"/>
@@ -6728,8 +6811,8 @@
       <c r="C18" s="59" t="s">
         <v>258</v>
       </c>
-      <c r="D18" s="178" t="s">
-        <v>314</v>
+      <c r="D18" s="162" t="s">
+        <v>311</v>
       </c>
       <c r="E18" s="64"/>
       <c r="F18" s="65"/>
@@ -7366,39 +7449,39 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="172" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="172" t="s">
+      <c r="C2" s="176" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="172" t="s">
+      <c r="D2" s="176" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="170" t="s">
+      <c r="E2" s="174" t="s">
         <v>126</v>
       </c>
       <c r="F2" s="98" t="s">
         <v>112</v>
       </c>
-      <c r="G2" s="166" t="s">
+      <c r="G2" s="170" t="s">
         <v>113</v>
       </c>
-      <c r="H2" s="166"/>
-      <c r="I2" s="166"/>
-      <c r="J2" s="167"/>
-      <c r="K2" s="166" t="s">
+      <c r="H2" s="170"/>
+      <c r="I2" s="170"/>
+      <c r="J2" s="171"/>
+      <c r="K2" s="170" t="s">
         <v>182</v>
       </c>
-      <c r="L2" s="166"/>
-      <c r="M2" s="166"/>
-      <c r="N2" s="167"/>
+      <c r="L2" s="170"/>
+      <c r="M2" s="170"/>
+      <c r="N2" s="171"/>
     </row>
     <row r="3" spans="1:14" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="169"/>
-      <c r="C3" s="173"/>
-      <c r="D3" s="173"/>
-      <c r="E3" s="171"/>
+      <c r="B3" s="173"/>
+      <c r="C3" s="177"/>
+      <c r="D3" s="177"/>
+      <c r="E3" s="175"/>
       <c r="F3" s="99" t="s">
         <v>111</v>
       </c>
@@ -8141,30 +8224,30 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="172" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="172" t="s">
+      <c r="C2" s="176" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="172" t="s">
+      <c r="D2" s="176" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="170" t="s">
+      <c r="E2" s="174" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="166" t="s">
+      <c r="F2" s="170" t="s">
         <v>182</v>
       </c>
-      <c r="G2" s="166"/>
-      <c r="H2" s="166"/>
-      <c r="I2" s="167"/>
+      <c r="G2" s="170"/>
+      <c r="H2" s="170"/>
+      <c r="I2" s="171"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="169"/>
-      <c r="C3" s="173"/>
-      <c r="D3" s="173"/>
-      <c r="E3" s="171"/>
+      <c r="B3" s="173"/>
+      <c r="C3" s="177"/>
+      <c r="D3" s="177"/>
+      <c r="E3" s="175"/>
       <c r="F3" s="99" t="s">
         <v>114</v>
       </c>
@@ -8542,30 +8625,30 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="172" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="172" t="s">
+      <c r="C2" s="176" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="172" t="s">
+      <c r="D2" s="176" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="170" t="s">
+      <c r="E2" s="174" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="166" t="s">
+      <c r="F2" s="170" t="s">
         <v>227</v>
       </c>
-      <c r="G2" s="166"/>
-      <c r="H2" s="166"/>
-      <c r="I2" s="167"/>
+      <c r="G2" s="170"/>
+      <c r="H2" s="170"/>
+      <c r="I2" s="171"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="169"/>
-      <c r="C3" s="173"/>
-      <c r="D3" s="173"/>
-      <c r="E3" s="171"/>
+      <c r="B3" s="173"/>
+      <c r="C3" s="177"/>
+      <c r="D3" s="177"/>
+      <c r="E3" s="175"/>
       <c r="F3" s="99" t="s">
         <v>114</v>
       </c>
@@ -8949,41 +9032,41 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="172" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="172" t="s">
+      <c r="C2" s="176" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="172" t="s">
+      <c r="D2" s="176" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="170" t="s">
+      <c r="E2" s="174" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="166" t="s">
+      <c r="F2" s="170" t="s">
         <v>259</v>
       </c>
-      <c r="G2" s="166"/>
-      <c r="H2" s="166"/>
-      <c r="I2" s="167"/>
+      <c r="G2" s="170"/>
+      <c r="H2" s="170"/>
+      <c r="I2" s="171"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="169"/>
-      <c r="C3" s="173"/>
-      <c r="D3" s="173"/>
-      <c r="E3" s="171"/>
+      <c r="B3" s="173"/>
+      <c r="C3" s="177"/>
+      <c r="D3" s="177"/>
+      <c r="E3" s="175"/>
       <c r="F3" s="99" t="s">
         <v>280</v>
       </c>
       <c r="G3" s="99" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H3" s="99" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I3" s="100" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -9177,7 +9260,7 @@
         <v>289</v>
       </c>
       <c r="I13" s="136" t="s">
-        <v>298</v>
+        <v>315</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
@@ -9199,7 +9282,7 @@
         <v>286</v>
       </c>
       <c r="I14" s="136" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
@@ -9222,8 +9305,8 @@
       <c r="H15" s="139" t="s">
         <v>287</v>
       </c>
-      <c r="I15" s="177" t="s">
-        <v>311</v>
+      <c r="I15" s="161" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="228.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -9245,7 +9328,7 @@
         <v>291</v>
       </c>
       <c r="I16" s="136" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -9372,41 +9455,41 @@
       <c r="E1" s="109"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="172" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="172" t="s">
+      <c r="C2" s="176" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="172" t="s">
+      <c r="D2" s="176" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="170" t="s">
+      <c r="E2" s="174" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="166" t="s">
+      <c r="F2" s="170" t="s">
         <v>279</v>
       </c>
-      <c r="G2" s="166"/>
-      <c r="H2" s="166"/>
-      <c r="I2" s="167"/>
+      <c r="G2" s="170"/>
+      <c r="H2" s="170"/>
+      <c r="I2" s="171"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="169"/>
-      <c r="C3" s="173"/>
-      <c r="D3" s="173"/>
-      <c r="E3" s="171"/>
+      <c r="B3" s="173"/>
+      <c r="C3" s="177"/>
+      <c r="D3" s="177"/>
+      <c r="E3" s="175"/>
       <c r="F3" s="99" t="s">
+        <v>301</v>
+      </c>
+      <c r="G3" s="99" t="s">
         <v>302</v>
       </c>
-      <c r="G3" s="99" t="s">
+      <c r="H3" s="99" t="s">
         <v>303</v>
       </c>
-      <c r="H3" s="99" t="s">
+      <c r="I3" s="100" t="s">
         <v>304</v>
-      </c>
-      <c r="I3" s="100" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -9441,9 +9524,9 @@
         <v>161</v>
       </c>
       <c r="F5" s="125" t="s">
-        <v>306</v>
-      </c>
-      <c r="G5" s="174"/>
+        <v>305</v>
+      </c>
+      <c r="G5" s="159"/>
       <c r="H5" s="125"/>
       <c r="I5" s="137"/>
     </row>
@@ -9587,9 +9670,9 @@
         <v>263</v>
       </c>
       <c r="F13" s="135" t="s">
-        <v>315</v>
-      </c>
-      <c r="G13" s="174"/>
+        <v>312</v>
+      </c>
+      <c r="G13" s="159"/>
       <c r="H13" s="135"/>
       <c r="I13" s="136"/>
     </row>
@@ -9607,9 +9690,11 @@
         <v>264</v>
       </c>
       <c r="F14" s="135" t="s">
-        <v>309</v>
-      </c>
-      <c r="G14" s="174"/>
+        <v>307</v>
+      </c>
+      <c r="G14" s="159" t="s">
+        <v>316</v>
+      </c>
       <c r="H14" s="135"/>
       <c r="I14" s="136"/>
     </row>
@@ -9627,13 +9712,13 @@
         <v>262</v>
       </c>
       <c r="F15" s="135" t="s">
-        <v>310</v>
-      </c>
-      <c r="G15" s="175"/>
+        <v>308</v>
+      </c>
+      <c r="G15" s="160"/>
       <c r="H15" s="139"/>
       <c r="I15" s="136"/>
     </row>
-    <row r="16" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="81" x14ac:dyDescent="0.3">
       <c r="B16" s="133" t="s">
         <v>85</v>
       </c>
@@ -9647,9 +9732,9 @@
         <v>265</v>
       </c>
       <c r="F16" s="135" t="s">
-        <v>312</v>
-      </c>
-      <c r="G16" s="174"/>
+        <v>317</v>
+      </c>
+      <c r="G16" s="159"/>
       <c r="H16" s="135"/>
       <c r="I16" s="136"/>
     </row>
@@ -9664,10 +9749,10 @@
         <v>178</v>
       </c>
       <c r="E17" s="115" t="s">
-        <v>269</v>
+        <v>313</v>
       </c>
       <c r="F17" s="157"/>
-      <c r="G17" s="176"/>
+      <c r="G17" s="157"/>
       <c r="H17" s="139"/>
       <c r="I17" s="138"/>
     </row>
@@ -9683,7 +9768,7 @@
       </c>
       <c r="E18" s="115"/>
       <c r="F18" s="157"/>
-      <c r="G18" s="176"/>
+      <c r="G18" s="135"/>
       <c r="H18" s="139"/>
       <c r="I18" s="138"/>
     </row>
@@ -9703,7 +9788,7 @@
       <c r="F19" s="135" t="s">
         <v>290</v>
       </c>
-      <c r="G19" s="175"/>
+      <c r="G19" s="160"/>
       <c r="I19" s="95"/>
     </row>
     <row r="20" spans="2:9" ht="14.25" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
1. weekly plan update
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\일정\ptc_heater_doc\1. 일정\1. Weekly Plan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\PROJECT\Gitlab\HMC\ptc_heater_doc\1. 일정\1. Weekly Plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="323">
   <si>
     <t>■</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2492,12 +2492,6 @@
   </si>
   <si>
     <t>[임제훈 사원]
-- LHD R로직 튜닝
-- RHD R로직 튜닝 (HVAC 미보유, 보류)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
 - R로직 튜닝</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -2587,16 +2581,6 @@
 wjdworms1357@hyundai.com
 김동환 연구원 010-4162-2776
 kdh2776@hyundai.com</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
-- 사이버 보안 항목 QV와 비교 및 리스트업 후 공조시스템설계팀 회신 (~11/05)
-  : ES95489-21 빼는 것은 안됨. 업데이트에 해당하는 항목 N/A로 하자고 회신 받음
-- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~11/05)
-- 설계 변경 진행 (~11/10)
-  : 기구팀 문의 결과, QV, SVm, BJ 담당자 전부 똑같다고 함. 결재 라인 똑같이 예정
-  : 설계 변경 문서 작성</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -2843,12 +2827,6 @@
   </si>
   <si>
     <t>[임제훈 사원]
-- PTC 벤치 테스트 한온에서 진행 (11/12)
-  : BJ RHD HVAC 수령 예정</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[임제훈 사원]
 - 공조시스템설계팀 김동환 연구원 사이버보안 일정 재문의 (11/03)
   : 일정 조율에 대한 사유 작성하여 재회신 예정, 조건부 승인으로 가면 된다고 함
   : 사이버 보안팀에 시료 제출하여 선 공정 검사 진행 여부는 확인 해본다고 함
@@ -2873,6 +2851,50 @@
     <t>[임제훈 사원]
 - 공조 로컬 CAN 심의회 진행 (11/10)
   : SVm, BJ, NX5e, MX5a, HE1i 대상</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- LHD R로직 튜닝
+- RHD R로직 튜닝 (HVAC 미보유, 보류)
+[김진겸 사원]
+- RHD R 로직 튜닝을 위한 HVAC 수령 대기 중
+  (11/12 기구팀 한온 출장 시 수령 예정)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- 사이버 보안 항목 QV와 비교 및 리스트업 후 공조시스템설계팀 회신 (~11/05)
+  : ES95489-21 빼는 것은 안됨. 업데이트에 해당하는 항목 N/A로 하자고 회신 받음
+- 제어사양서, 고장진단 사양, 로직검증 체크리스트 확인 및 갱신 (~11/05)
+- 설계 변경 진행 (~11/10)
+  : 기구팀 문의 결과, QV, SVm, BJ 담당자 전부 똑같다고 함. 결재 라인 똑같이 예정
+  : 설계 변경 문서 작성
+[김진겸 사원]
+- 설계변경 시 ERP 등록 준비(~11/10)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- 공조 로컬 CAN 심의회 진행 (11/10)
+  : SVm, BJ, NX5e, MX5a, HE1i 대상</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[김진겸 사원]
+- PROTO 차량 난방 평가 진행(10/31, 현대 남양연구소)
+- 난방 성능 불만족으로, 고객사 측에서 성능 증대 요청 중
+  (기구 대응 중, 김민수 선임)
+- 11/05~11/07 한온에서 동일 차량으로 평가 예정</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- PTC 벤치 테스트 한온에서 진행 (11/12)
+  : BJ RHD HVAC 수령 예정
+[김진겸 사원]
+- 열에너지차량시험팀 측에서 11/10(월) 챔버 확보
+  : 자동차 측에서 실차 튜닝 요청, 참석 인원 선정 필요</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -5123,6 +5145,49 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>2886076</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>1009650</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>4645520</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>1619250</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="그림 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9353551" y="4581525"/>
+          <a:ext cx="1759444" cy="609600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
   <a:themeElements>
@@ -6394,7 +6459,7 @@
         <v>82</v>
       </c>
       <c r="D13" s="34" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E13" s="6"/>
       <c r="F13" s="7"/>
@@ -6831,7 +6896,7 @@
         <v>258</v>
       </c>
       <c r="D18" s="162" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E18" s="64"/>
       <c r="F18" s="65"/>
@@ -9279,7 +9344,7 @@
         <v>289</v>
       </c>
       <c r="I13" s="136" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
@@ -9325,7 +9390,7 @@
         <v>287</v>
       </c>
       <c r="I15" s="161" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="228.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -9347,7 +9412,7 @@
         <v>291</v>
       </c>
       <c r="I16" s="136" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -9567,7 +9632,7 @@
       <c r="H6" s="125"/>
       <c r="I6" s="137"/>
     </row>
-    <row r="7" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="138" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="154" t="s">
         <v>75</v>
       </c>
@@ -9580,9 +9645,11 @@
       <c r="E7" s="102" t="s">
         <v>162</v>
       </c>
-      <c r="F7" s="116"/>
+      <c r="F7" s="125" t="s">
+        <v>321</v>
+      </c>
       <c r="G7" s="107" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="H7" s="91"/>
       <c r="I7" s="95"/>
@@ -9677,7 +9744,7 @@
       <c r="H12" s="140"/>
       <c r="I12" s="95"/>
     </row>
-    <row r="13" spans="1:9" ht="94.5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="135" x14ac:dyDescent="0.3">
       <c r="B13" s="134" t="s">
         <v>62</v>
       </c>
@@ -9691,7 +9758,7 @@
         <v>263</v>
       </c>
       <c r="F13" s="135" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="G13" s="159" t="s">
         <v>320</v>
@@ -9699,7 +9766,7 @@
       <c r="H13" s="135"/>
       <c r="I13" s="136"/>
     </row>
-    <row r="14" spans="1:9" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="94.5" x14ac:dyDescent="0.3">
       <c r="B14" s="133" t="s">
         <v>73</v>
       </c>
@@ -9713,10 +9780,10 @@
         <v>264</v>
       </c>
       <c r="F14" s="135" t="s">
-        <v>307</v>
+        <v>318</v>
       </c>
       <c r="G14" s="159" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="H14" s="135"/>
       <c r="I14" s="136"/>
@@ -9735,7 +9802,7 @@
         <v>262</v>
       </c>
       <c r="F15" s="135" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G15" s="160"/>
       <c r="H15" s="139"/>
@@ -9755,10 +9822,10 @@
         <v>265</v>
       </c>
       <c r="F16" s="135" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="G16" s="159" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="H16" s="135"/>
       <c r="I16" s="136"/>
@@ -9774,11 +9841,11 @@
         <v>178</v>
       </c>
       <c r="E17" s="115" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="F17" s="157"/>
       <c r="G17" s="121" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="H17" s="139"/>
       <c r="I17" s="138"/>
@@ -9847,5 +9914,6 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly Plan XV1 추가
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\일정\ptc_heater_doc\1. 일정\1. Weekly Plan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\001.Task\001.Woory\001.PTC\0.PTC\ptc_heater_doc\1. 일정\1. Weekly Plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7F9226E-15F0-451A-8FF0-B2CDE4AF76C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="8"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="대일정" sheetId="1" r:id="rId1"/>
@@ -23,17 +24,28 @@
     <sheet name="2026.1" sheetId="10" r:id="rId9"/>
     <sheet name="2026.2" sheetId="11" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1098" uniqueCount="441">
   <si>
     <t>■</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1699,17 +1711,6 @@
     <t>Proto (진행 중)
 P1 (26/04/01)
 P2 (26/10/01)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">[우리산업]
-PM : 유정호, 기구 : 공준석, HW : 신지훈, 
-제조 : 전진호, 품질 : 박상철, 일렉스 : 남시온, 류상근, 박철수, 슬로박법인 : 김예현
-[공조설계팀]
-안성민 책임연구원 010-2207-9180
-freshair@hyundai.com
-[신차 품질팀]
-</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -9630,11 +9631,68 @@
     - CAN DBC 파일 재요청</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>[조현진 전임]
+- LIN CheckList Application 제출 (1/30)
+- MCU 변경 (Renesas RH850 -&gt; ST STM8AF5288TCY)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[임제훈 사원]
+- SWE.3 SDDS 후속 작업 완료
+[조현진 전임]
+- SWE.4, SWE.5 후속 작업 완료</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>XV1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[우리산업]
+PM : 
+부품개발 :
+제조기술 :
+품질 : 
+기구 :
+[HKMC]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[우리산업]
+PM : 유정호 
+기구 : 공준석
+HW : 신지훈 
+제조 : 전진호
+품질 : 박상철
+일렉스 : 남시온, 류상근, 박철수
+슬로박법인 : 김예현
+[공조설계팀]
+안성민 책임연구원 010-2207-9180
+freshair@hyundai.com
+[신차 품질팀]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ALL출도
+5/31</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>통합P
+4/1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M
+9/1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="mm&quot;월&quot;\ dd&quot;일&quot;"/>
   </numFmts>
@@ -11625,6 +11683,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="88" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -11672,9 +11733,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="83" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -11751,15 +11809,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>39</xdr:col>
-      <xdr:colOff>283550</xdr:colOff>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>297157</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>39</xdr:col>
-      <xdr:colOff>313563</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>327170</xdr:colOff>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>176893</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -11775,8 +11833,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="13754621" y="0"/>
-          <a:ext cx="30013" cy="27350357"/>
+          <a:off x="15047300" y="0"/>
+          <a:ext cx="30013" cy="28003500"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -12352,8 +12410,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BL25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:BL26"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.375" customWidth="1"/>
@@ -12377,90 +12435,90 @@
       <c r="D1" s="21"/>
     </row>
     <row r="2" spans="1:64" ht="31.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="174" t="s">
+      <c r="B2" s="175" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="176" t="s">
+      <c r="C2" s="177" t="s">
         <v>76</v>
       </c>
-      <c r="D2" s="176" t="s">
+      <c r="D2" s="177" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="180">
+      <c r="E2" s="181">
         <v>23</v>
       </c>
-      <c r="F2" s="178"/>
-      <c r="G2" s="178"/>
-      <c r="H2" s="178"/>
-      <c r="I2" s="178"/>
-      <c r="J2" s="178"/>
-      <c r="K2" s="178"/>
-      <c r="L2" s="178"/>
-      <c r="M2" s="178"/>
-      <c r="N2" s="178"/>
-      <c r="O2" s="178"/>
-      <c r="P2" s="178"/>
-      <c r="Q2" s="178">
+      <c r="F2" s="179"/>
+      <c r="G2" s="179"/>
+      <c r="H2" s="179"/>
+      <c r="I2" s="179"/>
+      <c r="J2" s="179"/>
+      <c r="K2" s="179"/>
+      <c r="L2" s="179"/>
+      <c r="M2" s="179"/>
+      <c r="N2" s="179"/>
+      <c r="O2" s="179"/>
+      <c r="P2" s="179"/>
+      <c r="Q2" s="179">
         <v>24</v>
       </c>
-      <c r="R2" s="178"/>
-      <c r="S2" s="178"/>
-      <c r="T2" s="178"/>
-      <c r="U2" s="178"/>
-      <c r="V2" s="178"/>
-      <c r="W2" s="178"/>
-      <c r="X2" s="178"/>
-      <c r="Y2" s="178"/>
-      <c r="Z2" s="178"/>
-      <c r="AA2" s="178"/>
-      <c r="AB2" s="178"/>
-      <c r="AC2" s="178">
+      <c r="R2" s="179"/>
+      <c r="S2" s="179"/>
+      <c r="T2" s="179"/>
+      <c r="U2" s="179"/>
+      <c r="V2" s="179"/>
+      <c r="W2" s="179"/>
+      <c r="X2" s="179"/>
+      <c r="Y2" s="179"/>
+      <c r="Z2" s="179"/>
+      <c r="AA2" s="179"/>
+      <c r="AB2" s="179"/>
+      <c r="AC2" s="179">
         <v>25</v>
       </c>
-      <c r="AD2" s="178"/>
-      <c r="AE2" s="178"/>
-      <c r="AF2" s="178"/>
-      <c r="AG2" s="178"/>
-      <c r="AH2" s="178"/>
-      <c r="AI2" s="178"/>
-      <c r="AJ2" s="178"/>
-      <c r="AK2" s="178"/>
-      <c r="AL2" s="178"/>
-      <c r="AM2" s="178"/>
-      <c r="AN2" s="178"/>
-      <c r="AO2" s="178">
+      <c r="AD2" s="179"/>
+      <c r="AE2" s="179"/>
+      <c r="AF2" s="179"/>
+      <c r="AG2" s="179"/>
+      <c r="AH2" s="179"/>
+      <c r="AI2" s="179"/>
+      <c r="AJ2" s="179"/>
+      <c r="AK2" s="179"/>
+      <c r="AL2" s="179"/>
+      <c r="AM2" s="179"/>
+      <c r="AN2" s="179"/>
+      <c r="AO2" s="179">
         <v>26</v>
       </c>
-      <c r="AP2" s="178"/>
-      <c r="AQ2" s="178"/>
-      <c r="AR2" s="178"/>
-      <c r="AS2" s="178"/>
-      <c r="AT2" s="178"/>
-      <c r="AU2" s="178"/>
-      <c r="AV2" s="178"/>
-      <c r="AW2" s="178"/>
-      <c r="AX2" s="178"/>
-      <c r="AY2" s="178"/>
-      <c r="AZ2" s="179"/>
-      <c r="BA2" s="178">
+      <c r="AP2" s="179"/>
+      <c r="AQ2" s="179"/>
+      <c r="AR2" s="179"/>
+      <c r="AS2" s="179"/>
+      <c r="AT2" s="179"/>
+      <c r="AU2" s="179"/>
+      <c r="AV2" s="179"/>
+      <c r="AW2" s="179"/>
+      <c r="AX2" s="179"/>
+      <c r="AY2" s="179"/>
+      <c r="AZ2" s="180"/>
+      <c r="BA2" s="179">
         <v>27</v>
       </c>
-      <c r="BB2" s="178"/>
-      <c r="BC2" s="178"/>
-      <c r="BD2" s="178"/>
-      <c r="BE2" s="178"/>
-      <c r="BF2" s="178"/>
-      <c r="BG2" s="178"/>
-      <c r="BH2" s="178"/>
-      <c r="BI2" s="178"/>
-      <c r="BJ2" s="178"/>
-      <c r="BK2" s="178"/>
-      <c r="BL2" s="179"/>
+      <c r="BB2" s="179"/>
+      <c r="BC2" s="179"/>
+      <c r="BD2" s="179"/>
+      <c r="BE2" s="179"/>
+      <c r="BF2" s="179"/>
+      <c r="BG2" s="179"/>
+      <c r="BH2" s="179"/>
+      <c r="BI2" s="179"/>
+      <c r="BJ2" s="179"/>
+      <c r="BK2" s="179"/>
+      <c r="BL2" s="180"/>
     </row>
     <row r="3" spans="1:64" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="175"/>
-      <c r="C3" s="177"/>
-      <c r="D3" s="177"/>
+      <c r="B3" s="176"/>
+      <c r="C3" s="178"/>
+      <c r="D3" s="178"/>
       <c r="E3" s="22">
         <v>1</v>
       </c>
@@ -13201,7 +13259,7 @@
         <v>77</v>
       </c>
       <c r="D11" s="148" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E11" s="6"/>
       <c r="F11" s="7"/>
@@ -13284,7 +13342,7 @@
         <v>105</v>
       </c>
       <c r="D12" s="148" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="7"/>
@@ -13365,7 +13423,7 @@
         <v>82</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E13" s="6"/>
       <c r="F13" s="7"/>
@@ -13535,7 +13593,7 @@
       <c r="BK14" s="7"/>
       <c r="BL14" s="10"/>
     </row>
-    <row r="15" spans="1:64" ht="285.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:64" ht="210.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="27" t="s">
         <v>64</v>
       </c>
@@ -13543,7 +13601,7 @@
         <v>84</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>281</v>
+        <v>437</v>
       </c>
       <c r="E15" s="6"/>
       <c r="F15" s="7"/>
@@ -13709,7 +13767,7 @@
     </row>
     <row r="17" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="52" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C17" s="55" t="s">
         <v>104</v>
@@ -13755,7 +13813,7 @@
       <c r="AH17" s="37"/>
       <c r="AI17" s="33"/>
       <c r="AJ17" s="13" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="AK17" s="41"/>
       <c r="AL17" s="37"/>
@@ -13767,24 +13825,24 @@
       </c>
       <c r="AQ17" s="38"/>
       <c r="AR17" s="33" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AS17" s="37"/>
       <c r="AT17" s="38"/>
       <c r="AU17" s="37"/>
       <c r="AV17" s="37"/>
       <c r="AW17" s="38" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="AX17" s="13"/>
       <c r="AY17" s="37"/>
       <c r="AZ17" s="168" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="BA17" s="42"/>
       <c r="BB17" s="38"/>
       <c r="BC17" s="38" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="BD17" s="13" t="s">
         <v>192</v>
@@ -13806,7 +13864,7 @@
         <v>255</v>
       </c>
       <c r="D18" s="148" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E18" s="59"/>
       <c r="F18" s="60"/>
@@ -14053,7 +14111,7 @@
         <v>107</v>
       </c>
       <c r="D21" s="30" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E21" s="59"/>
       <c r="F21" s="60"/>
@@ -14100,7 +14158,7 @@
       <c r="AS21" s="60"/>
       <c r="AT21" s="60"/>
       <c r="AU21" s="64"/>
-      <c r="AV21" s="13" t="s">
+      <c r="AV21" s="64" t="s">
         <v>219</v>
       </c>
       <c r="AW21" s="60"/>
@@ -14108,7 +14166,7 @@
       <c r="AY21" s="64"/>
       <c r="AZ21" s="65"/>
       <c r="BA21" s="62"/>
-      <c r="BB21" s="13"/>
+      <c r="BB21" s="64"/>
       <c r="BC21" s="64"/>
       <c r="BD21" s="64" t="s">
         <v>230</v>
@@ -14119,7 +14177,7 @@
         <v>231</v>
       </c>
       <c r="BH21" s="64" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="BI21" s="64" t="s">
         <v>232</v>
@@ -14128,14 +14186,16 @@
       <c r="BK21" s="64"/>
       <c r="BL21" s="65"/>
     </row>
-    <row r="22" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:64" ht="108" x14ac:dyDescent="0.3">
       <c r="B22" s="52" t="s">
-        <v>166</v>
+        <v>435</v>
       </c>
       <c r="C22" s="70" t="s">
-        <v>107</v>
-      </c>
-      <c r="D22" s="35"/>
+        <v>104</v>
+      </c>
+      <c r="D22" s="66" t="s">
+        <v>436</v>
+      </c>
       <c r="E22" s="59"/>
       <c r="F22" s="60"/>
       <c r="G22" s="60"/>
@@ -14176,35 +14236,43 @@
       <c r="AP22" s="64"/>
       <c r="AQ22" s="64"/>
       <c r="AR22" s="64"/>
-      <c r="AS22" s="60"/>
+      <c r="AS22" s="64" t="s">
+        <v>438</v>
+      </c>
       <c r="AT22" s="60"/>
       <c r="AU22" s="64"/>
-      <c r="AV22" s="60"/>
+      <c r="AV22" s="64" t="s">
+        <v>219</v>
+      </c>
       <c r="AW22" s="60"/>
       <c r="AX22" s="60"/>
       <c r="AY22" s="64"/>
       <c r="AZ22" s="65"/>
       <c r="BA22" s="62"/>
-      <c r="BB22" s="60"/>
+      <c r="BB22" s="64"/>
       <c r="BC22" s="64"/>
-      <c r="BD22" s="60"/>
+      <c r="BD22" s="64" t="s">
+        <v>439</v>
+      </c>
       <c r="BE22" s="60"/>
       <c r="BF22" s="64"/>
       <c r="BG22" s="64"/>
       <c r="BH22" s="64"/>
-      <c r="BI22" s="64"/>
+      <c r="BI22" s="64" t="s">
+        <v>440</v>
+      </c>
       <c r="BJ22" s="64"/>
       <c r="BK22" s="64"/>
       <c r="BL22" s="65"/>
     </row>
     <row r="23" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="52" t="s">
-        <v>326</v>
-      </c>
-      <c r="C23" s="70"/>
-      <c r="D23" s="153" t="s">
-        <v>319</v>
-      </c>
+        <v>166</v>
+      </c>
+      <c r="C23" s="70" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23" s="35"/>
       <c r="E23" s="59"/>
       <c r="F23" s="60"/>
       <c r="G23" s="60"/>
@@ -14232,40 +14300,28 @@
       <c r="AC23" s="62"/>
       <c r="AD23" s="60"/>
       <c r="AE23" s="60"/>
-      <c r="AF23" s="64" t="s">
-        <v>320</v>
-      </c>
+      <c r="AF23" s="60"/>
       <c r="AG23" s="63"/>
       <c r="AH23" s="60"/>
       <c r="AI23" s="64"/>
       <c r="AJ23" s="60"/>
       <c r="AK23" s="60"/>
-      <c r="AL23" s="64" t="s">
-        <v>321</v>
-      </c>
+      <c r="AL23" s="60"/>
       <c r="AM23" s="60"/>
       <c r="AN23" s="61"/>
       <c r="AO23" s="62"/>
       <c r="AP23" s="64"/>
-      <c r="AQ23" s="64" t="s">
-        <v>328</v>
-      </c>
+      <c r="AQ23" s="64"/>
       <c r="AR23" s="64"/>
       <c r="AS23" s="60"/>
-      <c r="AT23" s="64" t="s">
-        <v>327</v>
-      </c>
+      <c r="AT23" s="60"/>
       <c r="AU23" s="64"/>
       <c r="AV23" s="60"/>
       <c r="AW23" s="60"/>
-      <c r="AX23" s="64" t="s">
-        <v>322</v>
-      </c>
+      <c r="AX23" s="60"/>
       <c r="AY23" s="64"/>
       <c r="AZ23" s="65"/>
-      <c r="BA23" s="154" t="s">
-        <v>323</v>
-      </c>
+      <c r="BA23" s="62"/>
       <c r="BB23" s="60"/>
       <c r="BC23" s="64"/>
       <c r="BD23" s="60"/>
@@ -14278,84 +14334,165 @@
       <c r="BK23" s="64"/>
       <c r="BL23" s="65"/>
     </row>
-    <row r="24" spans="2:64" ht="61.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="69" t="s">
+    <row r="24" spans="2:64" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="52" t="s">
         <v>325</v>
       </c>
-      <c r="C24" s="152"/>
-      <c r="D24" s="150" t="s">
+      <c r="C24" s="70"/>
+      <c r="D24" s="153" t="s">
         <v>318</v>
       </c>
-      <c r="E24" s="44"/>
-      <c r="F24" s="45"/>
-      <c r="G24" s="45"/>
-      <c r="H24" s="45"/>
-      <c r="I24" s="45"/>
-      <c r="J24" s="45"/>
-      <c r="K24" s="45"/>
-      <c r="L24" s="45"/>
-      <c r="M24" s="45"/>
-      <c r="N24" s="45"/>
-      <c r="O24" s="45"/>
-      <c r="P24" s="46"/>
-      <c r="Q24" s="47"/>
-      <c r="R24" s="45"/>
-      <c r="S24" s="45"/>
-      <c r="T24" s="45"/>
-      <c r="U24" s="45"/>
-      <c r="V24" s="45"/>
-      <c r="W24" s="45"/>
-      <c r="X24" s="45"/>
-      <c r="Y24" s="45"/>
-      <c r="Z24" s="45"/>
-      <c r="AA24" s="45"/>
-      <c r="AB24" s="46"/>
-      <c r="AC24" s="47"/>
-      <c r="AD24" s="45"/>
-      <c r="AE24" s="45"/>
-      <c r="AF24" s="45"/>
-      <c r="AG24" s="48"/>
-      <c r="AH24" s="49" t="s">
+      <c r="E24" s="59"/>
+      <c r="F24" s="60"/>
+      <c r="G24" s="60"/>
+      <c r="H24" s="60"/>
+      <c r="I24" s="60"/>
+      <c r="J24" s="60"/>
+      <c r="K24" s="60"/>
+      <c r="L24" s="60"/>
+      <c r="M24" s="60"/>
+      <c r="N24" s="60"/>
+      <c r="O24" s="60"/>
+      <c r="P24" s="61"/>
+      <c r="Q24" s="62"/>
+      <c r="R24" s="60"/>
+      <c r="S24" s="60"/>
+      <c r="T24" s="60"/>
+      <c r="U24" s="60"/>
+      <c r="V24" s="60"/>
+      <c r="W24" s="60"/>
+      <c r="X24" s="60"/>
+      <c r="Y24" s="60"/>
+      <c r="Z24" s="60"/>
+      <c r="AA24" s="60"/>
+      <c r="AB24" s="61"/>
+      <c r="AC24" s="62"/>
+      <c r="AD24" s="60"/>
+      <c r="AE24" s="60"/>
+      <c r="AF24" s="64" t="s">
+        <v>319</v>
+      </c>
+      <c r="AG24" s="63"/>
+      <c r="AH24" s="60"/>
+      <c r="AI24" s="64"/>
+      <c r="AJ24" s="60"/>
+      <c r="AK24" s="60"/>
+      <c r="AL24" s="64" t="s">
+        <v>320</v>
+      </c>
+      <c r="AM24" s="60"/>
+      <c r="AN24" s="61"/>
+      <c r="AO24" s="62"/>
+      <c r="AP24" s="64"/>
+      <c r="AQ24" s="64" t="s">
+        <v>327</v>
+      </c>
+      <c r="AR24" s="64"/>
+      <c r="AS24" s="60"/>
+      <c r="AT24" s="64" t="s">
+        <v>326</v>
+      </c>
+      <c r="AU24" s="64"/>
+      <c r="AV24" s="60"/>
+      <c r="AW24" s="60"/>
+      <c r="AX24" s="64" t="s">
+        <v>321</v>
+      </c>
+      <c r="AY24" s="64"/>
+      <c r="AZ24" s="65"/>
+      <c r="BA24" s="154" t="s">
+        <v>322</v>
+      </c>
+      <c r="BB24" s="60"/>
+      <c r="BC24" s="64"/>
+      <c r="BD24" s="60"/>
+      <c r="BE24" s="60"/>
+      <c r="BF24" s="64"/>
+      <c r="BG24" s="64"/>
+      <c r="BH24" s="64"/>
+      <c r="BI24" s="64"/>
+      <c r="BJ24" s="64"/>
+      <c r="BK24" s="64"/>
+      <c r="BL24" s="65"/>
+    </row>
+    <row r="25" spans="2:64" ht="61.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="69" t="s">
         <v>324</v>
       </c>
-      <c r="AI24" s="49"/>
-      <c r="AJ24" s="45"/>
-      <c r="AK24" s="45"/>
-      <c r="AL24" s="45"/>
-      <c r="AM24" s="45"/>
-      <c r="AN24" s="46"/>
-      <c r="AO24" s="47"/>
-      <c r="AP24" s="49"/>
-      <c r="AQ24" s="49"/>
-      <c r="AR24" s="49"/>
-      <c r="AS24" s="45"/>
-      <c r="AT24" s="49" t="s">
+      <c r="C25" s="152"/>
+      <c r="D25" s="150" t="s">
+        <v>317</v>
+      </c>
+      <c r="E25" s="44"/>
+      <c r="F25" s="45"/>
+      <c r="G25" s="45"/>
+      <c r="H25" s="45"/>
+      <c r="I25" s="45"/>
+      <c r="J25" s="45"/>
+      <c r="K25" s="45"/>
+      <c r="L25" s="45"/>
+      <c r="M25" s="45"/>
+      <c r="N25" s="45"/>
+      <c r="O25" s="45"/>
+      <c r="P25" s="46"/>
+      <c r="Q25" s="47"/>
+      <c r="R25" s="45"/>
+      <c r="S25" s="45"/>
+      <c r="T25" s="45"/>
+      <c r="U25" s="45"/>
+      <c r="V25" s="45"/>
+      <c r="W25" s="45"/>
+      <c r="X25" s="45"/>
+      <c r="Y25" s="45"/>
+      <c r="Z25" s="45"/>
+      <c r="AA25" s="45"/>
+      <c r="AB25" s="46"/>
+      <c r="AC25" s="47"/>
+      <c r="AD25" s="45"/>
+      <c r="AE25" s="45"/>
+      <c r="AF25" s="45"/>
+      <c r="AG25" s="48"/>
+      <c r="AH25" s="49" t="s">
+        <v>323</v>
+      </c>
+      <c r="AI25" s="49"/>
+      <c r="AJ25" s="45"/>
+      <c r="AK25" s="45"/>
+      <c r="AL25" s="45"/>
+      <c r="AM25" s="45"/>
+      <c r="AN25" s="46"/>
+      <c r="AO25" s="47"/>
+      <c r="AP25" s="49"/>
+      <c r="AQ25" s="49"/>
+      <c r="AR25" s="49"/>
+      <c r="AS25" s="45"/>
+      <c r="AT25" s="49" t="s">
+        <v>328</v>
+      </c>
+      <c r="AU25" s="49"/>
+      <c r="AV25" s="45"/>
+      <c r="AW25" s="45"/>
+      <c r="AX25" s="49" t="s">
         <v>329</v>
       </c>
-      <c r="AU24" s="49"/>
-      <c r="AV24" s="45"/>
-      <c r="AW24" s="45"/>
-      <c r="AX24" s="49" t="s">
+      <c r="AY25" s="49"/>
+      <c r="AZ25" s="50"/>
+      <c r="BA25" s="155" t="s">
         <v>330</v>
       </c>
-      <c r="AY24" s="49"/>
-      <c r="AZ24" s="50"/>
-      <c r="BA24" s="155" t="s">
-        <v>331</v>
-      </c>
-      <c r="BB24" s="45"/>
-      <c r="BC24" s="49"/>
-      <c r="BD24" s="45"/>
-      <c r="BE24" s="45"/>
-      <c r="BF24" s="49"/>
-      <c r="BG24" s="49"/>
-      <c r="BH24" s="49"/>
-      <c r="BI24" s="49"/>
-      <c r="BJ24" s="49"/>
-      <c r="BK24" s="49"/>
-      <c r="BL24" s="50"/>
-    </row>
-    <row r="25" spans="2:64" ht="17.25" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="BB25" s="45"/>
+      <c r="BC25" s="49"/>
+      <c r="BD25" s="45"/>
+      <c r="BE25" s="45"/>
+      <c r="BF25" s="49"/>
+      <c r="BG25" s="49"/>
+      <c r="BH25" s="49"/>
+      <c r="BI25" s="49"/>
+      <c r="BJ25" s="49"/>
+      <c r="BK25" s="49"/>
+      <c r="BL25" s="50"/>
+    </row>
+    <row r="26" spans="2:64" ht="17.25" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="B2:B3"/>
@@ -14375,7 +14512,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:J20"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -14400,33 +14537,33 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="183" t="s">
+      <c r="B2" s="184" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="187" t="s">
+      <c r="C2" s="188" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="187" t="s">
+      <c r="D2" s="188" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="185" t="s">
+      <c r="E2" s="186" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="181" t="s">
+      <c r="F2" s="182" t="s">
+        <v>377</v>
+      </c>
+      <c r="G2" s="182"/>
+      <c r="H2" s="182"/>
+      <c r="I2" s="190"/>
+      <c r="J2" s="183"/>
+    </row>
+    <row r="3" spans="1:10" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="185"/>
+      <c r="C3" s="189"/>
+      <c r="D3" s="189"/>
+      <c r="E3" s="187"/>
+      <c r="F3" s="87" t="s">
         <v>378</v>
-      </c>
-      <c r="G2" s="181"/>
-      <c r="H2" s="181"/>
-      <c r="I2" s="189"/>
-      <c r="J2" s="182"/>
-    </row>
-    <row r="3" spans="1:10" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="184"/>
-      <c r="C3" s="188"/>
-      <c r="D3" s="188"/>
-      <c r="E3" s="186"/>
-      <c r="F3" s="87" t="s">
-        <v>379</v>
       </c>
       <c r="G3" s="87"/>
       <c r="H3" s="87"/>
@@ -14446,13 +14583,15 @@
       <c r="E4" s="128" t="s">
         <v>140</v>
       </c>
-      <c r="F4" s="129"/>
+      <c r="F4" s="171" t="s">
+        <v>433</v>
+      </c>
       <c r="G4" s="130"/>
       <c r="H4" s="78"/>
       <c r="I4" s="159"/>
       <c r="J4" s="82"/>
     </row>
-    <row r="5" spans="1:10" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="54" x14ac:dyDescent="0.3">
       <c r="B5" s="142" t="s">
         <v>181</v>
       </c>
@@ -14465,7 +14604,9 @@
       <c r="E5" s="90" t="s">
         <v>161</v>
       </c>
-      <c r="F5" s="112"/>
+      <c r="F5" s="112" t="s">
+        <v>434</v>
+      </c>
       <c r="G5" s="112"/>
       <c r="H5" s="112"/>
       <c r="I5" s="160"/>
@@ -14689,7 +14830,7 @@
         <v>178</v>
       </c>
       <c r="E17" s="103" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F17" s="109"/>
       <c r="G17" s="157"/>
@@ -14771,7 +14912,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -14902,7 +15043,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:N22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -14928,39 +15069,39 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="183" t="s">
+      <c r="B2" s="184" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="187" t="s">
+      <c r="C2" s="188" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="187" t="s">
+      <c r="D2" s="188" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="185" t="s">
+      <c r="E2" s="186" t="s">
         <v>126</v>
       </c>
       <c r="F2" s="86" t="s">
         <v>112</v>
       </c>
-      <c r="G2" s="181" t="s">
+      <c r="G2" s="182" t="s">
         <v>113</v>
       </c>
-      <c r="H2" s="181"/>
-      <c r="I2" s="181"/>
-      <c r="J2" s="182"/>
-      <c r="K2" s="181" t="s">
+      <c r="H2" s="182"/>
+      <c r="I2" s="182"/>
+      <c r="J2" s="183"/>
+      <c r="K2" s="182" t="s">
         <v>182</v>
       </c>
-      <c r="L2" s="181"/>
-      <c r="M2" s="181"/>
-      <c r="N2" s="182"/>
+      <c r="L2" s="182"/>
+      <c r="M2" s="182"/>
+      <c r="N2" s="183"/>
     </row>
     <row r="3" spans="1:14" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="184"/>
-      <c r="C3" s="188"/>
-      <c r="D3" s="188"/>
-      <c r="E3" s="186"/>
+      <c r="B3" s="185"/>
+      <c r="C3" s="189"/>
+      <c r="D3" s="189"/>
+      <c r="E3" s="187"/>
       <c r="F3" s="87" t="s">
         <v>111</v>
       </c>
@@ -15678,7 +15819,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -15703,30 +15844,30 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="183" t="s">
+      <c r="B2" s="184" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="187" t="s">
+      <c r="C2" s="188" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="187" t="s">
+      <c r="D2" s="188" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="185" t="s">
+      <c r="E2" s="186" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="181" t="s">
+      <c r="F2" s="182" t="s">
         <v>182</v>
       </c>
-      <c r="G2" s="181"/>
-      <c r="H2" s="181"/>
-      <c r="I2" s="182"/>
+      <c r="G2" s="182"/>
+      <c r="H2" s="182"/>
+      <c r="I2" s="183"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="184"/>
-      <c r="C3" s="188"/>
-      <c r="D3" s="188"/>
-      <c r="E3" s="186"/>
+      <c r="B3" s="185"/>
+      <c r="C3" s="189"/>
+      <c r="D3" s="189"/>
+      <c r="E3" s="187"/>
       <c r="F3" s="87" t="s">
         <v>114</v>
       </c>
@@ -16079,7 +16220,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -16104,30 +16245,30 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="183" t="s">
+      <c r="B2" s="184" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="187" t="s">
+      <c r="C2" s="188" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="187" t="s">
+      <c r="D2" s="188" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="185" t="s">
+      <c r="E2" s="186" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="181" t="s">
+      <c r="F2" s="182" t="s">
         <v>224</v>
       </c>
-      <c r="G2" s="181"/>
-      <c r="H2" s="181"/>
-      <c r="I2" s="182"/>
+      <c r="G2" s="182"/>
+      <c r="H2" s="182"/>
+      <c r="I2" s="183"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="184"/>
-      <c r="C3" s="188"/>
-      <c r="D3" s="188"/>
-      <c r="E3" s="186"/>
+      <c r="B3" s="185"/>
+      <c r="C3" s="189"/>
+      <c r="D3" s="189"/>
+      <c r="E3" s="187"/>
       <c r="F3" s="87" t="s">
         <v>114</v>
       </c>
@@ -16486,7 +16627,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:I20"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -16511,41 +16652,41 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="183" t="s">
+      <c r="B2" s="184" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="187" t="s">
+      <c r="C2" s="188" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="187" t="s">
+      <c r="D2" s="188" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="185" t="s">
+      <c r="E2" s="186" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="181" t="s">
+      <c r="F2" s="182" t="s">
         <v>256</v>
       </c>
-      <c r="G2" s="181"/>
-      <c r="H2" s="181"/>
-      <c r="I2" s="182"/>
+      <c r="G2" s="182"/>
+      <c r="H2" s="182"/>
+      <c r="I2" s="183"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="184"/>
-      <c r="C3" s="188"/>
-      <c r="D3" s="188"/>
-      <c r="E3" s="186"/>
+      <c r="B3" s="185"/>
+      <c r="C3" s="189"/>
+      <c r="D3" s="189"/>
+      <c r="E3" s="187"/>
       <c r="F3" s="87" t="s">
         <v>277</v>
       </c>
       <c r="G3" s="87" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="H3" s="87" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="I3" s="88" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -16582,10 +16723,10 @@
       <c r="F5" s="104"/>
       <c r="G5" s="95"/>
       <c r="H5" s="112" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I5" s="124" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -16604,7 +16745,7 @@
       <c r="F6" s="112"/>
       <c r="G6" s="112"/>
       <c r="H6" s="122" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="I6" s="144"/>
     </row>
@@ -16625,7 +16766,7 @@
       <c r="G7" s="95"/>
       <c r="H7" s="79"/>
       <c r="I7" s="123" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="87.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -16645,7 +16786,7 @@
       <c r="G8" s="94"/>
       <c r="H8" s="79"/>
       <c r="I8" s="123" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -16734,10 +16875,10 @@
       <c r="F13" s="104"/>
       <c r="G13" s="95"/>
       <c r="H13" s="122" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="I13" s="123" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
@@ -16756,10 +16897,10 @@
       <c r="F14" s="104"/>
       <c r="G14" s="95"/>
       <c r="H14" s="122" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="I14" s="123" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
@@ -16780,10 +16921,10 @@
         <v>265</v>
       </c>
       <c r="H15" s="126" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="I15" s="147" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="228.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -16802,10 +16943,10 @@
       <c r="F16" s="104"/>
       <c r="G16" s="95"/>
       <c r="H16" s="122" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="I16" s="123" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -16826,10 +16967,10 @@
         <v>257</v>
       </c>
       <c r="H17" s="143" t="s">
+        <v>307</v>
+      </c>
+      <c r="I17" s="125" t="s">
         <v>308</v>
-      </c>
-      <c r="I17" s="125" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="18" spans="2:9" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -16868,10 +17009,10 @@
         <v>264</v>
       </c>
       <c r="H19" s="122" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I19" s="123" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="20" spans="2:9" ht="14.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -16909,7 +17050,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:I20"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -16934,41 +17075,41 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="183" t="s">
+      <c r="B2" s="184" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="187" t="s">
+      <c r="C2" s="188" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="187" t="s">
+      <c r="D2" s="188" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="185" t="s">
+      <c r="E2" s="186" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="181" t="s">
+      <c r="F2" s="182" t="s">
         <v>276</v>
       </c>
-      <c r="G2" s="181"/>
-      <c r="H2" s="181"/>
-      <c r="I2" s="182"/>
+      <c r="G2" s="182"/>
+      <c r="H2" s="182"/>
+      <c r="I2" s="183"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="184"/>
-      <c r="C3" s="188"/>
-      <c r="D3" s="188"/>
-      <c r="E3" s="186"/>
+      <c r="B3" s="185"/>
+      <c r="C3" s="189"/>
+      <c r="D3" s="189"/>
+      <c r="E3" s="187"/>
       <c r="F3" s="87" t="s">
+        <v>295</v>
+      </c>
+      <c r="G3" s="87" t="s">
         <v>296</v>
       </c>
-      <c r="G3" s="87" t="s">
+      <c r="H3" s="87" t="s">
         <v>297</v>
       </c>
-      <c r="H3" s="87" t="s">
+      <c r="I3" s="88" t="s">
         <v>298</v>
-      </c>
-      <c r="I3" s="88" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -17003,12 +17144,12 @@
         <v>161</v>
       </c>
       <c r="F5" s="112" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G5" s="145"/>
       <c r="H5" s="112"/>
       <c r="I5" s="124" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -17043,10 +17184,10 @@
         <v>162</v>
       </c>
       <c r="F7" s="112" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G7" s="95" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="H7" s="79"/>
       <c r="I7" s="83"/>
@@ -17153,16 +17294,16 @@
         <v>260</v>
       </c>
       <c r="F13" s="122" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G13" s="145" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="H13" s="95" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="I13" s="111" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="409.5" x14ac:dyDescent="0.3">
@@ -17179,16 +17320,16 @@
         <v>261</v>
       </c>
       <c r="F14" s="122" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G14" s="145" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="H14" s="95" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="I14" s="111" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="175.5" x14ac:dyDescent="0.3">
@@ -17205,16 +17346,16 @@
         <v>259</v>
       </c>
       <c r="F15" s="122" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="G15" s="122" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H15" s="151" t="s">
+        <v>343</v>
+      </c>
+      <c r="I15" s="111" t="s">
         <v>344</v>
-      </c>
-      <c r="I15" s="111" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="409.5" x14ac:dyDescent="0.3">
@@ -17231,16 +17372,16 @@
         <v>262</v>
       </c>
       <c r="F16" s="122" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="G16" s="145" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="H16" s="145" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="I16" s="111" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="162" x14ac:dyDescent="0.3">
@@ -17254,19 +17395,19 @@
         <v>178</v>
       </c>
       <c r="E17" s="103" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F17" s="143" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="G17" s="109" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="H17" s="151" t="s">
+        <v>339</v>
+      </c>
+      <c r="I17" s="156" t="s">
         <v>340</v>
-      </c>
-      <c r="I17" s="156" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.3">
@@ -17299,16 +17440,16 @@
         <v>156</v>
       </c>
       <c r="F19" s="122" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G19" s="146" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="H19" s="122" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="I19" s="123" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="20" spans="2:9" ht="14.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -17325,7 +17466,7 @@
         <v>258</v>
       </c>
       <c r="F20" s="149" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G20" s="135"/>
       <c r="H20" s="136"/>
@@ -17347,7 +17488,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:J20"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -17372,45 +17513,45 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="183" t="s">
+      <c r="B2" s="184" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="187" t="s">
+      <c r="C2" s="188" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="187" t="s">
+      <c r="D2" s="188" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="185" t="s">
+      <c r="E2" s="186" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="181" t="s">
+      <c r="F2" s="182" t="s">
+        <v>346</v>
+      </c>
+      <c r="G2" s="182"/>
+      <c r="H2" s="182"/>
+      <c r="I2" s="190"/>
+      <c r="J2" s="183"/>
+    </row>
+    <row r="3" spans="1:10" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="185"/>
+      <c r="C3" s="189"/>
+      <c r="D3" s="189"/>
+      <c r="E3" s="187"/>
+      <c r="F3" s="87" t="s">
+        <v>345</v>
+      </c>
+      <c r="G3" s="87" t="s">
         <v>347</v>
       </c>
-      <c r="G2" s="181"/>
-      <c r="H2" s="181"/>
-      <c r="I2" s="189"/>
-      <c r="J2" s="182"/>
-    </row>
-    <row r="3" spans="1:10" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="184"/>
-      <c r="C3" s="188"/>
-      <c r="D3" s="188"/>
-      <c r="E3" s="186"/>
-      <c r="F3" s="87" t="s">
-        <v>346</v>
-      </c>
-      <c r="G3" s="87" t="s">
+      <c r="H3" s="87" t="s">
         <v>348</v>
       </c>
-      <c r="H3" s="87" t="s">
+      <c r="I3" s="158" t="s">
         <v>349</v>
       </c>
-      <c r="I3" s="158" t="s">
+      <c r="J3" s="88" t="s">
         <v>350</v>
-      </c>
-      <c r="J3" s="88" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -17446,10 +17587,10 @@
         <v>161</v>
       </c>
       <c r="F5" s="112" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="G5" s="112" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="H5" s="112"/>
       <c r="I5" s="160"/>
@@ -17600,16 +17741,16 @@
         <v>260</v>
       </c>
       <c r="F13" s="95" t="s">
+        <v>365</v>
+      </c>
+      <c r="G13" s="145" t="s">
         <v>366</v>
       </c>
-      <c r="G13" s="145" t="s">
+      <c r="H13" s="95" t="s">
         <v>367</v>
       </c>
-      <c r="H13" s="95" t="s">
-        <v>368</v>
-      </c>
       <c r="I13" s="95" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="J13" s="111"/>
     </row>
@@ -17627,16 +17768,16 @@
         <v>261</v>
       </c>
       <c r="F14" s="95" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="G14" s="145" t="s">
+        <v>368</v>
+      </c>
+      <c r="H14" s="95" t="s">
         <v>369</v>
       </c>
-      <c r="H14" s="95" t="s">
+      <c r="I14" s="95" t="s">
         <v>370</v>
-      </c>
-      <c r="I14" s="95" t="s">
-        <v>371</v>
       </c>
       <c r="J14" s="111"/>
     </row>
@@ -17654,16 +17795,16 @@
         <v>259</v>
       </c>
       <c r="F15" s="95" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="G15" s="145" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="H15" s="145" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="I15" s="145" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="J15" s="111"/>
     </row>
@@ -17681,16 +17822,16 @@
         <v>262</v>
       </c>
       <c r="F16" s="95" t="s">
+        <v>358</v>
+      </c>
+      <c r="G16" s="145" t="s">
         <v>359</v>
       </c>
-      <c r="G16" s="145" t="s">
-        <v>360</v>
-      </c>
       <c r="H16" s="145" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="I16" s="145" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="J16" s="111"/>
     </row>
@@ -17705,19 +17846,19 @@
         <v>178</v>
       </c>
       <c r="E17" s="103" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F17" s="109" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G17" s="157" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="H17" s="157" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I17" s="157" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="J17" s="156"/>
     </row>
@@ -17752,7 +17893,7 @@
         <v>156</v>
       </c>
       <c r="F19" s="95" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G19" s="146"/>
       <c r="H19" s="122"/>
@@ -17795,7 +17936,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:I22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -17820,41 +17961,41 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="183" t="s">
+      <c r="B2" s="184" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="187" t="s">
+      <c r="C2" s="188" t="s">
         <v>176</v>
       </c>
-      <c r="D2" s="187" t="s">
+      <c r="D2" s="188" t="s">
         <v>177</v>
       </c>
-      <c r="E2" s="185" t="s">
+      <c r="E2" s="186" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="181" t="s">
+      <c r="F2" s="182" t="s">
+        <v>372</v>
+      </c>
+      <c r="G2" s="182"/>
+      <c r="H2" s="182"/>
+      <c r="I2" s="183"/>
+    </row>
+    <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="185"/>
+      <c r="C3" s="189"/>
+      <c r="D3" s="189"/>
+      <c r="E3" s="187"/>
+      <c r="F3" s="87" t="s">
         <v>373</v>
       </c>
-      <c r="G2" s="181"/>
-      <c r="H2" s="181"/>
-      <c r="I2" s="182"/>
-    </row>
-    <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="184"/>
-      <c r="C3" s="188"/>
-      <c r="D3" s="188"/>
-      <c r="E3" s="186"/>
-      <c r="F3" s="87" t="s">
+      <c r="G3" s="87" t="s">
         <v>374</v>
       </c>
-      <c r="G3" s="87" t="s">
+      <c r="H3" s="87" t="s">
         <v>375</v>
       </c>
-      <c r="H3" s="87" t="s">
+      <c r="I3" s="88" t="s">
         <v>376</v>
-      </c>
-      <c r="I3" s="88" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="67.5" x14ac:dyDescent="0.3">
@@ -17868,13 +18009,13 @@
         <v>178</v>
       </c>
       <c r="E4" s="128" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F4" s="171" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="G4" s="171" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="H4" s="78"/>
       <c r="I4" s="82"/>
@@ -17890,19 +18031,19 @@
         <v>180</v>
       </c>
       <c r="E5" s="90" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F5" s="112" t="s">
+        <v>402</v>
+      </c>
+      <c r="G5" s="112" t="s">
         <v>403</v>
       </c>
-      <c r="G5" s="112" t="s">
-        <v>404</v>
-      </c>
       <c r="H5" s="112" t="s">
+        <v>416</v>
+      </c>
+      <c r="I5" s="124" t="s">
         <v>417</v>
-      </c>
-      <c r="I5" s="124" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -17916,19 +18057,19 @@
         <v>178</v>
       </c>
       <c r="E6" s="90" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F6" s="112" t="s">
+        <v>392</v>
+      </c>
+      <c r="G6" s="112" t="s">
         <v>393</v>
       </c>
-      <c r="G6" s="112" t="s">
-        <v>394</v>
-      </c>
       <c r="H6" s="112" t="s">
+        <v>418</v>
+      </c>
+      <c r="I6" s="124" t="s">
         <v>419</v>
-      </c>
-      <c r="I6" s="124" t="s">
-        <v>420</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="310.5" x14ac:dyDescent="0.3">
@@ -17942,19 +18083,19 @@
         <v>178</v>
       </c>
       <c r="E7" s="90" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="F7" s="112" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="G7" s="95" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H7" s="95" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="I7" s="111" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
@@ -17989,7 +18130,7 @@
         <v>152</v>
       </c>
       <c r="F9" s="104" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="G9" s="95"/>
       <c r="I9" s="83"/>
@@ -18008,7 +18149,7 @@
         <v>153</v>
       </c>
       <c r="F10" s="104" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="G10" s="95"/>
       <c r="H10" s="79"/>
@@ -18028,7 +18169,7 @@
         <v>154</v>
       </c>
       <c r="F11" s="104" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="G11" s="95"/>
       <c r="H11" s="79"/>
@@ -18048,32 +18189,32 @@
         <v>155</v>
       </c>
       <c r="F12" s="104" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="G12" s="95"/>
       <c r="I12" s="83"/>
     </row>
     <row r="13" spans="1:9" ht="94.5" x14ac:dyDescent="0.3">
       <c r="B13" s="121" t="s">
+        <v>394</v>
+      </c>
+      <c r="C13" s="107" t="s">
+        <v>397</v>
+      </c>
+      <c r="D13" s="107" t="s">
+        <v>398</v>
+      </c>
+      <c r="E13" s="81" t="s">
         <v>395</v>
       </c>
-      <c r="C13" s="107" t="s">
-        <v>398</v>
-      </c>
-      <c r="D13" s="107" t="s">
-        <v>399</v>
-      </c>
-      <c r="E13" s="81" t="s">
+      <c r="F13" s="112" t="s">
         <v>396</v>
       </c>
-      <c r="F13" s="112" t="s">
-        <v>397</v>
-      </c>
       <c r="G13" s="169" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="H13" s="172" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="I13" s="170"/>
     </row>
@@ -18092,13 +18233,13 @@
       </c>
       <c r="F14" s="95"/>
       <c r="G14" s="145" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="H14" s="95" t="s">
+        <v>422</v>
+      </c>
+      <c r="I14" s="111" t="s">
         <v>423</v>
-      </c>
-      <c r="I14" s="111" t="s">
-        <v>424</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="409.5" x14ac:dyDescent="0.3">
@@ -18115,16 +18256,16 @@
         <v>261</v>
       </c>
       <c r="F15" s="95" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="G15" s="145" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="H15" s="95" t="s">
+        <v>424</v>
+      </c>
+      <c r="I15" s="111" t="s">
         <v>425</v>
-      </c>
-      <c r="I15" s="111" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="108" x14ac:dyDescent="0.3">
@@ -18141,16 +18282,16 @@
         <v>259</v>
       </c>
       <c r="F16" s="95" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="G16" s="145" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="H16" s="145" t="s">
+        <v>426</v>
+      </c>
+      <c r="I16" s="164" t="s">
         <v>427</v>
-      </c>
-      <c r="I16" s="164" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="409.5" x14ac:dyDescent="0.3">
@@ -18167,16 +18308,16 @@
         <v>262</v>
       </c>
       <c r="F17" s="95" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G17" s="145" t="s">
+        <v>409</v>
+      </c>
+      <c r="H17" s="145" t="s">
         <v>410</v>
       </c>
-      <c r="H17" s="145" t="s">
-        <v>411</v>
-      </c>
       <c r="I17" s="164" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="18" spans="2:9" ht="108" x14ac:dyDescent="0.3">
@@ -18190,19 +18331,19 @@
         <v>178</v>
       </c>
       <c r="E18" s="103" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F18" s="109" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="G18" s="157" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="H18" s="157" t="s">
+        <v>429</v>
+      </c>
+      <c r="I18" s="165" t="s">
         <v>430</v>
-      </c>
-      <c r="I18" s="165" t="s">
-        <v>431</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.3">
@@ -18238,13 +18379,13 @@
         <v>263</v>
       </c>
       <c r="G20" s="145" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="H20" s="95" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="I20" s="111" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="21" spans="2:9" ht="14.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -18264,13 +18405,13 @@
         <v>263</v>
       </c>
       <c r="G21" s="96" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="H21" s="173" t="s">
-        <v>408</v>
-      </c>
-      <c r="I21" s="190" t="s">
-        <v>420</v>
+        <v>407</v>
+      </c>
+      <c r="I21" s="174" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="22" spans="2:9" ht="14.25" thickTop="1" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Weekly Plan 수정 및 3월 추가
</commit_message>
<xml_diff>
--- a/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
+++ b/1. 일정/1. Weekly Plan/Air PTC Heater Weekly Plan.xlsx
@@ -22,6 +22,7 @@
     <sheet name="2025.12" sheetId="9" r:id="rId8"/>
     <sheet name="2026.1" sheetId="10" r:id="rId9"/>
     <sheet name="2026.2" sheetId="11" r:id="rId10"/>
+    <sheet name="2026.3" sheetId="12" r:id="rId11"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1137" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="480">
   <si>
     <t>■</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -11319,6 +11320,34 @@
     - 제어기 개발 현황 작성 (기아샤시시스템품질팀 김제일 매니저)
   [ 진행 및 검토 ]
     - 제어기 개발 현황 작성 완료</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>- 이슈 없음</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3월</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1주차 (02/27 ~ 03/05)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2주차 (03/06 ~ 03/12)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3주차 (03/13 ~ 03/19)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>4주차 (03/20 ~ 03/26)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>5주차 (03/27 ~ 04/02)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -11562,7 +11591,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="89">
+  <borders count="90">
     <border>
       <left/>
       <right/>
@@ -12763,6 +12792,19 @@
     </border>
     <border>
       <left/>
+      <right/>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
       <top style="hair">
         <color auto="1"/>
@@ -12793,7 +12835,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="197">
+  <cellXfs count="200">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -13334,9 +13376,6 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="65" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -13384,6 +13423,18 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="83" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="66" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="86" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="73" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="89" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -14267,90 +14318,90 @@
       <c r="D1" s="21"/>
     </row>
     <row r="2" spans="1:64" ht="31.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="181" t="s">
+      <c r="B2" s="180" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="183" t="s">
+      <c r="C2" s="182" t="s">
         <v>76</v>
       </c>
-      <c r="D2" s="183" t="s">
+      <c r="D2" s="182" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="187">
+      <c r="E2" s="186">
         <v>23</v>
       </c>
-      <c r="F2" s="185"/>
-      <c r="G2" s="185"/>
-      <c r="H2" s="185"/>
-      <c r="I2" s="185"/>
-      <c r="J2" s="185"/>
-      <c r="K2" s="185"/>
-      <c r="L2" s="185"/>
-      <c r="M2" s="185"/>
-      <c r="N2" s="185"/>
-      <c r="O2" s="185"/>
-      <c r="P2" s="185"/>
-      <c r="Q2" s="185">
+      <c r="F2" s="184"/>
+      <c r="G2" s="184"/>
+      <c r="H2" s="184"/>
+      <c r="I2" s="184"/>
+      <c r="J2" s="184"/>
+      <c r="K2" s="184"/>
+      <c r="L2" s="184"/>
+      <c r="M2" s="184"/>
+      <c r="N2" s="184"/>
+      <c r="O2" s="184"/>
+      <c r="P2" s="184"/>
+      <c r="Q2" s="184">
         <v>24</v>
       </c>
-      <c r="R2" s="185"/>
-      <c r="S2" s="185"/>
-      <c r="T2" s="185"/>
-      <c r="U2" s="185"/>
-      <c r="V2" s="185"/>
-      <c r="W2" s="185"/>
-      <c r="X2" s="185"/>
-      <c r="Y2" s="185"/>
-      <c r="Z2" s="185"/>
-      <c r="AA2" s="185"/>
-      <c r="AB2" s="185"/>
-      <c r="AC2" s="185">
+      <c r="R2" s="184"/>
+      <c r="S2" s="184"/>
+      <c r="T2" s="184"/>
+      <c r="U2" s="184"/>
+      <c r="V2" s="184"/>
+      <c r="W2" s="184"/>
+      <c r="X2" s="184"/>
+      <c r="Y2" s="184"/>
+      <c r="Z2" s="184"/>
+      <c r="AA2" s="184"/>
+      <c r="AB2" s="184"/>
+      <c r="AC2" s="184">
         <v>25</v>
       </c>
-      <c r="AD2" s="185"/>
-      <c r="AE2" s="185"/>
-      <c r="AF2" s="185"/>
-      <c r="AG2" s="185"/>
-      <c r="AH2" s="185"/>
-      <c r="AI2" s="185"/>
-      <c r="AJ2" s="185"/>
-      <c r="AK2" s="185"/>
-      <c r="AL2" s="185"/>
-      <c r="AM2" s="185"/>
-      <c r="AN2" s="185"/>
-      <c r="AO2" s="185">
+      <c r="AD2" s="184"/>
+      <c r="AE2" s="184"/>
+      <c r="AF2" s="184"/>
+      <c r="AG2" s="184"/>
+      <c r="AH2" s="184"/>
+      <c r="AI2" s="184"/>
+      <c r="AJ2" s="184"/>
+      <c r="AK2" s="184"/>
+      <c r="AL2" s="184"/>
+      <c r="AM2" s="184"/>
+      <c r="AN2" s="184"/>
+      <c r="AO2" s="184">
         <v>26</v>
       </c>
-      <c r="AP2" s="185"/>
-      <c r="AQ2" s="185"/>
-      <c r="AR2" s="185"/>
-      <c r="AS2" s="185"/>
-      <c r="AT2" s="185"/>
-      <c r="AU2" s="185"/>
-      <c r="AV2" s="185"/>
-      <c r="AW2" s="185"/>
-      <c r="AX2" s="185"/>
-      <c r="AY2" s="185"/>
-      <c r="AZ2" s="186"/>
-      <c r="BA2" s="185">
+      <c r="AP2" s="184"/>
+      <c r="AQ2" s="184"/>
+      <c r="AR2" s="184"/>
+      <c r="AS2" s="184"/>
+      <c r="AT2" s="184"/>
+      <c r="AU2" s="184"/>
+      <c r="AV2" s="184"/>
+      <c r="AW2" s="184"/>
+      <c r="AX2" s="184"/>
+      <c r="AY2" s="184"/>
+      <c r="AZ2" s="185"/>
+      <c r="BA2" s="184">
         <v>27</v>
       </c>
-      <c r="BB2" s="185"/>
-      <c r="BC2" s="185"/>
-      <c r="BD2" s="185"/>
-      <c r="BE2" s="185"/>
-      <c r="BF2" s="185"/>
-      <c r="BG2" s="185"/>
-      <c r="BH2" s="185"/>
-      <c r="BI2" s="185"/>
-      <c r="BJ2" s="185"/>
-      <c r="BK2" s="185"/>
-      <c r="BL2" s="186"/>
+      <c r="BB2" s="184"/>
+      <c r="BC2" s="184"/>
+      <c r="BD2" s="184"/>
+      <c r="BE2" s="184"/>
+      <c r="BF2" s="184"/>
+      <c r="BG2" s="184"/>
+      <c r="BH2" s="184"/>
+      <c r="BI2" s="184"/>
+      <c r="BJ2" s="184"/>
+      <c r="BK2" s="184"/>
+      <c r="BL2" s="185"/>
     </row>
     <row r="3" spans="1:64" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="182"/>
-      <c r="C3" s="184"/>
-      <c r="D3" s="184"/>
+      <c r="B3" s="181"/>
+      <c r="C3" s="183"/>
+      <c r="D3" s="183"/>
       <c r="E3" s="22">
         <v>1</v>
       </c>
@@ -16366,30 +16417,30 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="190" t="s">
+      <c r="B2" s="189" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="194" t="s">
+      <c r="C2" s="193" t="s">
         <v>174</v>
       </c>
-      <c r="D2" s="194" t="s">
+      <c r="D2" s="193" t="s">
         <v>175</v>
       </c>
-      <c r="E2" s="192" t="s">
+      <c r="E2" s="191" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="188" t="s">
+      <c r="F2" s="187" t="s">
         <v>374</v>
       </c>
-      <c r="G2" s="188"/>
-      <c r="H2" s="188"/>
-      <c r="I2" s="189"/>
+      <c r="G2" s="187"/>
+      <c r="H2" s="187"/>
+      <c r="I2" s="188"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="191"/>
-      <c r="C3" s="195"/>
-      <c r="D3" s="195"/>
-      <c r="E3" s="193"/>
+      <c r="B3" s="190"/>
+      <c r="C3" s="194"/>
+      <c r="D3" s="194"/>
+      <c r="E3" s="192"/>
       <c r="F3" s="87" t="s">
         <v>375</v>
       </c>
@@ -16761,7 +16812,9 @@
       <c r="H19" s="95" t="s">
         <v>260</v>
       </c>
-      <c r="I19" s="123"/>
+      <c r="I19" s="111" t="s">
+        <v>473</v>
+      </c>
     </row>
     <row r="20" spans="2:9" ht="14.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="176" t="s">
@@ -16785,7 +16838,9 @@
       <c r="H20" s="179" t="s">
         <v>260</v>
       </c>
-      <c r="I20" s="180"/>
+      <c r="I20" s="196" t="s">
+        <v>473</v>
+      </c>
     </row>
     <row r="21" spans="2:9" ht="14.25" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
@@ -16800,6 +16855,409 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.375" style="71" customWidth="1"/>
+    <col min="2" max="2" width="9" style="71"/>
+    <col min="3" max="4" width="14.75" style="71" customWidth="1"/>
+    <col min="5" max="5" width="43" style="71" customWidth="1"/>
+    <col min="6" max="6" width="61.875" style="71" customWidth="1"/>
+    <col min="7" max="10" width="62.125" style="71" customWidth="1"/>
+    <col min="11" max="16384" width="9" style="71"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="32.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="98" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="99" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="97"/>
+    </row>
+    <row r="2" spans="1:10" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="189" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="193" t="s">
+        <v>174</v>
+      </c>
+      <c r="D2" s="193" t="s">
+        <v>175</v>
+      </c>
+      <c r="E2" s="191" t="s">
+        <v>126</v>
+      </c>
+      <c r="F2" s="187" t="s">
+        <v>474</v>
+      </c>
+      <c r="G2" s="187"/>
+      <c r="H2" s="187"/>
+      <c r="I2" s="195"/>
+      <c r="J2" s="188"/>
+    </row>
+    <row r="3" spans="1:10" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="190"/>
+      <c r="C3" s="194"/>
+      <c r="D3" s="194"/>
+      <c r="E3" s="192"/>
+      <c r="F3" s="87" t="s">
+        <v>475</v>
+      </c>
+      <c r="G3" s="87" t="s">
+        <v>476</v>
+      </c>
+      <c r="H3" s="87" t="s">
+        <v>477</v>
+      </c>
+      <c r="I3" s="158" t="s">
+        <v>478</v>
+      </c>
+      <c r="J3" s="88" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="139" t="s">
+        <v>108</v>
+      </c>
+      <c r="C4" s="106" t="s">
+        <v>173</v>
+      </c>
+      <c r="D4" s="106" t="s">
+        <v>176</v>
+      </c>
+      <c r="E4" s="128" t="s">
+        <v>138</v>
+      </c>
+      <c r="F4" s="171"/>
+      <c r="G4" s="130"/>
+      <c r="H4" s="78"/>
+      <c r="I4" s="159"/>
+      <c r="J4" s="82"/>
+    </row>
+    <row r="5" spans="1:10" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="B5" s="142" t="s">
+        <v>179</v>
+      </c>
+      <c r="C5" s="107" t="s">
+        <v>264</v>
+      </c>
+      <c r="D5" s="107" t="s">
+        <v>178</v>
+      </c>
+      <c r="E5" s="90" t="s">
+        <v>159</v>
+      </c>
+      <c r="F5" s="112"/>
+      <c r="G5" s="112"/>
+      <c r="H5" s="112"/>
+      <c r="I5" s="160"/>
+      <c r="J5" s="124"/>
+    </row>
+    <row r="6" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="140" t="s">
+        <v>118</v>
+      </c>
+      <c r="C6" s="107" t="s">
+        <v>265</v>
+      </c>
+      <c r="D6" s="107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E6" s="90" t="s">
+        <v>159</v>
+      </c>
+      <c r="F6" s="112"/>
+      <c r="G6" s="112"/>
+      <c r="H6" s="112"/>
+      <c r="I6" s="160"/>
+      <c r="J6" s="124"/>
+    </row>
+    <row r="7" spans="1:10" ht="309" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="140" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="107" t="s">
+        <v>265</v>
+      </c>
+      <c r="D7" s="107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E7" s="90" t="s">
+        <v>160</v>
+      </c>
+      <c r="F7" s="112"/>
+      <c r="G7" s="95"/>
+      <c r="H7" s="95"/>
+      <c r="I7" s="197"/>
+      <c r="J7" s="111"/>
+    </row>
+    <row r="8" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="140" t="s">
+        <v>109</v>
+      </c>
+      <c r="C8" s="107" t="s">
+        <v>265</v>
+      </c>
+      <c r="D8" s="107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E8" s="81" t="s">
+        <v>137</v>
+      </c>
+      <c r="F8" s="104"/>
+      <c r="G8" s="94"/>
+      <c r="H8" s="79"/>
+      <c r="I8" s="161"/>
+      <c r="J8" s="83"/>
+    </row>
+    <row r="9" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="141" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" s="107" t="s">
+        <v>265</v>
+      </c>
+      <c r="D9" s="107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E9" s="81" t="s">
+        <v>150</v>
+      </c>
+      <c r="F9" s="104"/>
+      <c r="G9" s="95"/>
+      <c r="H9" s="79"/>
+      <c r="I9" s="175"/>
+      <c r="J9" s="83"/>
+    </row>
+    <row r="10" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="141" t="s">
+        <v>123</v>
+      </c>
+      <c r="C10" s="107" t="s">
+        <v>265</v>
+      </c>
+      <c r="D10" s="107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E10" s="81" t="s">
+        <v>151</v>
+      </c>
+      <c r="F10" s="104"/>
+      <c r="G10" s="95"/>
+      <c r="H10" s="79"/>
+      <c r="I10" s="161"/>
+      <c r="J10" s="83"/>
+    </row>
+    <row r="11" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="141" t="s">
+        <v>124</v>
+      </c>
+      <c r="C11" s="107" t="s">
+        <v>265</v>
+      </c>
+      <c r="D11" s="107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E11" s="81" t="s">
+        <v>152</v>
+      </c>
+      <c r="F11" s="104"/>
+      <c r="G11" s="95"/>
+      <c r="H11" s="79"/>
+      <c r="I11" s="161"/>
+      <c r="J11" s="83"/>
+    </row>
+    <row r="12" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="141" t="s">
+        <v>125</v>
+      </c>
+      <c r="C12" s="107" t="s">
+        <v>265</v>
+      </c>
+      <c r="D12" s="107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E12" s="81" t="s">
+        <v>153</v>
+      </c>
+      <c r="F12" s="104"/>
+      <c r="G12" s="95"/>
+      <c r="H12" s="79"/>
+      <c r="I12" s="175"/>
+      <c r="J12" s="83"/>
+    </row>
+    <row r="13" spans="1:10" ht="27" x14ac:dyDescent="0.3">
+      <c r="B13" s="121" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="107" t="s">
+        <v>267</v>
+      </c>
+      <c r="D13" s="107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E13" s="90" t="s">
+        <v>257</v>
+      </c>
+      <c r="F13" s="95"/>
+      <c r="G13" s="145"/>
+      <c r="H13" s="95"/>
+      <c r="I13" s="197"/>
+      <c r="J13" s="111"/>
+    </row>
+    <row r="14" spans="1:10" ht="27" x14ac:dyDescent="0.3">
+      <c r="B14" s="120" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="107" t="s">
+        <v>267</v>
+      </c>
+      <c r="D14" s="107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E14" s="90" t="s">
+        <v>258</v>
+      </c>
+      <c r="F14" s="95"/>
+      <c r="G14" s="145"/>
+      <c r="H14" s="95"/>
+      <c r="I14" s="197"/>
+      <c r="J14" s="111"/>
+    </row>
+    <row r="15" spans="1:10" ht="67.5" x14ac:dyDescent="0.3">
+      <c r="B15" s="121" t="s">
+        <v>444</v>
+      </c>
+      <c r="C15" s="107" t="s">
+        <v>267</v>
+      </c>
+      <c r="D15" s="107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E15" s="90" t="s">
+        <v>256</v>
+      </c>
+      <c r="F15" s="95"/>
+      <c r="G15" s="145"/>
+      <c r="H15" s="145"/>
+      <c r="I15" s="95"/>
+      <c r="J15" s="164"/>
+    </row>
+    <row r="16" spans="1:10" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="B16" s="120" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" s="107" t="s">
+        <v>267</v>
+      </c>
+      <c r="D16" s="107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E16" s="90" t="s">
+        <v>259</v>
+      </c>
+      <c r="F16" s="95"/>
+      <c r="G16" s="145"/>
+      <c r="H16" s="145"/>
+      <c r="I16" s="95"/>
+      <c r="J16" s="164"/>
+    </row>
+    <row r="17" spans="2:10" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="B17" s="119" t="s">
+        <v>165</v>
+      </c>
+      <c r="C17" s="107" t="s">
+        <v>267</v>
+      </c>
+      <c r="D17" s="107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E17" s="103" t="s">
+        <v>299</v>
+      </c>
+      <c r="F17" s="109"/>
+      <c r="G17" s="157"/>
+      <c r="H17" s="157"/>
+      <c r="I17" s="95"/>
+      <c r="J17" s="165"/>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B18" s="120" t="s">
+        <v>139</v>
+      </c>
+      <c r="C18" s="107" t="s">
+        <v>267</v>
+      </c>
+      <c r="D18" s="107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E18" s="103"/>
+      <c r="F18" s="109"/>
+      <c r="G18" s="109"/>
+      <c r="H18" s="109"/>
+      <c r="I18" s="198"/>
+      <c r="J18" s="156"/>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B19" s="138" t="s">
+        <v>443</v>
+      </c>
+      <c r="C19" s="127" t="s">
+        <v>267</v>
+      </c>
+      <c r="D19" s="127" t="s">
+        <v>176</v>
+      </c>
+      <c r="E19" s="81" t="s">
+        <v>154</v>
+      </c>
+      <c r="F19" s="95"/>
+      <c r="G19" s="95"/>
+      <c r="H19" s="95"/>
+      <c r="I19" s="197"/>
+      <c r="J19" s="111"/>
+    </row>
+    <row r="20" spans="2:10" ht="14.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="176" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="177" t="s">
+        <v>267</v>
+      </c>
+      <c r="D20" s="177" t="s">
+        <v>176</v>
+      </c>
+      <c r="E20" s="178" t="s">
+        <v>255</v>
+      </c>
+      <c r="F20" s="179"/>
+      <c r="G20" s="179"/>
+      <c r="H20" s="179"/>
+      <c r="I20" s="199"/>
+      <c r="J20" s="196"/>
+    </row>
+    <row r="21" spans="2:10" ht="14.25" thickTop="1" x14ac:dyDescent="0.3"/>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:J2"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -16961,39 +17419,39 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="190" t="s">
+      <c r="B2" s="189" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="194" t="s">
+      <c r="C2" s="193" t="s">
         <v>174</v>
       </c>
-      <c r="D2" s="194" t="s">
+      <c r="D2" s="193" t="s">
         <v>175</v>
       </c>
-      <c r="E2" s="192" t="s">
+      <c r="E2" s="191" t="s">
         <v>126</v>
       </c>
       <c r="F2" s="86" t="s">
         <v>112</v>
       </c>
-      <c r="G2" s="188" t="s">
+      <c r="G2" s="187" t="s">
         <v>113</v>
       </c>
-      <c r="H2" s="188"/>
-      <c r="I2" s="188"/>
-      <c r="J2" s="189"/>
-      <c r="K2" s="188" t="s">
+      <c r="H2" s="187"/>
+      <c r="I2" s="187"/>
+      <c r="J2" s="188"/>
+      <c r="K2" s="187" t="s">
         <v>180</v>
       </c>
-      <c r="L2" s="188"/>
-      <c r="M2" s="188"/>
-      <c r="N2" s="189"/>
+      <c r="L2" s="187"/>
+      <c r="M2" s="187"/>
+      <c r="N2" s="188"/>
     </row>
     <row r="3" spans="1:14" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="191"/>
-      <c r="C3" s="195"/>
-      <c r="D3" s="195"/>
-      <c r="E3" s="193"/>
+      <c r="B3" s="190"/>
+      <c r="C3" s="194"/>
+      <c r="D3" s="194"/>
+      <c r="E3" s="192"/>
       <c r="F3" s="87" t="s">
         <v>111</v>
       </c>
@@ -17736,30 +18194,30 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="190" t="s">
+      <c r="B2" s="189" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="194" t="s">
+      <c r="C2" s="193" t="s">
         <v>174</v>
       </c>
-      <c r="D2" s="194" t="s">
+      <c r="D2" s="193" t="s">
         <v>175</v>
       </c>
-      <c r="E2" s="192" t="s">
+      <c r="E2" s="191" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="188" t="s">
+      <c r="F2" s="187" t="s">
         <v>180</v>
       </c>
-      <c r="G2" s="188"/>
-      <c r="H2" s="188"/>
-      <c r="I2" s="189"/>
+      <c r="G2" s="187"/>
+      <c r="H2" s="187"/>
+      <c r="I2" s="188"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="191"/>
-      <c r="C3" s="195"/>
-      <c r="D3" s="195"/>
-      <c r="E3" s="193"/>
+      <c r="B3" s="190"/>
+      <c r="C3" s="194"/>
+      <c r="D3" s="194"/>
+      <c r="E3" s="192"/>
       <c r="F3" s="87" t="s">
         <v>114</v>
       </c>
@@ -18137,30 +18595,30 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="190" t="s">
+      <c r="B2" s="189" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="194" t="s">
+      <c r="C2" s="193" t="s">
         <v>174</v>
       </c>
-      <c r="D2" s="194" t="s">
+      <c r="D2" s="193" t="s">
         <v>175</v>
       </c>
-      <c r="E2" s="192" t="s">
+      <c r="E2" s="191" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="188" t="s">
+      <c r="F2" s="187" t="s">
         <v>221</v>
       </c>
-      <c r="G2" s="188"/>
-      <c r="H2" s="188"/>
-      <c r="I2" s="189"/>
+      <c r="G2" s="187"/>
+      <c r="H2" s="187"/>
+      <c r="I2" s="188"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="191"/>
-      <c r="C3" s="195"/>
-      <c r="D3" s="195"/>
-      <c r="E3" s="193"/>
+      <c r="B3" s="190"/>
+      <c r="C3" s="194"/>
+      <c r="D3" s="194"/>
+      <c r="E3" s="192"/>
       <c r="F3" s="87" t="s">
         <v>114</v>
       </c>
@@ -18544,30 +19002,30 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="190" t="s">
+      <c r="B2" s="189" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="194" t="s">
+      <c r="C2" s="193" t="s">
         <v>174</v>
       </c>
-      <c r="D2" s="194" t="s">
+      <c r="D2" s="193" t="s">
         <v>175</v>
       </c>
-      <c r="E2" s="192" t="s">
+      <c r="E2" s="191" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="188" t="s">
+      <c r="F2" s="187" t="s">
         <v>253</v>
       </c>
-      <c r="G2" s="188"/>
-      <c r="H2" s="188"/>
-      <c r="I2" s="189"/>
+      <c r="G2" s="187"/>
+      <c r="H2" s="187"/>
+      <c r="I2" s="188"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="191"/>
-      <c r="C3" s="195"/>
-      <c r="D3" s="195"/>
-      <c r="E3" s="193"/>
+      <c r="B3" s="190"/>
+      <c r="C3" s="194"/>
+      <c r="D3" s="194"/>
+      <c r="E3" s="192"/>
       <c r="F3" s="87" t="s">
         <v>274</v>
       </c>
@@ -18967,30 +19425,30 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="190" t="s">
+      <c r="B2" s="189" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="194" t="s">
+      <c r="C2" s="193" t="s">
         <v>174</v>
       </c>
-      <c r="D2" s="194" t="s">
+      <c r="D2" s="193" t="s">
         <v>175</v>
       </c>
-      <c r="E2" s="192" t="s">
+      <c r="E2" s="191" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="188" t="s">
+      <c r="F2" s="187" t="s">
         <v>273</v>
       </c>
-      <c r="G2" s="188"/>
-      <c r="H2" s="188"/>
-      <c r="I2" s="189"/>
+      <c r="G2" s="187"/>
+      <c r="H2" s="187"/>
+      <c r="I2" s="188"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="191"/>
-      <c r="C3" s="195"/>
-      <c r="D3" s="195"/>
-      <c r="E3" s="193"/>
+      <c r="B3" s="190"/>
+      <c r="C3" s="194"/>
+      <c r="D3" s="194"/>
+      <c r="E3" s="192"/>
       <c r="F3" s="87" t="s">
         <v>292</v>
       </c>
@@ -19405,31 +19863,31 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="190" t="s">
+      <c r="B2" s="189" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="194" t="s">
+      <c r="C2" s="193" t="s">
         <v>174</v>
       </c>
-      <c r="D2" s="194" t="s">
+      <c r="D2" s="193" t="s">
         <v>175</v>
       </c>
-      <c r="E2" s="192" t="s">
+      <c r="E2" s="191" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="188" t="s">
+      <c r="F2" s="187" t="s">
         <v>343</v>
       </c>
-      <c r="G2" s="188"/>
-      <c r="H2" s="188"/>
-      <c r="I2" s="196"/>
-      <c r="J2" s="189"/>
+      <c r="G2" s="187"/>
+      <c r="H2" s="187"/>
+      <c r="I2" s="195"/>
+      <c r="J2" s="188"/>
     </row>
     <row r="3" spans="1:10" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="191"/>
-      <c r="C3" s="195"/>
-      <c r="D3" s="195"/>
-      <c r="E3" s="193"/>
+      <c r="B3" s="190"/>
+      <c r="C3" s="194"/>
+      <c r="D3" s="194"/>
+      <c r="E3" s="192"/>
       <c r="F3" s="87" t="s">
         <v>342</v>
       </c>
@@ -19853,30 +20311,30 @@
       <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="190" t="s">
+      <c r="B2" s="189" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="194" t="s">
+      <c r="C2" s="193" t="s">
         <v>174</v>
       </c>
-      <c r="D2" s="194" t="s">
+      <c r="D2" s="193" t="s">
         <v>175</v>
       </c>
-      <c r="E2" s="192" t="s">
+      <c r="E2" s="191" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="188" t="s">
+      <c r="F2" s="187" t="s">
         <v>369</v>
       </c>
-      <c r="G2" s="188"/>
-      <c r="H2" s="188"/>
-      <c r="I2" s="189"/>
+      <c r="G2" s="187"/>
+      <c r="H2" s="187"/>
+      <c r="I2" s="188"/>
     </row>
     <row r="3" spans="1:9" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="191"/>
-      <c r="C3" s="195"/>
-      <c r="D3" s="195"/>
-      <c r="E3" s="193"/>
+      <c r="B3" s="190"/>
+      <c r="C3" s="194"/>
+      <c r="D3" s="194"/>
+      <c r="E3" s="192"/>
       <c r="F3" s="87" t="s">
         <v>370</v>
       </c>

</xml_diff>